<commit_message>
Record the second CreatorHub Live answer and draft its copy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -604,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U51"/>
+  <dimension ref="A1:U52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1050,7 +1050,7 @@
       <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr"/>
     </row>
-    <row r="9" ht="150" customHeight="1">
+    <row r="9" ht="300" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>CreatorHub Live</t>
@@ -1061,9 +1061,9 @@
           <t>creatorhub-live</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>August 2025</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -1078,11 +1078,19 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>There was no event where entrepreneurs and creators could come together to learn business and media production. The only competition in the space belonged to MrBeast, the largest media entity on the planet, so building an event people would trust enough to pay for meant pushing through real resistance from sponsors and attendees who were not ready to try something new.
-The stakes were hundreds of thousands of dollars, our reputation, and the trust of the speakers and creators brought in by Xtend Creators, our co-owner. If it flopped, Patrick Israel and Xtend would lose relational capital with every sponsor and creator they had brought to the table.</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr"/>
+          <t>There was no event where entrepreneurs and creators could come together to learn business and media production. The largest event at this capacity was run and owned by MrBeast, the biggest media entity on the planet, so building something people would trust enough to pay for meant pushing through heavy resistance.
+A brand new event with no history is a hard sell in the creator economy. Sponsors did not want to be first in, the platforms that mattered most, YouTube, TikTok and Snapchat, had to be won over, and getting bodies in the room was just as hard.
+The stakes were a multi six figure investment, the reputation of everyone involved, and the trust of the speakers and creators brought in by co-owner Xtend Creators. If it flopped, Patrick Israel and Xtend would lose relational capital with every sponsor and creator they had brought to the table.</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>1. Rebuilt the sponsorship strategy around in person meetings, and used after party brand activations to give partners a way in.
+2. Replaced the standard gold, platinum and silver packages with a la carte options, so each sponsor could find a natural way into the event.
+3. Built the hub model: other events contract one of the stages and run their own mini event inside CreatorHub, which is where the name comes from. It put attendees from several communities under one roof with the same purpose, and it is what delivered the attendance.
+4. Brought a Lamborghini into the Marriott to be painted live during the networking mixer. Getting it inside meant physically removing part of the hotel's frame, and a 50 foot enclosure built with the Marriott kept every drop of paint off the venue and protected an almost six figure deposit. It had never been attempted in a Marriott before.</t>
+        </is>
+      </c>
       <c r="H9" s="5" t="inlineStr"/>
       <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr"/>
@@ -1106,29 +1114,29 @@
       <c r="T9" s="5" t="inlineStr"/>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>Naming MrBeast on a public page: third party brand, see the open decision in the protocol. "Hundreds of thousands of dollars" hints at the budget (house rule 2). Leads to confirm: 36 round tables sold; 100+ testimonials from the on site studio; a 2026 edition in production. Month of the 2025 edition?</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
+          <t>Voice: no first person on this page (Iconic's call), so its section headings (What We Did) need a third person variant when built. Is the Marriott the main venue, or where the mixer was? The index says FTL Downtown Event Center. "Integrated organically into the post": into the post event content, or the event itself? Leads still to confirm: 36 round tables sold; 100+ testimonials from the on site studio; a 2026 edition in production. "Almost six figure deposit" hints at spend, flagged for rule 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Creator Hub Madrid</t>
+          <t>Creator Fest</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>creator-hub-madrid</t>
+          <t>creator-fest</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>August 2024</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Universal Music Group</t>
+          <t>None. Iconic's own event</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1144,28 +1152,28 @@
       <c r="K10" s="5" t="inlineStr"/>
       <c r="L10" s="5" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr"/>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>Madrid, Spain</t>
-        </is>
-      </c>
+      <c r="N10" s="5" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr"/>
       <c r="P10" s="5" t="inlineStr"/>
       <c r="Q10" s="5" t="inlineStr"/>
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr"/>
       <c r="T10" s="5" t="inlineStr"/>
-      <c r="U10" s="5" t="inlineStr"/>
+      <c r="U10" s="7" t="inlineStr">
+        <is>
+          <t>The first edition of what became CreatorHub Live. Not on the website grid yet; add it with the next approved site change.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>PMUW 2025</t>
+          <t>Creator Hub Madrid</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>pmuw-2025</t>
+          <t>creator-hub-madrid</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1175,7 +1183,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Danny Tran</t>
+          <t>Universal Music Group</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -1191,7 +1199,11 @@
       <c r="K11" s="5" t="inlineStr"/>
       <c r="L11" s="5" t="inlineStr"/>
       <c r="M11" s="5" t="inlineStr"/>
-      <c r="N11" s="5" t="inlineStr"/>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>Madrid, Spain</t>
+        </is>
+      </c>
       <c r="O11" s="5" t="inlineStr"/>
       <c r="P11" s="5" t="inlineStr"/>
       <c r="Q11" s="5" t="inlineStr"/>
@@ -1203,12 +1215,12 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Fast Start Forum 2025</t>
+          <t>PMUW 2025</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>fast-start-forum-2025</t>
+          <t>pmuw-2025</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1218,7 +1230,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Tom Wall</t>
+          <t>Danny Tran</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -1246,12 +1258,12 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Hell Yes Live</t>
+          <t>Fast Start Forum 2025</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>hell-yes-live</t>
+          <t>fast-start-forum-2025</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -1261,7 +1273,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Becca Pike</t>
+          <t>Tom Wall</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1289,12 +1301,12 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Closers.io Retreat</t>
+          <t>Hell Yes Live</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>closers-io-retreat</t>
+          <t>hell-yes-live</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -1304,7 +1316,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Cole Gordon</t>
+          <t>Becca Pike</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1332,12 +1344,12 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Maxxed Out Summit</t>
+          <t>Closers.io Retreat</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>maxxed-out-summit</t>
+          <t>closers-io-retreat</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -1347,7 +1359,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Max Willett</t>
+          <t>Cole Gordon</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -1375,12 +1387,12 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Her Last Call</t>
+          <t>Maxxed Out Summit</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>her-last-call</t>
+          <t>maxxed-out-summit</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -1390,7 +1402,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Alexis Mai</t>
+          <t>Max Willett</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1418,12 +1430,12 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>PimCon 2025</t>
+          <t>Her Last Call</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>pimcon-2025</t>
+          <t>her-last-call</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1433,7 +1445,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Rankings.io</t>
+          <t>Alexis Mai</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1461,12 +1473,12 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>DealCon 2025</t>
+          <t>PimCon 2025</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>dealcon-2025</t>
+          <t>pimcon-2025</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -1476,7 +1488,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Tom Shipley</t>
+          <t>Rankings.io</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1504,22 +1516,22 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Freedom Queen Live 2024</t>
+          <t>DealCon 2025</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>freedom-queen-live-2024</t>
+          <t>dealcon-2025</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>November 2024</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Bridget James Ling</t>
+          <t>Tom Shipley</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1547,27 +1559,27 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Bad After Dark</t>
+          <t>Freedom Queen Live 2024</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>bad-after-dark</t>
+          <t>freedom-queen-live-2024</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>January 2024</t>
+          <t>November 2024</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Eddie Maalouf</t>
+          <t>Bridget James Ling</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr"/>
@@ -1590,27 +1602,27 @@
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>PMUW 2024</t>
+          <t>Bad After Dark</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>pmuw-2024</t>
+          <t>bad-after-dark</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>January 2024</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Danny Tran</t>
+          <t>Eddie Maalouf</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr"/>
@@ -1633,12 +1645,12 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Fast Start Forum 2024</t>
+          <t>PMUW 2024</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>fast-start-forum-2024</t>
+          <t>pmuw-2024</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -1648,7 +1660,7 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Tom Wall</t>
+          <t>Danny Tran</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1676,12 +1688,12 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>PimCon 2024</t>
+          <t>Fast Start Forum 2024</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>pimcon-2024</t>
+          <t>fast-start-forum-2024</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -1691,7 +1703,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Rankings.io</t>
+          <t>Tom Wall</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1719,27 +1731,27 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Casino Royale</t>
+          <t>PimCon 2024</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>casino-royale</t>
+          <t>pimcon-2024</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>October 2023</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Ben Newman</t>
+          <t>Rankings.io</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr"/>
@@ -1750,11 +1762,7 @@
       <c r="K24" s="5" t="inlineStr"/>
       <c r="L24" s="5" t="inlineStr"/>
       <c r="M24" s="5" t="inlineStr"/>
-      <c r="N24" s="5" t="inlineStr">
-        <is>
-          <t>Las Vegas, NV</t>
-        </is>
-      </c>
+      <c r="N24" s="5" t="inlineStr"/>
       <c r="O24" s="5" t="inlineStr"/>
       <c r="P24" s="5" t="inlineStr"/>
       <c r="Q24" s="5" t="inlineStr"/>
@@ -1766,27 +1774,27 @@
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>The Black Course</t>
+          <t>Casino Royale</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>the-black-course</t>
+          <t>casino-royale</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>June 2023</t>
+          <t>October 2023</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Chase Hughes</t>
+          <t>Ben Newman</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr"/>
@@ -1797,7 +1805,11 @@
       <c r="K25" s="5" t="inlineStr"/>
       <c r="L25" s="5" t="inlineStr"/>
       <c r="M25" s="5" t="inlineStr"/>
-      <c r="N25" s="5" t="inlineStr"/>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>Las Vegas, NV</t>
+        </is>
+      </c>
       <c r="O25" s="5" t="inlineStr"/>
       <c r="P25" s="5" t="inlineStr"/>
       <c r="Q25" s="5" t="inlineStr"/>
@@ -1809,12 +1821,12 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Viral Ecom Adz</t>
+          <t>The Black Course</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>viral-ecom-adz</t>
+          <t>the-black-course</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -1824,12 +1836,12 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Noah Brewer</t>
+          <t>Chase Hughes</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr"/>
@@ -1852,27 +1864,27 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>PMUW 2023</t>
+          <t>Viral Ecom Adz</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>pmuw-2023</t>
+          <t>viral-ecom-adz</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>April 2023</t>
+          <t>June 2023</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Danny Tran</t>
+          <t>Noah Brewer</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr"/>
@@ -1895,27 +1907,27 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Chase Hughes, London</t>
+          <t>PMUW 2023</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>chase-hughes-london</t>
+          <t>pmuw-2023</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>February 2023</t>
+          <t>April 2023</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Chase Hughes</t>
+          <t>Danny Tran</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr"/>
@@ -1926,11 +1938,7 @@
       <c r="K28" s="5" t="inlineStr"/>
       <c r="L28" s="5" t="inlineStr"/>
       <c r="M28" s="5" t="inlineStr"/>
-      <c r="N28" s="5" t="inlineStr">
-        <is>
-          <t>London, UK</t>
-        </is>
-      </c>
+      <c r="N28" s="5" t="inlineStr"/>
       <c r="O28" s="5" t="inlineStr"/>
       <c r="P28" s="5" t="inlineStr"/>
       <c r="Q28" s="5" t="inlineStr"/>
@@ -1942,17 +1950,17 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Behavior Pilot</t>
+          <t>Chase Hughes, London</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>behavior-pilot</t>
+          <t>chase-hughes-london</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>February 2023</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -1962,7 +1970,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr"/>
@@ -1973,7 +1981,11 @@
       <c r="K29" s="5" t="inlineStr"/>
       <c r="L29" s="5" t="inlineStr"/>
       <c r="M29" s="5" t="inlineStr"/>
-      <c r="N29" s="5" t="inlineStr"/>
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t>London, UK</t>
+        </is>
+      </c>
       <c r="O29" s="5" t="inlineStr"/>
       <c r="P29" s="5" t="inlineStr"/>
       <c r="Q29" s="5" t="inlineStr"/>
@@ -1985,12 +1997,12 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Sales Momentum Live</t>
+          <t>Behavior Pilot</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>sales-momentum-live</t>
+          <t>behavior-pilot</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -2000,7 +2012,7 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Aaron Platt</t>
+          <t>Chase Hughes</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -2028,12 +2040,12 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>E.P.I.C</t>
+          <t>Sales Momentum Live</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>e-p-i-c</t>
+          <t>sales-momentum-live</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -2043,7 +2055,7 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Kaaba Luum</t>
+          <t>Aaron Platt</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -2071,12 +2083,12 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Founder OS</t>
+          <t>E.P.I.C</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>founder-os</t>
+          <t>e-p-i-c</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -2086,7 +2098,7 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Matt Gray</t>
+          <t>Kaaba Luum</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -2114,12 +2126,12 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Scaling With Systems LIVE 2023</t>
+          <t>Founder OS</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>scaling-with-systems-live-2023</t>
+          <t>founder-os</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -2129,7 +2141,7 @@
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Ravi Abuvala</t>
+          <t>Matt Gray</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -2157,22 +2169,22 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>The CEO Lawyer Summit 2022</t>
+          <t>Scaling With Systems LIVE 2023</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>the-ceo-lawyer-summit-2022</t>
+          <t>scaling-with-systems-live-2023</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>December 2022</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Ali Awad</t>
+          <t>Ravi Abuvala</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -2200,22 +2212,22 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>The Behavior Panel Live</t>
+          <t>The CEO Lawyer Summit 2022</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>the-behavior-panel-live</t>
+          <t>the-ceo-lawyer-summit-2022</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>July 2022</t>
+          <t>December 2022</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>The Behavior Panel</t>
+          <t>Ali Awad</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -2231,11 +2243,7 @@
       <c r="K35" s="5" t="inlineStr"/>
       <c r="L35" s="5" t="inlineStr"/>
       <c r="M35" s="5" t="inlineStr"/>
-      <c r="N35" s="5" t="inlineStr">
-        <is>
-          <t>Las Vegas, NV</t>
-        </is>
-      </c>
+      <c r="N35" s="5" t="inlineStr"/>
       <c r="O35" s="5" t="inlineStr"/>
       <c r="P35" s="5" t="inlineStr"/>
       <c r="Q35" s="5" t="inlineStr"/>
@@ -2247,22 +2255,22 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>The Guardians Annual</t>
+          <t>The Behavior Panel Live</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>the-guardians-annual</t>
+          <t>the-behavior-panel-live</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>April 2022</t>
+          <t>July 2022</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Thaddeus Gala</t>
+          <t>The Behavior Panel</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -2278,7 +2286,11 @@
       <c r="K36" s="5" t="inlineStr"/>
       <c r="L36" s="5" t="inlineStr"/>
       <c r="M36" s="5" t="inlineStr"/>
-      <c r="N36" s="5" t="inlineStr"/>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>Las Vegas, NV</t>
+        </is>
+      </c>
       <c r="O36" s="5" t="inlineStr"/>
       <c r="P36" s="5" t="inlineStr"/>
       <c r="Q36" s="5" t="inlineStr"/>
@@ -2290,12 +2302,12 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Rise X</t>
+          <t>The Guardians Annual</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>rise-x</t>
+          <t>the-guardians-annual</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -2305,7 +2317,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Joel Kaplan and Sergio Tavarez</t>
+          <t>Thaddeus Gala</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -2321,11 +2333,7 @@
       <c r="K37" s="5" t="inlineStr"/>
       <c r="L37" s="5" t="inlineStr"/>
       <c r="M37" s="5" t="inlineStr"/>
-      <c r="N37" s="5" t="inlineStr">
-        <is>
-          <t>Costa Rica</t>
-        </is>
-      </c>
+      <c r="N37" s="5" t="inlineStr"/>
       <c r="O37" s="5" t="inlineStr"/>
       <c r="P37" s="5" t="inlineStr"/>
       <c r="Q37" s="5" t="inlineStr"/>
@@ -2337,22 +2345,22 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>Bulletproof Financial Accelerator</t>
+          <t>Rise X</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>bulletproof-financial-accelerator</t>
+          <t>rise-x</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>March 2022</t>
+          <t>April 2022</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>John Whiting</t>
+          <t>Joel Kaplan and Sergio Tavarez</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -2370,7 +2378,7 @@
       <c r="M38" s="5" t="inlineStr"/>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>Orlando, FL</t>
+          <t>Costa Rica</t>
         </is>
       </c>
       <c r="O38" s="5" t="inlineStr"/>
@@ -2384,22 +2392,22 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Ace Interstellar</t>
+          <t>Bulletproof Financial Accelerator</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>ace-interstellar</t>
+          <t>bulletproof-financial-accelerator</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>January 2022</t>
+          <t>March 2022</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Michael Sheridan</t>
+          <t>John Whiting</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -2417,7 +2425,7 @@
       <c r="M39" s="5" t="inlineStr"/>
       <c r="N39" s="5" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Orlando, FL</t>
         </is>
       </c>
       <c r="O39" s="5" t="inlineStr"/>
@@ -2431,22 +2439,22 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Powerhouse</t>
+          <t>Ace Interstellar</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>powerhouse</t>
+          <t>ace-interstellar</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>January 2022</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Los Silva</t>
+          <t>Michael Sheridan</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -2462,7 +2470,11 @@
       <c r="K40" s="5" t="inlineStr"/>
       <c r="L40" s="5" t="inlineStr"/>
       <c r="M40" s="5" t="inlineStr"/>
-      <c r="N40" s="5" t="inlineStr"/>
+      <c r="N40" s="5" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
       <c r="O40" s="5" t="inlineStr"/>
       <c r="P40" s="5" t="inlineStr"/>
       <c r="Q40" s="5" t="inlineStr"/>
@@ -2474,12 +2486,12 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>EGC 2022</t>
+          <t>Powerhouse</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>egc-2022</t>
+          <t>powerhouse</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -2489,7 +2501,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Austin Zelan</t>
+          <t>Los Silva</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -2517,12 +2529,12 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Scaling With Systems LIVE 2022</t>
+          <t>EGC 2022</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>scaling-with-systems-live-2022</t>
+          <t>egc-2022</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -2532,7 +2544,7 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Ravi Abuvala</t>
+          <t>Austin Zelan</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -2548,11 +2560,7 @@
       <c r="K42" s="5" t="inlineStr"/>
       <c r="L42" s="5" t="inlineStr"/>
       <c r="M42" s="5" t="inlineStr"/>
-      <c r="N42" s="5" t="inlineStr">
-        <is>
-          <t>Miami, FL</t>
-        </is>
-      </c>
+      <c r="N42" s="5" t="inlineStr"/>
       <c r="O42" s="5" t="inlineStr"/>
       <c r="P42" s="5" t="inlineStr"/>
       <c r="Q42" s="5" t="inlineStr"/>
@@ -2564,27 +2572,27 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>The CEO Lawyer Summit 2021</t>
+          <t>Scaling With Systems LIVE 2022</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>ceo-lawyer-summit</t>
+          <t>scaling-with-systems-live-2022</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>December 2021</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Ali Awad</t>
+          <t>Ravi Abuvala</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr"/>
@@ -2595,7 +2603,11 @@
       <c r="K43" s="5" t="inlineStr"/>
       <c r="L43" s="5" t="inlineStr"/>
       <c r="M43" s="5" t="inlineStr"/>
-      <c r="N43" s="5" t="inlineStr"/>
+      <c r="N43" s="5" t="inlineStr">
+        <is>
+          <t>Miami, FL</t>
+        </is>
+      </c>
       <c r="O43" s="5" t="inlineStr"/>
       <c r="P43" s="5" t="inlineStr"/>
       <c r="Q43" s="5" t="inlineStr"/>
@@ -2607,27 +2619,27 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Epic Growth Conference 2021</t>
+          <t>The CEO Lawyer Summit 2021</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>epic-growth-conference-2021</t>
+          <t>ceo-lawyer-summit</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>November 2021</t>
+          <t>December 2021</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Tyler Cerny and Austin Zelan</t>
+          <t>Ali Awad</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr"/>
@@ -2638,11 +2650,7 @@
       <c r="K44" s="5" t="inlineStr"/>
       <c r="L44" s="5" t="inlineStr"/>
       <c r="M44" s="5" t="inlineStr"/>
-      <c r="N44" s="5" t="inlineStr">
-        <is>
-          <t>Las Vegas, NV</t>
-        </is>
-      </c>
+      <c r="N44" s="5" t="inlineStr"/>
       <c r="O44" s="5" t="inlineStr"/>
       <c r="P44" s="5" t="inlineStr"/>
       <c r="Q44" s="5" t="inlineStr"/>
@@ -2654,22 +2662,22 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Behavioral Selling</t>
+          <t>Epic Growth Conference 2021</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>behavioral-selling</t>
+          <t>epic-growth-conference-2021</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>October 2021</t>
+          <t>November 2021</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Chase Hughes</t>
+          <t>Tyler Cerny and Austin Zelan</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -2687,7 +2695,7 @@
       <c r="M45" s="5" t="inlineStr"/>
       <c r="N45" s="5" t="inlineStr">
         <is>
-          <t>Miami, FL</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="O45" s="5" t="inlineStr"/>
@@ -2701,22 +2709,22 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Takeover Live 3</t>
+          <t>Behavioral Selling</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>takeover-live-3</t>
+          <t>behavioral-selling</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>August 2021</t>
+          <t>October 2021</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Danny Tran</t>
+          <t>Chase Hughes</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -2734,7 +2742,7 @@
       <c r="M46" s="5" t="inlineStr"/>
       <c r="N46" s="5" t="inlineStr">
         <is>
-          <t>Sundance, UT</t>
+          <t>Miami, FL</t>
         </is>
       </c>
       <c r="O46" s="5" t="inlineStr"/>
@@ -2748,12 +2756,12 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Group Convert Live</t>
+          <t>Takeover Live 3</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>group-convert-live</t>
+          <t>takeover-live-3</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
@@ -2763,7 +2771,7 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Kim Dang</t>
+          <t>Danny Tran</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -2781,7 +2789,7 @@
       <c r="M47" s="5" t="inlineStr"/>
       <c r="N47" s="5" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Sundance, UT</t>
         </is>
       </c>
       <c r="O47" s="5" t="inlineStr"/>
@@ -2795,22 +2803,22 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Takeover Live 2</t>
+          <t>Group Convert Live</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>takeover-live-2</t>
+          <t>group-convert-live</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>May 2021</t>
+          <t>August 2021</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Danny Tran</t>
+          <t>Kim Dang</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -2842,27 +2850,27 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Scaling With Systems LIVE 2021</t>
+          <t>Takeover Live 2</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>scaling-with-systems-live</t>
+          <t>takeover-live-2</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>April 2021</t>
+          <t>May 2021</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Ravi Abuvala</t>
+          <t>Danny Tran</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Built</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr"/>
@@ -2875,7 +2883,7 @@
       <c r="M49" s="5" t="inlineStr"/>
       <c r="N49" s="5" t="inlineStr">
         <is>
-          <t>1111 Miami</t>
+          <t>Las Vegas, NV</t>
         </is>
       </c>
       <c r="O49" s="5" t="inlineStr"/>
@@ -2884,36 +2892,32 @@
       <c r="R49" s="5" t="inlineStr"/>
       <c r="S49" s="5" t="inlineStr"/>
       <c r="T49" s="5" t="inlineStr"/>
-      <c r="U49" s="5" t="inlineStr">
-        <is>
-          <t>Built from the old site copy. Revenue published by Iconic's one time exception. Interview Q4 and Q5 still open.</t>
-        </is>
-      </c>
+      <c r="U49" s="5" t="inlineStr"/>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>7-Figure Agency</t>
+          <t>Scaling With Systems LIVE 2021</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>7-figure-agency</t>
+          <t>scaling-with-systems-live</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>January 2021</t>
+          <t>April 2021</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Joel Kaplan</t>
+          <t>Ravi Abuvala</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr"/>
@@ -2926,7 +2930,7 @@
       <c r="M50" s="5" t="inlineStr"/>
       <c r="N50" s="5" t="inlineStr">
         <is>
-          <t>Playa del Carmen, Mexico</t>
+          <t>1111 Miami</t>
         </is>
       </c>
       <c r="O50" s="5" t="inlineStr"/>
@@ -2935,17 +2939,21 @@
       <c r="R50" s="5" t="inlineStr"/>
       <c r="S50" s="5" t="inlineStr"/>
       <c r="T50" s="5" t="inlineStr"/>
-      <c r="U50" s="5" t="inlineStr"/>
+      <c r="U50" s="5" t="inlineStr">
+        <is>
+          <t>Built from the old site copy. Revenue published by Iconic's one time exception. Interview Q4 and Q5 still open.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Takeover Live 1</t>
+          <t>7-Figure Agency</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>takeover-live-1</t>
+          <t>7-figure-agency</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -2955,7 +2963,7 @@
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Danny Tran</t>
+          <t>Joel Kaplan</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -2973,7 +2981,7 @@
       <c r="M51" s="5" t="inlineStr"/>
       <c r="N51" s="5" t="inlineStr">
         <is>
-          <t>Las Vegas, NV</t>
+          <t>Playa del Carmen, Mexico</t>
         </is>
       </c>
       <c r="O51" s="5" t="inlineStr"/>
@@ -2983,6 +2991,53 @@
       <c r="S51" s="5" t="inlineStr"/>
       <c r="T51" s="5" t="inlineStr"/>
       <c r="U51" s="5" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Takeover Live 1</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>takeover-live-1</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>January 2021</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Danny Tran</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr"/>
+      <c r="G52" s="5" t="inlineStr"/>
+      <c r="H52" s="5" t="inlineStr"/>
+      <c r="I52" s="5" t="inlineStr"/>
+      <c r="J52" s="5" t="inlineStr"/>
+      <c r="K52" s="5" t="inlineStr"/>
+      <c r="L52" s="5" t="inlineStr"/>
+      <c r="M52" s="5" t="inlineStr"/>
+      <c r="N52" s="5" t="inlineStr">
+        <is>
+          <t>Las Vegas, NV</t>
+        </is>
+      </c>
+      <c r="O52" s="5" t="inlineStr"/>
+      <c r="P52" s="5" t="inlineStr"/>
+      <c r="Q52" s="5" t="inlineStr"/>
+      <c r="R52" s="5" t="inlineStr"/>
+      <c r="S52" s="5" t="inlineStr"/>
+      <c r="T52" s="5" t="inlineStr"/>
+      <c r="U52" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Record the CreatorHub Live what nearly broke answer and draft its copy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -604,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U52"/>
+  <dimension ref="A1:W52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -628,6 +628,8 @@
     <col width="24" customWidth="1" min="19" max="19"/>
     <col width="28" customWidth="1" min="20" max="20"/>
     <col width="50" customWidth="1" min="21" max="21"/>
+    <col width="60" customWidth="1" min="22" max="22"/>
+    <col width="60" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -734,6 +736,16 @@
       <c r="U1" s="4" t="inlineStr">
         <is>
           <t>Open questions and flags</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
+        <is>
+          <t>What Nearly Broke</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>Right for / wrong for</t>
         </is>
       </c>
     </row>
@@ -783,6 +795,8 @@
       <c r="S2" s="5" t="inlineStr"/>
       <c r="T2" s="5" t="inlineStr"/>
       <c r="U2" s="5" t="inlineStr"/>
+      <c r="V2" s="5" t="n"/>
+      <c r="W2" s="5" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -830,6 +844,8 @@
       <c r="S3" s="5" t="inlineStr"/>
       <c r="T3" s="5" t="inlineStr"/>
       <c r="U3" s="5" t="inlineStr"/>
+      <c r="V3" s="5" t="n"/>
+      <c r="W3" s="5" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -873,6 +889,8 @@
       <c r="S4" s="5" t="inlineStr"/>
       <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr"/>
+      <c r="V4" s="5" t="n"/>
+      <c r="W4" s="5" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -916,6 +934,8 @@
       <c r="S5" s="5" t="inlineStr"/>
       <c r="T5" s="5" t="inlineStr"/>
       <c r="U5" s="5" t="inlineStr"/>
+      <c r="V5" s="5" t="n"/>
+      <c r="W5" s="5" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -959,6 +979,8 @@
       <c r="S6" s="5" t="inlineStr"/>
       <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr"/>
+      <c r="V6" s="5" t="n"/>
+      <c r="W6" s="5" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -1006,6 +1028,8 @@
       <c r="S7" s="5" t="inlineStr"/>
       <c r="T7" s="5" t="inlineStr"/>
       <c r="U7" s="5" t="inlineStr"/>
+      <c r="V7" s="5" t="n"/>
+      <c r="W7" s="5" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -1049,8 +1073,10 @@
       <c r="S8" s="5" t="inlineStr"/>
       <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9" ht="300" customHeight="1">
+      <c r="V8" s="5" t="n"/>
+      <c r="W8" s="5" t="n"/>
+    </row>
+    <row r="9" ht="330" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>CreatorHub Live</t>
@@ -1088,18 +1114,24 @@
           <t>1. Rebuilt the sponsorship strategy around in person meetings, and used after party brand activations to give partners a way in.
 2. Replaced the standard gold, platinum and silver packages with a la carte options, so each sponsor could find a natural way into the event.
 3. Built the hub model: other events contract one of the stages and run their own mini event inside CreatorHub, which is where the name comes from. It put attendees from several communities under one roof with the same purpose, and it is what delivered the attendance.
-4. Brought a Lamborghini into the Marriott to be painted live during the networking mixer. Getting it inside meant physically removing part of the hotel's frame, and a 50 foot enclosure built with the Marriott kept every drop of paint off the venue and protected an almost six figure deposit. It had never been attempted in a Marriott before.</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr"/>
+4. Ran three stages at once as three separate events that happened to share a building, each with its own dedicated stage manager.
+5. Brought a Lamborghini into the Marriott Bonnet Creek to be painted live during the networking mixer, inside a 50 foot glass enclosure built with the Marriott so not a drop of paint touched the venue.</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>The hub model delivered the attendance the event needed. Three stages ran at once on a clean run of show.
+The round tables, fireside chats with a speaker at each table, were planned for 45 minutes. Attendees loved them so much they stayed for about three and a half hours.</t>
+        </is>
+      </c>
       <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr"/>
       <c r="K9" s="5" t="inlineStr"/>
       <c r="L9" s="5" t="inlineStr"/>
       <c r="M9" s="5" t="inlineStr"/>
-      <c r="N9" s="5" t="inlineStr">
-        <is>
-          <t>Fort Lauderdale, FL</t>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>Marriott Bonnet Creek, Orlando, FL</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr">
@@ -1114,9 +1146,16 @@
       <c r="T9" s="5" t="inlineStr"/>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>Voice: no first person on this page (Iconic's call), so its section headings (What We Did) need a third person variant when built. Is the Marriott the main venue, or where the mixer was? The index says FTL Downtown Event Center. "Integrated organically into the post": into the post event content, or the event itself? Leads still to confirm: 36 round tables sold; 100+ testimonials from the on site studio; a 2026 edition in production. "Almost six figure deposit" hints at spend, flagged for rule 2.</t>
-        </is>
-      </c>
+          <t>Page needs two new sections for this: What Nearly Broke, and Right for / wrong for (Iconic to decide; protocol section 3). Heading on this page: How It Was Built, no first person. Speaker count: exact number needed (answer was about 40 to 60). Venue fix on the site: Marriott Bonnet Creek, Orlando, not FTL Downtown Event Center. Leads still to confirm: 36 round tables sold; 100+ testimonials from the on site studio; a 2026 edition in production.</t>
+        </is>
+      </c>
+      <c r="V9" s="7" t="inlineStr">
+        <is>
+          <t>Ticket sales opened before the hubs were ready, so the first couple of months were a rocky road, with real uncertainty about where ticket sales stood.
+The Lamborghini nearly did not make it in. It was the performance version, wider than planned, and it cleared the doorway by a couple of millimeters on each side after a door came off the Marriott. Without it the mixer would have had nothing, Lamborghini would have been a disappointed sponsor, and a badly built enclosure could have meant hundreds of thousands of dollars in insurance claims if paint escaped into the venue.</t>
+        </is>
+      </c>
+      <c r="W9" s="5" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -1152,7 +1191,11 @@
       <c r="K10" s="5" t="inlineStr"/>
       <c r="L10" s="5" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr"/>
-      <c r="N10" s="5" t="inlineStr"/>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>Marriott Bonnet Creek, Orlando, FL</t>
+        </is>
+      </c>
       <c r="O10" s="5" t="inlineStr"/>
       <c r="P10" s="5" t="inlineStr"/>
       <c r="Q10" s="5" t="inlineStr"/>
@@ -1164,6 +1207,8 @@
           <t>The first edition of what became CreatorHub Live. Not on the website grid yet; add it with the next approved site change.</t>
         </is>
       </c>
+      <c r="V10" s="5" t="n"/>
+      <c r="W10" s="5" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1211,6 +1256,8 @@
       <c r="S11" s="5" t="inlineStr"/>
       <c r="T11" s="5" t="inlineStr"/>
       <c r="U11" s="5" t="inlineStr"/>
+      <c r="V11" s="5" t="n"/>
+      <c r="W11" s="5" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -1254,6 +1301,8 @@
       <c r="S12" s="5" t="inlineStr"/>
       <c r="T12" s="5" t="inlineStr"/>
       <c r="U12" s="5" t="inlineStr"/>
+      <c r="V12" s="5" t="n"/>
+      <c r="W12" s="5" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1297,6 +1346,8 @@
       <c r="S13" s="5" t="inlineStr"/>
       <c r="T13" s="5" t="inlineStr"/>
       <c r="U13" s="5" t="inlineStr"/>
+      <c r="V13" s="5" t="n"/>
+      <c r="W13" s="5" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -1340,6 +1391,8 @@
       <c r="S14" s="5" t="inlineStr"/>
       <c r="T14" s="5" t="inlineStr"/>
       <c r="U14" s="5" t="inlineStr"/>
+      <c r="V14" s="5" t="n"/>
+      <c r="W14" s="5" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1383,6 +1436,8 @@
       <c r="S15" s="5" t="inlineStr"/>
       <c r="T15" s="5" t="inlineStr"/>
       <c r="U15" s="5" t="inlineStr"/>
+      <c r="V15" s="5" t="n"/>
+      <c r="W15" s="5" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -1426,6 +1481,8 @@
       <c r="S16" s="5" t="inlineStr"/>
       <c r="T16" s="5" t="inlineStr"/>
       <c r="U16" s="5" t="inlineStr"/>
+      <c r="V16" s="5" t="n"/>
+      <c r="W16" s="5" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -1469,6 +1526,8 @@
       <c r="S17" s="5" t="inlineStr"/>
       <c r="T17" s="5" t="inlineStr"/>
       <c r="U17" s="5" t="inlineStr"/>
+      <c r="V17" s="5" t="n"/>
+      <c r="W17" s="5" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1512,6 +1571,8 @@
       <c r="S18" s="5" t="inlineStr"/>
       <c r="T18" s="5" t="inlineStr"/>
       <c r="U18" s="5" t="inlineStr"/>
+      <c r="V18" s="5" t="n"/>
+      <c r="W18" s="5" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1555,6 +1616,8 @@
       <c r="S19" s="5" t="inlineStr"/>
       <c r="T19" s="5" t="inlineStr"/>
       <c r="U19" s="5" t="inlineStr"/>
+      <c r="V19" s="5" t="n"/>
+      <c r="W19" s="5" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -1598,6 +1661,8 @@
       <c r="S20" s="5" t="inlineStr"/>
       <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr"/>
+      <c r="V20" s="5" t="n"/>
+      <c r="W20" s="5" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -1641,6 +1706,8 @@
       <c r="S21" s="5" t="inlineStr"/>
       <c r="T21" s="5" t="inlineStr"/>
       <c r="U21" s="5" t="inlineStr"/>
+      <c r="V21" s="5" t="n"/>
+      <c r="W21" s="5" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -1684,6 +1751,8 @@
       <c r="S22" s="5" t="inlineStr"/>
       <c r="T22" s="5" t="inlineStr"/>
       <c r="U22" s="5" t="inlineStr"/>
+      <c r="V22" s="5" t="n"/>
+      <c r="W22" s="5" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -1727,6 +1796,8 @@
       <c r="S23" s="5" t="inlineStr"/>
       <c r="T23" s="5" t="inlineStr"/>
       <c r="U23" s="5" t="inlineStr"/>
+      <c r="V23" s="5" t="n"/>
+      <c r="W23" s="5" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
@@ -1770,6 +1841,8 @@
       <c r="S24" s="5" t="inlineStr"/>
       <c r="T24" s="5" t="inlineStr"/>
       <c r="U24" s="5" t="inlineStr"/>
+      <c r="V24" s="5" t="n"/>
+      <c r="W24" s="5" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -1817,6 +1890,8 @@
       <c r="S25" s="5" t="inlineStr"/>
       <c r="T25" s="5" t="inlineStr"/>
       <c r="U25" s="5" t="inlineStr"/>
+      <c r="V25" s="5" t="n"/>
+      <c r="W25" s="5" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
@@ -1860,6 +1935,8 @@
       <c r="S26" s="5" t="inlineStr"/>
       <c r="T26" s="5" t="inlineStr"/>
       <c r="U26" s="5" t="inlineStr"/>
+      <c r="V26" s="5" t="n"/>
+      <c r="W26" s="5" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -1903,6 +1980,8 @@
       <c r="S27" s="5" t="inlineStr"/>
       <c r="T27" s="5" t="inlineStr"/>
       <c r="U27" s="5" t="inlineStr"/>
+      <c r="V27" s="5" t="n"/>
+      <c r="W27" s="5" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
@@ -1946,6 +2025,8 @@
       <c r="S28" s="5" t="inlineStr"/>
       <c r="T28" s="5" t="inlineStr"/>
       <c r="U28" s="5" t="inlineStr"/>
+      <c r="V28" s="5" t="n"/>
+      <c r="W28" s="5" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -1993,6 +2074,8 @@
       <c r="S29" s="5" t="inlineStr"/>
       <c r="T29" s="5" t="inlineStr"/>
       <c r="U29" s="5" t="inlineStr"/>
+      <c r="V29" s="5" t="n"/>
+      <c r="W29" s="5" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
@@ -2036,6 +2119,8 @@
       <c r="S30" s="5" t="inlineStr"/>
       <c r="T30" s="5" t="inlineStr"/>
       <c r="U30" s="5" t="inlineStr"/>
+      <c r="V30" s="5" t="n"/>
+      <c r="W30" s="5" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -2079,6 +2164,8 @@
       <c r="S31" s="5" t="inlineStr"/>
       <c r="T31" s="5" t="inlineStr"/>
       <c r="U31" s="5" t="inlineStr"/>
+      <c r="V31" s="5" t="n"/>
+      <c r="W31" s="5" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
@@ -2122,6 +2209,8 @@
       <c r="S32" s="5" t="inlineStr"/>
       <c r="T32" s="5" t="inlineStr"/>
       <c r="U32" s="5" t="inlineStr"/>
+      <c r="V32" s="5" t="n"/>
+      <c r="W32" s="5" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -2165,6 +2254,8 @@
       <c r="S33" s="5" t="inlineStr"/>
       <c r="T33" s="5" t="inlineStr"/>
       <c r="U33" s="5" t="inlineStr"/>
+      <c r="V33" s="5" t="n"/>
+      <c r="W33" s="5" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
@@ -2208,6 +2299,8 @@
       <c r="S34" s="5" t="inlineStr"/>
       <c r="T34" s="5" t="inlineStr"/>
       <c r="U34" s="5" t="inlineStr"/>
+      <c r="V34" s="5" t="n"/>
+      <c r="W34" s="5" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -2251,6 +2344,8 @@
       <c r="S35" s="5" t="inlineStr"/>
       <c r="T35" s="5" t="inlineStr"/>
       <c r="U35" s="5" t="inlineStr"/>
+      <c r="V35" s="5" t="n"/>
+      <c r="W35" s="5" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
@@ -2298,6 +2393,8 @@
       <c r="S36" s="5" t="inlineStr"/>
       <c r="T36" s="5" t="inlineStr"/>
       <c r="U36" s="5" t="inlineStr"/>
+      <c r="V36" s="5" t="n"/>
+      <c r="W36" s="5" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
@@ -2341,6 +2438,8 @@
       <c r="S37" s="5" t="inlineStr"/>
       <c r="T37" s="5" t="inlineStr"/>
       <c r="U37" s="5" t="inlineStr"/>
+      <c r="V37" s="5" t="n"/>
+      <c r="W37" s="5" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
@@ -2388,6 +2487,8 @@
       <c r="S38" s="5" t="inlineStr"/>
       <c r="T38" s="5" t="inlineStr"/>
       <c r="U38" s="5" t="inlineStr"/>
+      <c r="V38" s="5" t="n"/>
+      <c r="W38" s="5" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
@@ -2435,6 +2536,8 @@
       <c r="S39" s="5" t="inlineStr"/>
       <c r="T39" s="5" t="inlineStr"/>
       <c r="U39" s="5" t="inlineStr"/>
+      <c r="V39" s="5" t="n"/>
+      <c r="W39" s="5" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
@@ -2482,6 +2585,8 @@
       <c r="S40" s="5" t="inlineStr"/>
       <c r="T40" s="5" t="inlineStr"/>
       <c r="U40" s="5" t="inlineStr"/>
+      <c r="V40" s="5" t="n"/>
+      <c r="W40" s="5" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
@@ -2525,6 +2630,8 @@
       <c r="S41" s="5" t="inlineStr"/>
       <c r="T41" s="5" t="inlineStr"/>
       <c r="U41" s="5" t="inlineStr"/>
+      <c r="V41" s="5" t="n"/>
+      <c r="W41" s="5" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
@@ -2568,6 +2675,8 @@
       <c r="S42" s="5" t="inlineStr"/>
       <c r="T42" s="5" t="inlineStr"/>
       <c r="U42" s="5" t="inlineStr"/>
+      <c r="V42" s="5" t="n"/>
+      <c r="W42" s="5" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
@@ -2615,6 +2724,8 @@
       <c r="S43" s="5" t="inlineStr"/>
       <c r="T43" s="5" t="inlineStr"/>
       <c r="U43" s="5" t="inlineStr"/>
+      <c r="V43" s="5" t="n"/>
+      <c r="W43" s="5" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
@@ -2658,6 +2769,8 @@
       <c r="S44" s="5" t="inlineStr"/>
       <c r="T44" s="5" t="inlineStr"/>
       <c r="U44" s="5" t="inlineStr"/>
+      <c r="V44" s="5" t="n"/>
+      <c r="W44" s="5" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
@@ -2705,6 +2818,8 @@
       <c r="S45" s="5" t="inlineStr"/>
       <c r="T45" s="5" t="inlineStr"/>
       <c r="U45" s="5" t="inlineStr"/>
+      <c r="V45" s="5" t="n"/>
+      <c r="W45" s="5" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
@@ -2752,6 +2867,8 @@
       <c r="S46" s="5" t="inlineStr"/>
       <c r="T46" s="5" t="inlineStr"/>
       <c r="U46" s="5" t="inlineStr"/>
+      <c r="V46" s="5" t="n"/>
+      <c r="W46" s="5" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
@@ -2799,6 +2916,8 @@
       <c r="S47" s="5" t="inlineStr"/>
       <c r="T47" s="5" t="inlineStr"/>
       <c r="U47" s="5" t="inlineStr"/>
+      <c r="V47" s="5" t="n"/>
+      <c r="W47" s="5" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
@@ -2846,6 +2965,8 @@
       <c r="S48" s="5" t="inlineStr"/>
       <c r="T48" s="5" t="inlineStr"/>
       <c r="U48" s="5" t="inlineStr"/>
+      <c r="V48" s="5" t="n"/>
+      <c r="W48" s="5" t="n"/>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
@@ -2893,6 +3014,8 @@
       <c r="S49" s="5" t="inlineStr"/>
       <c r="T49" s="5" t="inlineStr"/>
       <c r="U49" s="5" t="inlineStr"/>
+      <c r="V49" s="5" t="n"/>
+      <c r="W49" s="5" t="n"/>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
@@ -2944,6 +3067,8 @@
           <t>Built from the old site copy. Revenue published by Iconic's one time exception. Interview Q4 and Q5 still open.</t>
         </is>
       </c>
+      <c r="V50" s="5" t="n"/>
+      <c r="W50" s="5" t="n"/>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
@@ -2991,6 +3116,8 @@
       <c r="S51" s="5" t="inlineStr"/>
       <c r="T51" s="5" t="inlineStr"/>
       <c r="U51" s="5" t="inlineStr"/>
+      <c r="V51" s="5" t="n"/>
+      <c r="W51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -3038,6 +3165,8 @@
       <c r="S52" s="5" t="inlineStr"/>
       <c r="T52" s="5" t="inlineStr"/>
       <c r="U52" s="5" t="inlineStr"/>
+      <c r="V52" s="5" t="n"/>
+      <c r="W52" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Record the CreatorHub Live right for answer and new interview rules
Add the Challenges Overcome section to the protocol, allow estimated
speaker and sponsor counts, and allow interview notes to be pushed to the
working branch without asking each time.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -740,7 +740,7 @@
       </c>
       <c r="V1" s="4" t="inlineStr">
         <is>
-          <t>What Nearly Broke</t>
+          <t>Challenges Overcome</t>
         </is>
       </c>
       <c r="W1" s="4" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>The hub model delivered the attendance the event needed. Three stages ran at once on a clean run of show.
+          <t>The hub model delivered the attendance the event needed. Three stages ran at once on a clean run of show, with about 40 speakers across them.
 The round tables, fireside chats with a speaker at each table, were planned for 45 minutes. Attendees loved them so much they stayed for about three and a half hours.</t>
         </is>
       </c>
@@ -1146,16 +1146,21 @@
       <c r="T9" s="5" t="inlineStr"/>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>Page needs two new sections for this: What Nearly Broke, and Right for / wrong for (Iconic to decide; protocol section 3). Heading on this page: How It Was Built, no first person. Speaker count: exact number needed (answer was about 40 to 60). Venue fix on the site: Marriott Bonnet Creek, Orlando, not FTL Downtown Event Center. Leads still to confirm: 36 round tables sold; 100+ testimonials from the on site studio; a 2026 edition in production.</t>
+          <t>Heading on this page: How It Was Built, no first person. Venue fix on the site: Marriott Bonnet Creek, Orlando, not FTL Downtown Event Center. Leads still to confirm: 36 round tables sold; 100+ testimonials from the on site studio; a 2026 edition in production. Wrong for: not answered.</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>Ticket sales opened before the hubs were ready, so the first couple of months were a rocky road, with real uncertainty about where ticket sales stood.
-The Lamborghini nearly did not make it in. It was the performance version, wider than planned, and it cleared the doorway by a couple of millimeters on each side after a door came off the Marriott. Without it the mixer would have had nothing, Lamborghini would have been a disappointed sponsor, and a badly built enclosure could have meant hundreds of thousands of dollars in insurance claims if paint escaped into the venue.</t>
-        </is>
-      </c>
-      <c r="W9" s="5" t="n"/>
+          <t>Ticket sales opened before the hubs were ready, and the first couple of months were uncertain. The answer was the hub model itself: once other events could contract a stage and bring their own communities, attendance followed.
+The Lamborghini turned out to be the performance version, wider than planned. Getting it inside took removing a door from the Marriott and threading it through with a couple of millimeters to spare on each side, then sealing it in a 50 foot glass enclosure so not a drop of paint reached the venue. The mixer went ahead with its centerpiece, Lamborghini got the moment it signed up for, and the venue stayed spotless.</t>
+        </is>
+      </c>
+      <c r="W9" s="7" t="inlineStr">
+        <is>
+          <t>Right for: companies that want a front row seat in the creator economy and a direct line to creators who are building real businesses, and companies that help brands build digital media empires, with total coverage across the internet.
+Wrong for: not answered yet.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Finish the CreatorHub Live interview draft
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1120,15 +1120,39 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>The hub model delivered the attendance the event needed. Three stages ran at once on a clean run of show, with about 40 speakers across them.
-The round tables, fireside chats with a speaker at each table, were planned for 45 minutes. Attendees loved them so much they stayed for about three and a half hours.</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr"/>
-      <c r="K9" s="5" t="inlineStr"/>
-      <c r="L9" s="5" t="inlineStr"/>
-      <c r="M9" s="5" t="inlineStr"/>
+          <t>The hub model delivered the attendance the event needed: more than 1,500 people over three and a half days. Three stages ran at once on a clean run of show, with about 40 speakers across them.
+The round tables, fireside chats with a speaker at each table, were planned for 45 minutes. Attendees loved them so much they stayed for about three and a half hours.
+The standout moment came at the mixer. The live Lamborghini painting was the draw, and an auto tune microphone passed around the room took it up a level, with attendees singing to each other.
+The event is renewing for 2027. The organic content from this edition is what lets the next one aim for 3,000 people.</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>1,500+ | Attendees
+3 | Stages running at once
+3.5 hrs | Round tables, planned for 45 minutes</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Owner and producer: event strategy, sponsorship design (a la carte packages, brand activations), the hub model, venue and vendor coordination with the Marriott, three stage production and show flow, the Lamborghini build and on site execution.</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>CreatorHub Live set out to fill a gap: no event brought entrepreneurs and creators together to learn business and media production, and the biggest event at this capacity belonged to MrBeast. Sponsors and attendees were wary of a brand new event. The answer was a hub model, where other events ran their own stages inside CreatorHub, plus a la carte sponsorships and a Lamborghini painted live at the mixer. More than 1,500 people attended over three and a half days at the Marriott Bonnet Creek in Orlando, and the event is now building toward 3,000 in 2027.</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>How CreatorHub Live Brought 1,500+ Creators and Entrepreneurs Under One Roof</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>Want to bring your community under one roof?</t>
+        </is>
+      </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
           <t>Marriott Bonnet Creek, Orlando, FL</t>
@@ -1136,17 +1160,21 @@
       </c>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>917</t>
-        </is>
-      </c>
-      <c r="P9" s="5" t="inlineStr"/>
+          <t>1,500+</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
       <c r="Q9" s="5" t="inlineStr"/>
       <c r="R9" s="5" t="inlineStr"/>
       <c r="S9" s="5" t="inlineStr"/>
       <c r="T9" s="5" t="inlineStr"/>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>Heading on this page: How It Was Built, no first person. Venue fix on the site: Marriott Bonnet Creek, Orlando, not FTL Downtown Event Center. Leads still to confirm: 36 round tables sold; 100+ testimonials from the on site studio; a 2026 edition in production. Wrong for: not answered.</t>
+          <t>Heading on this page: How It Was Built, no first person. Site fixes when built: venue Marriott Bonnet Creek, Orlando (not FTL Downtown Event Center), attendance 1,500+ (not 917), date August 2025. Attendance was given as "north of about 1,500": 1,500+ is the floor. Auto tune moment: the sentence trailed off; anything to add? Scope is drafted from the interview, check it.</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
@@ -1157,8 +1185,7 @@
       </c>
       <c r="W9" s="7" t="inlineStr">
         <is>
-          <t>Right for: companies that want a front row seat in the creator economy and a direct line to creators who are building real businesses, and companies that help brands build digital media empires, with total coverage across the internet.
-Wrong for: not answered yet.</t>
+          <t>Right for: companies that want a front row seat in the creator economy and a direct line to creators who are building real businesses, and companies that help brands build digital media empires, with total coverage across the internet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add the CreatorHub Live podcast studios to its draft
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1115,7 +1115,8 @@
 2. Replaced the standard gold, platinum and silver packages with a la carte options, so each sponsor could find a natural way into the event.
 3. Built the hub model: other events contract one of the stages and run their own mini event inside CreatorHub, which is where the name comes from. It put attendees from several communities under one roof with the same purpose, and it is what delivered the attendance.
 4. Ran three stages at once as three separate events that happened to share a building, each with its own dedicated stage manager.
-5. Brought a Lamborghini into the Marriott Bonnet Creek to be painted live during the networking mixer, inside a 50 foot glass enclosure built with the Marriott so not a drop of paint touched the venue.</t>
+5. Brought a Lamborghini into the Marriott Bonnet Creek to be painted live during the networking mixer, inside a 50 foot glass enclosure built with the Marriott so not a drop of paint touched the venue.
+6. Planned the content strategy around live podcast studios that ran throughout the event, so every hour on site doubled as content production.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -1123,7 +1124,7 @@
           <t>The hub model delivered the attendance the event needed: more than 1,500 people over three and a half days. Three stages ran at once on a clean run of show, with about 40 speakers across them.
 The round tables, fireside chats with a speaker at each table, were planned for 45 minutes. Attendees loved them so much they stayed for about three and a half hours.
 The standout moment came at the mixer. The live Lamborghini painting was the draw, and an auto tune microphone passed around the room took it up a level, with attendees singing to each other.
-The event is renewing for 2027. The organic content from this edition is what lets the next one aim for 3,000 people.</t>
+The live podcast studios captured dozens of testimonials and hundreds of clips. That organic content is what the event is renewing on: it fuels the 2027 edition, which is aiming for 3,000 people.</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
@@ -1135,7 +1136,7 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Owner and producer: event strategy, sponsorship design (a la carte packages, brand activations), the hub model, venue and vendor coordination with the Marriott, three stage production and show flow, the Lamborghini build and on site execution.</t>
+          <t>Owner and producer: event strategy, sponsorship design (a la carte packages, brand activations), the hub model, content strategy and live podcast studios, venue and vendor coordination with the Marriott, three stage production and show flow, the Lamborghini build and on site execution.</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Approve the CreatorHub Live draft and add a Steal This block
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -47,7 +47,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -113,6 +118,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -604,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W52"/>
+  <dimension ref="A1:X52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -630,6 +638,7 @@
     <col width="50" customWidth="1" min="21" max="21"/>
     <col width="60" customWidth="1" min="22" max="22"/>
     <col width="60" customWidth="1" min="23" max="23"/>
+    <col width="60" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -746,6 +755,11 @@
       <c r="W1" s="4" t="inlineStr">
         <is>
           <t>Right for / wrong for</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>Steal This</t>
         </is>
       </c>
     </row>
@@ -797,6 +811,7 @@
       <c r="U2" s="5" t="inlineStr"/>
       <c r="V2" s="5" t="n"/>
       <c r="W2" s="5" t="n"/>
+      <c r="X2" s="5" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -846,6 +861,7 @@
       <c r="U3" s="5" t="inlineStr"/>
       <c r="V3" s="5" t="n"/>
       <c r="W3" s="5" t="n"/>
+      <c r="X3" s="5" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -891,6 +907,7 @@
       <c r="U4" s="5" t="inlineStr"/>
       <c r="V4" s="5" t="n"/>
       <c r="W4" s="5" t="n"/>
+      <c r="X4" s="5" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -936,6 +953,7 @@
       <c r="U5" s="5" t="inlineStr"/>
       <c r="V5" s="5" t="n"/>
       <c r="W5" s="5" t="n"/>
+      <c r="X5" s="5" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -981,6 +999,7 @@
       <c r="U6" s="5" t="inlineStr"/>
       <c r="V6" s="5" t="n"/>
       <c r="W6" s="5" t="n"/>
+      <c r="X6" s="5" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -1030,6 +1049,7 @@
       <c r="U7" s="5" t="inlineStr"/>
       <c r="V7" s="5" t="n"/>
       <c r="W7" s="5" t="n"/>
+      <c r="X7" s="5" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -1075,6 +1095,7 @@
       <c r="U8" s="5" t="inlineStr"/>
       <c r="V8" s="5" t="n"/>
       <c r="W8" s="5" t="n"/>
+      <c r="X8" s="5" t="n"/>
     </row>
     <row r="9" ht="330" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -1087,29 +1108,29 @@
           <t>creatorhub-live</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>August 2025</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>None. Iconic's own event, co-owned with Xtend Creators</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
+          <t>Ready to build</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>There was no event where entrepreneurs and creators could come together to learn business and media production. The largest event at this capacity was run and owned by MrBeast, the biggest media entity on the planet, so building something people would trust enough to pay for meant pushing through heavy resistance.
 A brand new event with no history is a hard sell in the creator economy. Sponsors did not want to be first in, the platforms that mattered most, YouTube, TikTok and Snapchat, had to be won over, and getting bodies in the room was just as hard.
 The stakes were a multi six figure investment, the reputation of everyone involved, and the trust of the speakers and creators brought in by co-owner Xtend Creators. If it flopped, Patrick Israel and Xtend would lose relational capital with every sponsor and creator they had brought to the table.</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>1. Rebuilt the sponsorship strategy around in person meetings, and used after party brand activations to give partners a way in.
 2. Replaced the standard gold, platinum and silver packages with a la carte options, so each sponsor could find a natural way into the event.
@@ -1119,7 +1140,7 @@
 6. Planned the content strategy around live podcast studios that ran throughout the event, so every hour on site doubled as content production.</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>The hub model delivered the attendance the event needed: more than 1,500 people over three and a half days. Three stages ran at once on a clean run of show, with about 40 speakers across them.
 The round tables, fireside chats with a speaker at each table, were planned for 45 minutes. Attendees loved them so much they stayed for about three and a half hours.
@@ -1127,44 +1148,44 @@
 The live podcast studios captured dozens of testimonials and hundreds of clips. That organic content is what the event is renewing on: it fuels the 2027 edition, which is aiming for 3,000 people.</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>1,500+ | Attendees
 3 | Stages running at once
 3.5 hrs | Round tables, planned for 45 minutes</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>Owner and producer: event strategy, sponsorship design (a la carte packages, brand activations), the hub model, content strategy and live podcast studios, venue and vendor coordination with the Marriott, three stage production and show flow, the Lamborghini build and on site execution.</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="K9" s="8" t="inlineStr">
         <is>
           <t>CreatorHub Live set out to fill a gap: no event brought entrepreneurs and creators together to learn business and media production, and the biggest event at this capacity belonged to MrBeast. Sponsors and attendees were wary of a brand new event. The answer was a hub model, where other events ran their own stages inside CreatorHub, plus a la carte sponsorships and a Lamborghini painted live at the mixer. More than 1,500 people attended over three and a half days at the Marriott Bonnet Creek in Orlando, and the event is now building toward 3,000 in 2027.</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr">
+      <c r="L9" s="8" t="inlineStr">
         <is>
           <t>How CreatorHub Live Brought 1,500+ Creators and Entrepreneurs Under One Roof</t>
         </is>
       </c>
-      <c r="M9" s="7" t="inlineStr">
+      <c r="M9" s="8" t="inlineStr">
         <is>
           <t>Want to bring your community under one roof?</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr">
+      <c r="N9" s="8" t="inlineStr">
         <is>
           <t>Marriott Bonnet Creek, Orlando, FL</t>
         </is>
       </c>
-      <c r="O9" s="7" t="inlineStr">
+      <c r="O9" s="8" t="inlineStr">
         <is>
           <t>1,500+</t>
         </is>
       </c>
-      <c r="P9" s="7" t="inlineStr">
+      <c r="P9" s="8" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
@@ -1173,20 +1194,27 @@
       <c r="R9" s="5" t="inlineStr"/>
       <c r="S9" s="5" t="inlineStr"/>
       <c r="T9" s="5" t="inlineStr"/>
-      <c r="U9" s="7" t="inlineStr">
-        <is>
-          <t>Heading on this page: How It Was Built, no first person. Site fixes when built: venue Marriott Bonnet Creek, Orlando (not FTL Downtown Event Center), attendance 1,500+ (not 917), date August 2025. Attendance was given as "north of about 1,500": 1,500+ is the floor. Auto tune moment: the sentence trailed off; anything to add? Scope is drafted from the interview, check it.</t>
-        </is>
-      </c>
-      <c r="V9" s="7" t="inlineStr">
+      <c r="U9" s="5" t="inlineStr">
+        <is>
+          <t>Approved by Iconic 2026-09-30, except Steal This (new). Heading on this page: How It Was Built, no first person. Site fixes when built: venue Marriott Bonnet Creek, Orlando; attendance 1,500+; date August 2025.</t>
+        </is>
+      </c>
+      <c r="V9" s="8" t="inlineStr">
         <is>
           <t>Ticket sales opened before the hubs were ready, and the first couple of months were uncertain. The answer was the hub model itself: once other events could contract a stage and bring their own communities, attendance followed.
 The Lamborghini turned out to be the performance version, wider than planned. Getting it inside took removing a door from the Marriott and threading it through with a couple of millimeters to spare on each side, then sealing it in a 50 foot glass enclosure so not a drop of paint reached the venue. The mixer went ahead with its centerpiece, Lamborghini got the moment it signed up for, and the venue stayed spotless.</t>
         </is>
       </c>
-      <c r="W9" s="7" t="inlineStr">
+      <c r="W9" s="8" t="inlineStr">
         <is>
           <t>Right for: companies that want a front row seat in the creator economy and a direct line to creators who are building real businesses, and companies that help brands build digital media empires, with total coverage across the internet.</t>
+        </is>
+      </c>
+      <c r="X9" s="7" t="inlineStr">
+        <is>
+          <t>Two ideas any event host can take:
+Run a live podcast studio the whole time. Attendees and speakers step in between sessions, and the event walks away with dozens of testimonials and hundreds of clips to market the next edition.
+Borrow the hub model. Let other events contract a stage and run their own mini event inside yours. Each one brings its own community, so the room fills from several audiences at once, all there for the same reason.</t>
         </is>
       </c>
     </row>
@@ -1242,6 +1270,7 @@
       </c>
       <c r="V10" s="5" t="n"/>
       <c r="W10" s="5" t="n"/>
+      <c r="X10" s="5" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1291,6 +1320,7 @@
       <c r="U11" s="5" t="inlineStr"/>
       <c r="V11" s="5" t="n"/>
       <c r="W11" s="5" t="n"/>
+      <c r="X11" s="5" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -1336,6 +1366,7 @@
       <c r="U12" s="5" t="inlineStr"/>
       <c r="V12" s="5" t="n"/>
       <c r="W12" s="5" t="n"/>
+      <c r="X12" s="5" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1381,6 +1412,7 @@
       <c r="U13" s="5" t="inlineStr"/>
       <c r="V13" s="5" t="n"/>
       <c r="W13" s="5" t="n"/>
+      <c r="X13" s="5" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -1426,6 +1458,7 @@
       <c r="U14" s="5" t="inlineStr"/>
       <c r="V14" s="5" t="n"/>
       <c r="W14" s="5" t="n"/>
+      <c r="X14" s="5" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1471,6 +1504,7 @@
       <c r="U15" s="5" t="inlineStr"/>
       <c r="V15" s="5" t="n"/>
       <c r="W15" s="5" t="n"/>
+      <c r="X15" s="5" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -1516,6 +1550,7 @@
       <c r="U16" s="5" t="inlineStr"/>
       <c r="V16" s="5" t="n"/>
       <c r="W16" s="5" t="n"/>
+      <c r="X16" s="5" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -1561,6 +1596,7 @@
       <c r="U17" s="5" t="inlineStr"/>
       <c r="V17" s="5" t="n"/>
       <c r="W17" s="5" t="n"/>
+      <c r="X17" s="5" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1606,6 +1642,7 @@
       <c r="U18" s="5" t="inlineStr"/>
       <c r="V18" s="5" t="n"/>
       <c r="W18" s="5" t="n"/>
+      <c r="X18" s="5" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1651,6 +1688,7 @@
       <c r="U19" s="5" t="inlineStr"/>
       <c r="V19" s="5" t="n"/>
       <c r="W19" s="5" t="n"/>
+      <c r="X19" s="5" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -1696,6 +1734,7 @@
       <c r="U20" s="5" t="inlineStr"/>
       <c r="V20" s="5" t="n"/>
       <c r="W20" s="5" t="n"/>
+      <c r="X20" s="5" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -1741,6 +1780,7 @@
       <c r="U21" s="5" t="inlineStr"/>
       <c r="V21" s="5" t="n"/>
       <c r="W21" s="5" t="n"/>
+      <c r="X21" s="5" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -1786,6 +1826,7 @@
       <c r="U22" s="5" t="inlineStr"/>
       <c r="V22" s="5" t="n"/>
       <c r="W22" s="5" t="n"/>
+      <c r="X22" s="5" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -1831,6 +1872,7 @@
       <c r="U23" s="5" t="inlineStr"/>
       <c r="V23" s="5" t="n"/>
       <c r="W23" s="5" t="n"/>
+      <c r="X23" s="5" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
@@ -1876,6 +1918,7 @@
       <c r="U24" s="5" t="inlineStr"/>
       <c r="V24" s="5" t="n"/>
       <c r="W24" s="5" t="n"/>
+      <c r="X24" s="5" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -1925,6 +1968,7 @@
       <c r="U25" s="5" t="inlineStr"/>
       <c r="V25" s="5" t="n"/>
       <c r="W25" s="5" t="n"/>
+      <c r="X25" s="5" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
@@ -1970,6 +2014,7 @@
       <c r="U26" s="5" t="inlineStr"/>
       <c r="V26" s="5" t="n"/>
       <c r="W26" s="5" t="n"/>
+      <c r="X26" s="5" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -2015,6 +2060,7 @@
       <c r="U27" s="5" t="inlineStr"/>
       <c r="V27" s="5" t="n"/>
       <c r="W27" s="5" t="n"/>
+      <c r="X27" s="5" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
@@ -2060,6 +2106,7 @@
       <c r="U28" s="5" t="inlineStr"/>
       <c r="V28" s="5" t="n"/>
       <c r="W28" s="5" t="n"/>
+      <c r="X28" s="5" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -2109,6 +2156,7 @@
       <c r="U29" s="5" t="inlineStr"/>
       <c r="V29" s="5" t="n"/>
       <c r="W29" s="5" t="n"/>
+      <c r="X29" s="5" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
@@ -2154,6 +2202,7 @@
       <c r="U30" s="5" t="inlineStr"/>
       <c r="V30" s="5" t="n"/>
       <c r="W30" s="5" t="n"/>
+      <c r="X30" s="5" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -2199,6 +2248,7 @@
       <c r="U31" s="5" t="inlineStr"/>
       <c r="V31" s="5" t="n"/>
       <c r="W31" s="5" t="n"/>
+      <c r="X31" s="5" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
@@ -2244,6 +2294,7 @@
       <c r="U32" s="5" t="inlineStr"/>
       <c r="V32" s="5" t="n"/>
       <c r="W32" s="5" t="n"/>
+      <c r="X32" s="5" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -2289,6 +2340,7 @@
       <c r="U33" s="5" t="inlineStr"/>
       <c r="V33" s="5" t="n"/>
       <c r="W33" s="5" t="n"/>
+      <c r="X33" s="5" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
@@ -2334,6 +2386,7 @@
       <c r="U34" s="5" t="inlineStr"/>
       <c r="V34" s="5" t="n"/>
       <c r="W34" s="5" t="n"/>
+      <c r="X34" s="5" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -2379,6 +2432,7 @@
       <c r="U35" s="5" t="inlineStr"/>
       <c r="V35" s="5" t="n"/>
       <c r="W35" s="5" t="n"/>
+      <c r="X35" s="5" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
@@ -2428,6 +2482,7 @@
       <c r="U36" s="5" t="inlineStr"/>
       <c r="V36" s="5" t="n"/>
       <c r="W36" s="5" t="n"/>
+      <c r="X36" s="5" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
@@ -2473,6 +2528,7 @@
       <c r="U37" s="5" t="inlineStr"/>
       <c r="V37" s="5" t="n"/>
       <c r="W37" s="5" t="n"/>
+      <c r="X37" s="5" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
@@ -2522,6 +2578,7 @@
       <c r="U38" s="5" t="inlineStr"/>
       <c r="V38" s="5" t="n"/>
       <c r="W38" s="5" t="n"/>
+      <c r="X38" s="5" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
@@ -2571,6 +2628,7 @@
       <c r="U39" s="5" t="inlineStr"/>
       <c r="V39" s="5" t="n"/>
       <c r="W39" s="5" t="n"/>
+      <c r="X39" s="5" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
@@ -2620,6 +2678,7 @@
       <c r="U40" s="5" t="inlineStr"/>
       <c r="V40" s="5" t="n"/>
       <c r="W40" s="5" t="n"/>
+      <c r="X40" s="5" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
@@ -2665,6 +2724,7 @@
       <c r="U41" s="5" t="inlineStr"/>
       <c r="V41" s="5" t="n"/>
       <c r="W41" s="5" t="n"/>
+      <c r="X41" s="5" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
@@ -2710,6 +2770,7 @@
       <c r="U42" s="5" t="inlineStr"/>
       <c r="V42" s="5" t="n"/>
       <c r="W42" s="5" t="n"/>
+      <c r="X42" s="5" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
@@ -2759,6 +2820,7 @@
       <c r="U43" s="5" t="inlineStr"/>
       <c r="V43" s="5" t="n"/>
       <c r="W43" s="5" t="n"/>
+      <c r="X43" s="5" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
@@ -2804,6 +2866,7 @@
       <c r="U44" s="5" t="inlineStr"/>
       <c r="V44" s="5" t="n"/>
       <c r="W44" s="5" t="n"/>
+      <c r="X44" s="5" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
@@ -2853,6 +2916,7 @@
       <c r="U45" s="5" t="inlineStr"/>
       <c r="V45" s="5" t="n"/>
       <c r="W45" s="5" t="n"/>
+      <c r="X45" s="5" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
@@ -2902,6 +2966,7 @@
       <c r="U46" s="5" t="inlineStr"/>
       <c r="V46" s="5" t="n"/>
       <c r="W46" s="5" t="n"/>
+      <c r="X46" s="5" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
@@ -2951,6 +3016,7 @@
       <c r="U47" s="5" t="inlineStr"/>
       <c r="V47" s="5" t="n"/>
       <c r="W47" s="5" t="n"/>
+      <c r="X47" s="5" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
@@ -3000,6 +3066,7 @@
       <c r="U48" s="5" t="inlineStr"/>
       <c r="V48" s="5" t="n"/>
       <c r="W48" s="5" t="n"/>
+      <c r="X48" s="5" t="n"/>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
@@ -3049,6 +3116,7 @@
       <c r="U49" s="5" t="inlineStr"/>
       <c r="V49" s="5" t="n"/>
       <c r="W49" s="5" t="n"/>
+      <c r="X49" s="5" t="n"/>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
@@ -3102,6 +3170,7 @@
       </c>
       <c r="V50" s="5" t="n"/>
       <c r="W50" s="5" t="n"/>
+      <c r="X50" s="5" t="n"/>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
@@ -3151,6 +3220,7 @@
       <c r="U51" s="5" t="inlineStr"/>
       <c r="V51" s="5" t="n"/>
       <c r="W51" s="5" t="n"/>
+      <c r="X51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -3200,6 +3270,7 @@
       <c r="U52" s="5" t="inlineStr"/>
       <c r="V52" s="5" t="n"/>
       <c r="W52" s="5" t="n"/>
+      <c r="X52" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Skip Creator Hub Madrid for now and start Freedom Queen Live 2024
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1265,7 +1265,7 @@
       <c r="T10" s="5" t="inlineStr"/>
       <c r="U10" s="7" t="inlineStr">
         <is>
-          <t>The first edition of what became CreatorHub Live. Not on the website grid yet; add it with the next approved site change.</t>
+          <t>The first edition of what became CreatorHub Live. Not on the website grid yet; add it with the next approved site change. Skipped for now (Iconic, 2026-09-30).</t>
         </is>
       </c>
       <c r="V10" s="5" t="n"/>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr"/>
@@ -1317,7 +1317,11 @@
       <c r="R11" s="5" t="inlineStr"/>
       <c r="S11" s="5" t="inlineStr"/>
       <c r="T11" s="5" t="inlineStr"/>
-      <c r="U11" s="5" t="inlineStr"/>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>Skipped for now (Iconic, 2026-09-30).</t>
+        </is>
+      </c>
       <c r="V11" s="5" t="n"/>
       <c r="W11" s="5" t="n"/>
       <c r="X11" s="5" t="n"/>
@@ -1713,7 +1717,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Interviewing</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Record the first Freedom Queen Live 2024 answer and draft its problem
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1694,7 +1694,7 @@
       <c r="W19" s="5" t="n"/>
       <c r="X19" s="5" t="n"/>
     </row>
-    <row r="20" ht="18" customHeight="1">
+    <row r="20" ht="90" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Freedom Queen Live 2024</t>
@@ -1720,7 +1720,11 @@
           <t>Interviewing</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr"/>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Bridget James Ling had never run a live event, but she had already built a devoted community of Freedom Queens. Her first event had to meet their expectations and live up to the legacy and class of the Freedom Queen name.</t>
+        </is>
+      </c>
       <c r="G20" s="5" t="inlineStr"/>
       <c r="H20" s="5" t="inlineStr"/>
       <c r="I20" s="5" t="inlineStr"/>
@@ -1735,7 +1739,11 @@
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr"/>
       <c r="T20" s="5" t="inlineStr"/>
-      <c r="U20" s="5" t="inlineStr"/>
+      <c r="U20" s="5" t="inlineStr">
+        <is>
+          <t>First edition. No stakes on the page (Iconic). Round tables lead: 40 sold, edition unknown.</t>
+        </is>
+      </c>
       <c r="V20" s="5" t="n"/>
       <c r="W20" s="5" t="n"/>
       <c r="X20" s="5" t="n"/>

</xml_diff>

<commit_message>
Record the Freedom Queen Live 2024 venue answer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1694,7 +1694,7 @@
       <c r="W19" s="5" t="n"/>
       <c r="X19" s="5" t="n"/>
     </row>
-    <row r="20" ht="90" customHeight="1">
+    <row r="20" ht="150" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Freedom Queen Live 2024</t>
@@ -1722,17 +1722,26 @@
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Bridget James Ling had never run a live event, but she had already built a devoted community of Freedom Queens. Her first event had to meet their expectations and live up to the legacy and class of the Freedom Queen name.</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr"/>
+          <t>Bridget James Ling had never run a live event, but she had already built a devoted community of Freedom Queens. Her first event had to meet their expectations and live up to the legacy and class of the Freedom Queen name.
+Attendees did not know what to expect, so the room had to answer that question the moment they walked in. It had to be in the Tampa area at Bridget's request, and it had to feel as elegant and timeless as her brand.</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>1. Chose the Vinoy: in the Tampa area as Bridget asked, and as elegant and timeless as the Freedom Queen brand.</t>
+        </is>
+      </c>
       <c r="H20" s="5" t="inlineStr"/>
       <c r="I20" s="5" t="inlineStr"/>
       <c r="J20" s="5" t="inlineStr"/>
       <c r="K20" s="5" t="inlineStr"/>
       <c r="L20" s="5" t="inlineStr"/>
       <c r="M20" s="5" t="inlineStr"/>
-      <c r="N20" s="5" t="inlineStr"/>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>The Vinoy (city to confirm: St. Petersburg?)</t>
+        </is>
+      </c>
       <c r="O20" s="5" t="inlineStr"/>
       <c r="P20" s="5" t="inlineStr"/>
       <c r="Q20" s="5" t="inlineStr"/>
@@ -1741,7 +1750,7 @@
       <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>First edition. No stakes on the page (Iconic). Round tables lead: 40 sold, edition unknown.</t>
+          <t>First edition. No stakes on the page (Iconic). Venue city: the Vinoy is in St. Petersburg, Tampa Bay; confirm. Round tables lead: 40 sold, edition unknown, revenue anyway.</t>
         </is>
       </c>
       <c r="V20" s="5" t="n"/>

</xml_diff>

<commit_message>
Record the Freedom Queen Live 2024 decisions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1728,7 +1728,9 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>1. Chose the Vinoy: in the Tampa area as Bridget asked, and as elegant and timeless as the Freedom Queen brand.</t>
+          <t>1. Chose the Vinoy in St. Petersburg: in the Tampa Bay area as Bridget asked, and as elegant and timeless as the Freedom Queen brand.
+2. Built installations that added to the experience instead of decorating it, like a wishing tree where attendees wrote a physical prayer and hung it on the branches.
+3. Helped Bridget design the offer for her first large sales from stage event.</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr"/>
@@ -1739,7 +1741,7 @@
       <c r="M20" s="5" t="inlineStr"/>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>The Vinoy (city to confirm: St. Petersburg?)</t>
+          <t>The Vinoy, St. Petersburg, FL</t>
         </is>
       </c>
       <c r="O20" s="5" t="inlineStr"/>
@@ -1750,7 +1752,7 @@
       <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>First edition. No stakes on the page (Iconic). Venue city: the Vinoy is in St. Petersburg, Tampa Bay; confirm. Round tables lead: 40 sold, edition unknown, revenue anyway.</t>
+          <t>First edition. No stakes on the page (Iconic). Do not mention the sales team (Iconic). Step 3, the offer design: keep it, or two decisions only? Round tables lead: 40 sold, edition unknown, revenue anyway.</t>
         </is>
       </c>
       <c r="V20" s="5" t="n"/>

</xml_diff>

<commit_message>
Record the Freedom Queen Live 2024 right for answer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1752,11 +1752,19 @@
       <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>First edition. No stakes on the page (Iconic). Do not mention the sales team (Iconic). Step 3, the offer design: keep it, or two decisions only? Round tables lead: 40 sold, edition unknown, revenue anyway.</t>
-        </is>
-      </c>
-      <c r="V20" s="5" t="n"/>
-      <c r="W20" s="5" t="n"/>
+          <t>First edition. No stakes on the page. Do not mention the sales team. No Challenges Overcome section. Round tables lead: 40 sold, edition unknown, revenue anyway.</t>
+        </is>
+      </c>
+      <c r="V20" s="5" t="inlineStr">
+        <is>
+          <t>None (Iconic: no challenges overcome for this event).</t>
+        </is>
+      </c>
+      <c r="W20" s="7" t="inlineStr">
+        <is>
+          <t>Right for: a founder with a loyal community who wants a more reserved, timeless experience. Less about mixers and parties, more about the education.</t>
+        </is>
+      </c>
       <c r="X20" s="5" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">

</xml_diff>

<commit_message>
Draft the rest of the Freedom Queen Live 2024 row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1694,7 +1694,7 @@
       <c r="W19" s="5" t="n"/>
       <c r="X19" s="5" t="n"/>
     </row>
-    <row r="20" ht="150" customHeight="1">
+    <row r="20" ht="200" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Freedom Queen Live 2024</t>
@@ -1733,26 +1733,63 @@
 3. Helped Bridget design the offer for her first large sales from stage event.</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr"/>
-      <c r="I20" s="5" t="inlineStr"/>
-      <c r="J20" s="5" t="inlineStr"/>
-      <c r="K20" s="5" t="inlineStr"/>
-      <c r="L20" s="5" t="inlineStr"/>
-      <c r="M20" s="5" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>The event went phenomenally. Bridget launched her offer from the stage, and her Freedom Queens left thrilled, bonded and connected to each other. That connection became the foundation of her next step: she launched her inner circle community.</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>400 | Freedom Queens on site
+1st | Live event, and her first offer launched from stage</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>Venue sourcing and selection, installation design including the wishing tree, offer design support for her first sales from stage, event production and on site execution.</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>Bridget James Ling had built a devoted community of Freedom Queens but had never run a live event. Her first had to meet their expectations and live up to the elegance of her brand. We chose the Vinoy in St. Petersburg for its timeless feel, built installations like a wishing tree where attendees hung a written prayer, and helped her design the offer for her first sales from stage event. About 400 attendees left bonded and connected, Bridget launched her offer, and she opened her inner circle community.</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>How Bridget James Ling Launched Her First Live Event and Her Inner Circle at Freedom Queen Live</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>Want your community's first live event to feel like it has always existed?</t>
+        </is>
+      </c>
       <c r="N20" s="7" t="inlineStr">
         <is>
           <t>The Vinoy, St. Petersburg, FL</t>
         </is>
       </c>
-      <c r="O20" s="5" t="inlineStr"/>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>About 400 (confirm how to publish)</t>
+        </is>
+      </c>
       <c r="P20" s="5" t="inlineStr"/>
       <c r="Q20" s="5" t="inlineStr"/>
-      <c r="R20" s="5" t="inlineStr"/>
-      <c r="S20" s="5" t="inlineStr"/>
+      <c r="R20" s="7" t="inlineStr">
+        <is>
+          <t>Exists, link needed</t>
+        </is>
+      </c>
+      <c r="S20" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>First edition. No stakes on the page. Do not mention the sales team. No Challenges Overcome section. Round tables lead: 40 sold, edition unknown, revenue anyway.</t>
+          <t>First edition. No stakes on the page. Do not mention the sales team. No Challenges Overcome section. Attendance was given as about 400: publish as 400, or hold for the exact count (house rule 3 allows estimates only for speakers and sponsors). Days on site? Aftermovie link? No photo folder on file.</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
@@ -1765,7 +1802,11 @@
           <t>Right for: a founder with a loyal community who wants a more reserved, timeless experience. Less about mixers and parties, more about the education.</t>
         </is>
       </c>
-      <c r="X20" s="5" t="n"/>
+      <c r="X20" s="7" t="inlineStr">
+        <is>
+          <t>Build a wishing tree. Give attendees a physical place to write a prayer or intention for the next event and hang it on the branches. It turns a moment of reflection into a shared installation, and it gives your community a reason to come back and see what came true.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Approve the Freedom Queen Live 2024 row and start 2025
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Interviewing</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr"/>
@@ -1717,79 +1717,87 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
+          <t>Ready to build</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>Bridget James Ling had never run a live event, but she had already built a devoted community of Freedom Queens. Her first event had to meet their expectations and live up to the legacy and class of the Freedom Queen name.
 Attendees did not know what to expect, so the room had to answer that question the moment they walked in. It had to be in the Tampa area at Bridget's request, and it had to feel as elegant and timeless as her brand.</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>1. Chose the Vinoy in St. Petersburg: in the Tampa Bay area as Bridget asked, and as elegant and timeless as the Freedom Queen brand.
 2. Built installations that added to the experience instead of decorating it, like a wishing tree where attendees wrote a physical prayer and hung it on the branches.
 3. Helped Bridget design the offer for her first large sales from stage event.</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>The event went phenomenally. Bridget launched her offer from the stage, and her Freedom Queens left thrilled, bonded and connected to each other. That connection became the foundation of her next step: she launched her inner circle community.</t>
-        </is>
-      </c>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>400 | Freedom Queens on site
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>The event went phenomenally, with 451 attendees on site over three and a half days. Bridget launched her offer from the stage, and her Freedom Queens left thrilled, bonded and connected to each other. That connection became the foundation of her next step: she launched her inner circle community.</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>451 | Freedom Queens on site
 1st | Live event, and her first offer launched from stage</t>
         </is>
       </c>
-      <c r="J20" s="7" t="inlineStr">
+      <c r="J20" s="8" t="inlineStr">
         <is>
           <t>Venue sourcing and selection, installation design including the wishing tree, offer design support for her first sales from stage, event production and on site execution.</t>
         </is>
       </c>
-      <c r="K20" s="7" t="inlineStr">
-        <is>
-          <t>Bridget James Ling had built a devoted community of Freedom Queens but had never run a live event. Her first had to meet their expectations and live up to the elegance of her brand. We chose the Vinoy in St. Petersburg for its timeless feel, built installations like a wishing tree where attendees hung a written prayer, and helped her design the offer for her first sales from stage event. About 400 attendees left bonded and connected, Bridget launched her offer, and she opened her inner circle community.</t>
-        </is>
-      </c>
-      <c r="L20" s="7" t="inlineStr">
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>Bridget James Ling had built a devoted community of Freedom Queens but had never run a live event. Her first had to meet their expectations and live up to the elegance of her brand. We chose the Vinoy in St. Petersburg for its timeless feel, built installations like a wishing tree where attendees hung a written prayer, and helped her design the offer for her first sales from stage event. 451 attendees left bonded and connected, Bridget launched her offer, and she opened her inner circle community.</t>
+        </is>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
         <is>
           <t>How Bridget James Ling Launched Her First Live Event and Her Inner Circle at Freedom Queen Live</t>
         </is>
       </c>
-      <c r="M20" s="7" t="inlineStr">
+      <c r="M20" s="8" t="inlineStr">
         <is>
           <t>Want your community's first live event to feel like it has always existed?</t>
         </is>
       </c>
-      <c r="N20" s="7" t="inlineStr">
+      <c r="N20" s="8" t="inlineStr">
         <is>
           <t>The Vinoy, St. Petersburg, FL</t>
         </is>
       </c>
-      <c r="O20" s="7" t="inlineStr">
-        <is>
-          <t>About 400 (confirm how to publish)</t>
-        </is>
-      </c>
-      <c r="P20" s="5" t="inlineStr"/>
+      <c r="O20" s="8" t="inlineStr">
+        <is>
+          <t>451</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
       <c r="Q20" s="5" t="inlineStr"/>
       <c r="R20" s="7" t="inlineStr">
         <is>
           <t>Exists, link needed</t>
         </is>
       </c>
-      <c r="S20" s="7" t="inlineStr">
+      <c r="S20" s="8" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="T20" s="5" t="inlineStr"/>
+      <c r="T20" s="7" t="inlineStr">
+        <is>
+          <t>Photos to come in later</t>
+        </is>
+      </c>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>First edition. No stakes on the page. Do not mention the sales team. No Challenges Overcome section. Attendance was given as about 400: publish as 400, or hold for the exact count (house rule 3 allows estimates only for speakers and sponsors). Days on site? Aftermovie link? No photo folder on file.</t>
+          <t>Approved by Iconic 2026-09-30. Still needed: aftermovie link; photos to come in later. No stakes on the page. Do not mention the sales team. No Challenges Overcome section.</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
@@ -1797,12 +1805,12 @@
           <t>None (Iconic: no challenges overcome for this event).</t>
         </is>
       </c>
-      <c r="W20" s="7" t="inlineStr">
+      <c r="W20" s="8" t="inlineStr">
         <is>
           <t>Right for: a founder with a loyal community who wants a more reserved, timeless experience. Less about mixers and parties, more about the education.</t>
         </is>
       </c>
-      <c r="X20" s="7" t="inlineStr">
+      <c r="X20" s="8" t="inlineStr">
         <is>
           <t>Build a wishing tree. Give attendees a physical place to write a prayer or intention for the next event and hang it on the branches. It turns a moment of reflection into a shared installation, and it gives your community a reason to come back and see what came true.</t>
         </is>

</xml_diff>

<commit_message>
Record the first Freedom Queen Live 2025 answer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1051,7 +1051,7 @@
       <c r="W7" s="5" t="n"/>
       <c r="X7" s="5" t="n"/>
     </row>
-    <row r="8" ht="18" customHeight="1">
+    <row r="8" ht="110" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Freedom Queen Live 2025</t>
@@ -1077,8 +1077,17 @@
           <t>Interviewing</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr"/>
-      <c r="G8" s="5" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>For year two, Bridget James Ling wanted to move away from the idea of a business conference and lean into her theatrical roots. She wanted a show: Broadway style, with performers, rehearsed dance numbers and a room that felt less like a conference and more like a theatrical performance.</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>1. Built the program around rehearsed musical sets and dance numbers, with performers woven through the event.
+2. Turned the butler service into part of the performance, staged at the front of the stage.</t>
+        </is>
+      </c>
       <c r="H8" s="5" t="inlineStr"/>
       <c r="I8" s="5" t="inlineStr"/>
       <c r="J8" s="5" t="inlineStr"/>
@@ -1092,7 +1101,11 @@
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr"/>
       <c r="T8" s="5" t="inlineStr"/>
-      <c r="U8" s="5" t="inlineStr"/>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>"It was still a bit annoying": unclear, ask. Venue? Round tables lead: 40 sold, edition unknown, revenue anyway.</t>
+        </is>
+      </c>
       <c r="V8" s="5" t="n"/>
       <c r="W8" s="5" t="n"/>
       <c r="X8" s="5" t="n"/>

</xml_diff>

<commit_message>
Record the Freedom Queen Live 2025 rehearsal answer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1051,7 +1051,7 @@
       <c r="W7" s="5" t="n"/>
       <c r="X7" s="5" t="n"/>
     </row>
-    <row r="8" ht="110" customHeight="1">
+    <row r="8" ht="200" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Freedom Queen Live 2025</t>
@@ -1079,13 +1079,16 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>For year two, Bridget James Ling wanted to move away from the idea of a business conference and lean into her theatrical roots. She wanted a show: Broadway style, with performers, rehearsed dance numbers and a room that felt less like a conference and more like a theatrical performance.</t>
+          <t>For year two, Bridget James Ling wanted to move away from the idea of a business conference and lean into her theatrical roots. She wanted a show: Broadway style, with performers, rehearsed dance numbers and a room that felt less like a conference and more like a theatrical performance.
+A show needs a cast, rehearsals and split second timing, and all of it had to stay a surprise for the attendees.</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>1. Built the program around rehearsed musical sets and dance numbers, with performers woven through the event.
-2. Turned the butler service into part of the performance, staged at the front of the stage.</t>
+          <t>1. Returned to the Vinoy in St. Petersburg, the home Bridget's community already knew, and restaged it as a theater.
+2. Sourced the dance performers and built the program around rehearsed musical sets and dance numbers.
+3. Opened with a flash mob, then ran rehearsed dance performances through the day, every cue timed and synced with the AV and stage elements.
+4. Turned the butler service into part of the performance, staged at the front of the stage.</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr"/>
@@ -1094,7 +1097,11 @@
       <c r="K8" s="5" t="inlineStr"/>
       <c r="L8" s="5" t="inlineStr"/>
       <c r="M8" s="5" t="inlineStr"/>
-      <c r="N8" s="5" t="inlineStr"/>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>The Vinoy, St. Petersburg, FL</t>
+        </is>
+      </c>
       <c r="O8" s="5" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr"/>
       <c r="Q8" s="5" t="inlineStr"/>
@@ -1103,10 +1110,14 @@
       <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>"It was still a bit annoying": unclear, ask. Venue? Round tables lead: 40 sold, edition unknown, revenue anyway.</t>
-        </is>
-      </c>
-      <c r="V8" s="5" t="n"/>
+          <t>Round tables lead: 40 sold, edition unknown, revenue anyway.</t>
+        </is>
+      </c>
+      <c r="V8" s="7" t="inlineStr">
+        <is>
+          <t>Fitting dance rehearsals around speaker rehearsals was the hard part. Both had to happen in the same rooms on the same days, and the performances had to stay a secret from the attendees until the flash mob opened the event. The schedule held, every cue landed with the AV and stage, and the surprises arrived intact.</t>
+        </is>
+      </c>
       <c r="W8" s="5" t="n"/>
       <c r="X8" s="5" t="n"/>
     </row>

</xml_diff>

<commit_message>
Draft the rest of the Freedom Queen Live 2025 row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1091,26 +1091,60 @@
 4. Turned the butler service into part of the performance, staged at the front of the stage.</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="5" t="inlineStr"/>
-      <c r="K8" s="5" t="inlineStr"/>
-      <c r="L8" s="5" t="inlineStr"/>
-      <c r="M8" s="5" t="inlineStr"/>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Attendees loved it. The opening was a wild, show stopping moment that woke the room up and told everyone this was not another business conference.
+The show also made the event's media. The content that came out of it set the expectation that Freedom Queen Live is meant to be different from every other event, and attendance grew to about 500 in its second year.</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>500 | Attendees, up from 451 in year one
+1 | Flash mob to open the show</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>Show concept and program design, sourcing dance performers, rehearsal scheduling around speaker rehearsals, cueing performances with AV and stage, butler service staging, venue, production and on site execution.</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>For year two of Freedom Queen Live, Bridget James Ling wanted a show, not a business conference: Broadway style, with performers and rehearsed dance numbers. We sourced the dancers, fitted their rehearsals around the speakers', and cued every performance to the AV and stage while keeping it all a surprise. A flash mob opened the event, dance numbers ran through the day, and even the butler service became part of the performance. Attendance grew to about 500, and the media from the show set the event apart.</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>How Freedom Queen Live Turned a Business Event Into a Broadway Style Show in Year Two</t>
+        </is>
+      </c>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
+          <t>Want your next event to feel like opening night?</t>
+        </is>
+      </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
           <t>The Vinoy, St. Petersburg, FL</t>
         </is>
       </c>
-      <c r="O8" s="5" t="inlineStr"/>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
+          <t>About 500 (exact to confirm)</t>
+        </is>
+      </c>
       <c r="P8" s="5" t="inlineStr"/>
       <c r="Q8" s="5" t="inlineStr"/>
-      <c r="R8" s="5" t="inlineStr"/>
+      <c r="R8" s="7" t="inlineStr">
+        <is>
+          <t>Exists, link needed</t>
+        </is>
+      </c>
       <c r="S8" s="5" t="inlineStr"/>
       <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>Round tables lead: 40 sold, edition unknown, revenue anyway.</t>
+          <t>Attendance given as about 500: exact count for the page? Days on site? Aftermovie link? No photo folder. Round tables lead: 40 sold, edition unknown, revenue anyway.</t>
         </is>
       </c>
       <c r="V8" s="7" t="inlineStr">
@@ -1118,8 +1152,16 @@
           <t>Fitting dance rehearsals around speaker rehearsals was the hard part. Both had to happen in the same rooms on the same days, and the performances had to stay a secret from the attendees until the flash mob opened the event. The schedule held, every cue landed with the AV and stage, and the surprises arrived intact.</t>
         </is>
       </c>
-      <c r="W8" s="5" t="n"/>
-      <c r="X8" s="5" t="n"/>
+      <c r="W8" s="7" t="inlineStr">
+        <is>
+          <t>None (Iconic: no right for section for this event).</t>
+        </is>
+      </c>
+      <c r="X8" s="7" t="inlineStr">
+        <is>
+          <t>Open with a surprise. A flash mob or rehearsed performance in the first minutes tells attendees this is not another conference, and it hands your social team the clip that sells the next edition.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="330" customHeight="1">
       <c r="A9" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Approve the Freedom Queen Live 2025 row and sharpen the headline rule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1074,16 +1074,16 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
+          <t>Ready to build</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>For year two, Bridget James Ling wanted to move away from the idea of a business conference and lean into her theatrical roots. She wanted a show: Broadway style, with performers, rehearsed dance numbers and a room that felt less like a conference and more like a theatrical performance.
 A show needs a cast, rehearsals and split second timing, and all of it had to stay a surprise for the attendees.</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>1. Returned to the Vinoy in St. Petersburg, the venue Bridget's community already knew from year one.
 2. Sourced the dance performers and built the program around rehearsed musical sets and dance numbers.
@@ -1091,73 +1091,85 @@
 4. Turned the butler service into part of the performance, staged at the front of the stage.</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>Attendees loved it. The opening was a wild, show stopping moment that woke the room up and told everyone this was not another business conference.
-The show also made the event's media. The content that came out of it set the expectation that Freedom Queen Live is meant to be different from every other event, and attendance grew to about 500 in its second year.</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr">
-        <is>
-          <t>500 | Attendees, up from 451 in year one
+The show also made the event's media. The content that came out of it set the expectation that Freedom Queen Live is meant to be different from every other event, and attendance grew to 530 in its second year.</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>530 | Attendees, up from 451 in year one
 1 | Flash mob to open the show</t>
         </is>
       </c>
-      <c r="J8" s="7" t="inlineStr">
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>Show concept and program design, sourcing dance performers, rehearsal scheduling around speaker rehearsals, cueing performances with AV and stage, butler service staging, venue, production and on site execution.</t>
         </is>
       </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>For year two of Freedom Queen Live, Bridget James Ling wanted a show, not a business conference: Broadway style, with performers and rehearsed dance numbers. We sourced the dancers, fitted their rehearsals around the speakers', and cued every performance to the AV and stage while keeping it all a surprise. A flash mob opened the event, dance numbers ran through the day, and even the butler service became part of the performance. Attendance grew to about 500, and the media from the show set the event apart.</t>
-        </is>
-      </c>
-      <c r="L8" s="7" t="inlineStr">
-        <is>
-          <t>How Freedom Queen Live Turned a Business Event Into a Broadway Style Show in Year Two</t>
-        </is>
-      </c>
-      <c r="M8" s="7" t="inlineStr">
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>For year two of Freedom Queen Live, Bridget James Ling wanted a show, not a business conference: Broadway style, with performers and rehearsed dance numbers. We sourced the dancers, fitted their rehearsals around the speakers', and cued every performance to the AV and stage while keeping it all a surprise. A flash mob opened the event, dance numbers ran through the day, and even the butler service became part of the performance. Attendance grew to 530 over three and a half days, and the media from the show set the event apart.</t>
+        </is>
+      </c>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>How Freedom Queen Live Rewrote the Business Event Format and Drew 530 Attendees to a Broadway Style Show</t>
+        </is>
+      </c>
+      <c r="M8" s="8" t="inlineStr">
         <is>
           <t>Want your next event to feel like opening night?</t>
         </is>
       </c>
-      <c r="N8" s="7" t="inlineStr">
+      <c r="N8" s="8" t="inlineStr">
         <is>
           <t>The Vinoy, St. Petersburg, FL</t>
         </is>
       </c>
-      <c r="O8" s="7" t="inlineStr">
-        <is>
-          <t>About 500 (exact to confirm)</t>
-        </is>
-      </c>
-      <c r="P8" s="5" t="inlineStr"/>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t>530</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
       <c r="Q8" s="5" t="inlineStr"/>
       <c r="R8" s="7" t="inlineStr">
         <is>
-          <t>Exists, link needed</t>
-        </is>
-      </c>
-      <c r="S8" s="5" t="inlineStr"/>
-      <c r="T8" s="5" t="inlineStr"/>
+          <t>Link to come later</t>
+        </is>
+      </c>
+      <c r="S8" s="7" t="inlineStr">
+        <is>
+          <t>Link to come later</t>
+        </is>
+      </c>
+      <c r="T8" s="7" t="inlineStr">
+        <is>
+          <t>Photos to come later</t>
+        </is>
+      </c>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>Attendance given as about 500: exact count for the page? Days on site? Aftermovie link? No photo folder. Round tables lead: 40 sold, edition unknown, revenue anyway.</t>
-        </is>
-      </c>
-      <c r="V8" s="7" t="inlineStr">
+          <t>Approved by Iconic 2026-10-01 with a new headline. 530 attendees supplied by Iconic. Aftermovie and testimonial links to come later; photos to come later.</t>
+        </is>
+      </c>
+      <c r="V8" s="8" t="inlineStr">
         <is>
           <t>Fitting dance rehearsals around speaker rehearsals was the hard part. Both had to happen in the same rooms on the same days, and the performances had to stay a secret from the attendees until the flash mob opened the event. The schedule held, every cue landed with the AV and stage, and the surprises arrived intact.</t>
         </is>
       </c>
-      <c r="W8" s="7" t="inlineStr">
+      <c r="W8" s="8" t="inlineStr">
         <is>
           <t>None (Iconic: no right for section for this event).</t>
         </is>
       </c>
-      <c r="X8" s="7" t="inlineStr">
+      <c r="X8" s="8" t="inlineStr">
         <is>
           <t>Open with a surprise. A flash mob or rehearsed performance in the first minutes tells attendees this is not another conference, and it hands your social team the clip that sells the next edition.</t>
         </is>
@@ -1848,12 +1860,12 @@
       <c r="Q20" s="5" t="inlineStr"/>
       <c r="R20" s="7" t="inlineStr">
         <is>
-          <t>Exists, link needed</t>
+          <t>Link to come later</t>
         </is>
       </c>
       <c r="S20" s="8" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Link to come later</t>
         </is>
       </c>
       <c r="T20" s="7" t="inlineStr">
@@ -1863,7 +1875,7 @@
       </c>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>Approved by Iconic 2026-09-30. Still needed: aftermovie link; photos to come in later. No stakes on the page. Do not mention the sales team. No Challenges Overcome section.</t>
+          <t>Approved by Iconic 2026-09-30. Aftermovie and testimonial links to come later; photos to come in later. No stakes on the page. Do not mention the sales team. No Challenges Overcome section.</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
@@ -2231,7 +2243,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Interviewing</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Start PMUW 2023 from the old site's own case study
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -2220,7 +2220,7 @@
       <c r="W27" s="5" t="n"/>
       <c r="X27" s="5" t="n"/>
     </row>
-    <row r="28" ht="18" customHeight="1">
+    <row r="28" ht="260" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
           <t>PMUW 2023</t>
@@ -2236,9 +2236,9 @@
           <t>April 2023</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Danny Tran</t>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Danny Tran, High Stroke Media</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2246,22 +2246,65 @@
           <t>Interviewing</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr"/>
-      <c r="G28" s="5" t="inlineStr"/>
-      <c r="H28" s="5" t="inlineStr"/>
-      <c r="I28" s="5" t="inlineStr"/>
-      <c r="J28" s="5" t="inlineStr"/>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>The permanent makeup industry had been underserved for too long: its largest live event drew only about 300 people. Danny Tran wanted to blow that out of the water, and not with another boring PMU conference. He wanted workshops and business combined, and he wanted it to be the largest PMU event in the country, which meant passing 800 people on site.
+Danny had never run an event this size, had no audience behind him, and gave us five months to build it.</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>1. Teased the event with media for months before there was any way to buy a ticket. When sales opened about 60 days out, they went from 0 to about 400 in 45 days, and sponsors started coming to us.
+2. Secured the Hard Rock Hotel on one of the most popular weekends of the year, through our network.
+3. Ran two stages like a music festival: one for business, one for practice, so attendees could learn and do on site. Added a sponsor hall and a VIP area.
+4. Made installations the highlight, built for selfies and content. When South Florida installation companies could not produce what we needed, we built them ourselves.</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>About 600 attendees showed up on day one. By the end, as word spread, almost 900 were on site, making it the largest PMU event in North America. Five months earlier there was no event at all.
+Attendees loved the two stage format and left wanting to come back next year.</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>850 | Attendees on site
+#1 | Largest PMU event in North America
+$148K | Saved off contracts</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>Coordination, production, content, installation buildout, attendee management, negotiations, sponsorship management, speaker management, post production content.</t>
+        </is>
+      </c>
       <c r="K28" s="5" t="inlineStr"/>
       <c r="L28" s="5" t="inlineStr"/>
       <c r="M28" s="5" t="inlineStr"/>
-      <c r="N28" s="5" t="inlineStr"/>
-      <c r="O28" s="5" t="inlineStr"/>
+      <c r="N28" s="7" t="inlineStr">
+        <is>
+          <t>Hard Rock Hotel, FL (which one?)</t>
+        </is>
+      </c>
+      <c r="O28" s="7" t="inlineStr">
+        <is>
+          <t>850 or almost 900?</t>
+        </is>
+      </c>
       <c r="P28" s="5" t="inlineStr"/>
-      <c r="Q28" s="5" t="inlineStr"/>
+      <c r="Q28" s="7" t="inlineStr">
+        <is>
+          <t>$148,000</t>
+        </is>
+      </c>
       <c r="R28" s="5" t="inlineStr"/>
       <c r="S28" s="5" t="inlineStr"/>
       <c r="T28" s="5" t="inlineStr"/>
-      <c r="U28" s="5" t="inlineStr"/>
+      <c r="U28" s="5" t="inlineStr">
+        <is>
+          <t>Drafted from the old site's own copy (row 5). Left out: the event cost (rule 2) and the failed festival comparison (third party brand). Attendance: the old page says 850 and almost 900. Which Hard Rock? Danny's title? Q4 Challenges Overcome, Q5 Right for, Steal This: from the interview.</t>
+        </is>
+      </c>
       <c r="V28" s="5" t="n"/>
       <c r="W28" s="5" t="n"/>
       <c r="X28" s="5" t="n"/>

</xml_diff>

<commit_message>
Mark the three new case studies built and set the PMUW order
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1074,7 +1074,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Ready to build</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Ready to build</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Ready to build</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
@@ -2302,7 +2302,7 @@
       <c r="T28" s="5" t="inlineStr"/>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>Drafted from the old site's own copy (row 5). Left out: the event cost (rule 2) and the failed festival comparison (third party brand). Attendance: the old page says 850 and almost 900. Which Hard Rock? Danny's title? Q4 Challenges Overcome, Q5 Right for, Steal This: from the interview.</t>
+          <t>Drafted from the old site's own copy (row 5). Left out: the event cost (rule 2) and the failed festival comparison (third party brand). Attendance: the old page says 850 and almost 900. Which Hard Rock? Danny's title? Q4 Challenges Overcome, Q5 Right for, Steal This: from the interview. Order: PMUW 2023, then 2024, then 2025 (Iconic).</t>
         </is>
       </c>
       <c r="V28" s="5" t="n"/>

</xml_diff>

<commit_message>
Record the PMUW 2023 facts and challenge, and draft the rest of its row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -2238,7 +2238,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Danny Tran, High Stroke Media</t>
+          <t>Danny Tran, CEO, HighStoke Media</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2255,20 +2255,20 @@
       <c r="G28" s="7" t="inlineStr">
         <is>
           <t>1. Teased the event with media for months before there was any way to buy a ticket. When sales opened about 60 days out, they went from 0 to about 400 in 45 days, and sponsors started coming to us.
-2. Secured the Hard Rock Hotel on one of the most popular weekends of the year, through our network.
+2. Secured the Seminole Hard Rock, the Guitar Hotel, on one of the most popular weekends of the year, through our network.
 3. Ran two stages like a music festival: one for business, one for practice, so attendees could learn and do on site. Added a sponsor hall and a VIP area.
 4. Made installations the highlight, built for selfies and content. When South Florida installation companies could not produce what we needed, we built them ourselves.</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>About 600 attendees showed up on day one. By the end, as word spread, almost 900 were on site, making it the largest PMU event in North America. Five months earlier there was no event at all.
+          <t>About 600 attendees showed up on day one. By the end, as word spread, 900 were on site, making it the largest PMU event in North America. Five months earlier there was no event at all.
 Attendees loved the two stage format and left wanting to come back next year.</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>850 | Attendees on site
+          <t>900 | Attendees on site
 #1 | Largest PMU event in North America
 $148K | Saved off contracts</t>
         </is>
@@ -2278,17 +2278,29 @@
           <t>Coordination, production, content, installation buildout, attendee management, negotiations, sponsorship management, speaker management, post production content.</t>
         </is>
       </c>
-      <c r="K28" s="5" t="inlineStr"/>
-      <c r="L28" s="5" t="inlineStr"/>
-      <c r="M28" s="5" t="inlineStr"/>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t>The permanent makeup industry's largest live event drew about 300 people. Danny Tran, CEO of HighStoke Media, wanted to build the biggest one in North America in five months, with no audience behind him and an industry that doubted him. We teased the event with media for months before tickets went on sale, secured the Seminole Hard Rock, ran two stages like a music festival, one for business and one for practice, and built the installations ourselves. Sales went from 0 to about 400 in 45 days, and 900 attendees were on site by the end.</t>
+        </is>
+      </c>
+      <c r="L28" s="7" t="inlineStr">
+        <is>
+          <t>How Danny Tran Built the Largest Permanent Makeup Event in North America in Five Months</t>
+        </is>
+      </c>
+      <c r="M28" s="7" t="inlineStr">
+        <is>
+          <t>Want to build the biggest event in your industry?</t>
+        </is>
+      </c>
       <c r="N28" s="7" t="inlineStr">
         <is>
-          <t>Hard Rock Hotel, FL (which one?)</t>
+          <t>Seminole Hard Rock (the Guitar Hotel), Hollywood, FL</t>
         </is>
       </c>
       <c r="O28" s="7" t="inlineStr">
         <is>
-          <t>850 or almost 900?</t>
+          <t>900</t>
         </is>
       </c>
       <c r="P28" s="5" t="inlineStr"/>
@@ -2302,10 +2314,15 @@
       <c r="T28" s="5" t="inlineStr"/>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>Drafted from the old site's own copy (row 5). Left out: the event cost (rule 2) and the failed festival comparison (third party brand). Attendance: the old page says 850 and almost 900. Which Hard Rock? Danny's title? Q4 Challenges Overcome, Q5 Right for, Steal This: from the interview. Order: PMUW 2023, then 2024, then 2025 (Iconic).</t>
-        </is>
-      </c>
-      <c r="V28" s="5" t="n"/>
+          <t>Drafted from the old site's own copy (row 5) plus the interview. Left out: the event cost (rule 2) and the failed festival comparison. Confirm: Hollywood, FL; HighStoke capitalization. Still to answer: Right for, Steal This, days on site, aftermovie. Order: PMUW 2023, then 2024, then 2025.</t>
+        </is>
+      </c>
+      <c r="V28" s="7" t="inlineStr">
+        <is>
+          <t>Nobody believed in this event. Danny ran a marketing agency in an industry that is mostly women, and many doubted a man could pull it off. No permanent makeup event had ever been attempted at this size, so he was trying to build the biggest event the industry had seen while beating a wave of doubt from people who did not know him.
+The answer was to let the event prove itself before asking anyone to buy. Months of teaser media built curiosity first, so when tickets opened 60 days out, sales went from 0 to about 400 in 45 days and sponsors started coming to us. By the last day, 900 people were on site.</t>
+        </is>
+      </c>
       <c r="W28" s="5" t="n"/>
       <c r="X28" s="5" t="n"/>
     </row>

</xml_diff>

<commit_message>
Correct PMUW 2023 from Iconic's research and add its niche Steal This
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -2220,7 +2220,7 @@
       <c r="W27" s="5" t="n"/>
       <c r="X27" s="5" t="n"/>
     </row>
-    <row r="28" ht="260" customHeight="1">
+    <row r="28" ht="300" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
           <t>PMUW 2023</t>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Danny Tran, CEO, HighStoke Media</t>
+          <t>Danny Tran, Founder and CEO, Highstoke Media</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2248,27 +2248,27 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>The permanent makeup industry had been underserved for too long: its largest live event drew only about 300 people. Danny Tran wanted to blow that out of the water, and not with another boring PMU conference. He wanted workshops and business combined, and he wanted it to be the largest PMU event in the country, which meant passing 800 people on site.
-Danny had never run an event this size, had no audience behind him, and gave us five months to build it.</t>
+          <t>The permanent makeup industry had been underserved for too long: its largest live event drew only about 300 people. Danny Tran wanted to blow that out of the water, and not with another boring PMU conference. He wanted workshops and business combined, and he wanted it to be the largest PMU event in the country.
+This was the first PMU World. The brand was only seven months old, with no attendee list and no past footage to market with, and Danny had never run an event this size. We had five months to build it.</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>1. Teased the event with media for months before there was any way to buy a ticket. When sales opened about 60 days out, they went from 0 to about 400 in 45 days, and sponsors started coming to us.
-2. Secured the Seminole Hard Rock, the Guitar Hotel, on one of the most popular weekends of the year, through our network.
-3. Ran two stages like a music festival: one for business, one for practice, so attendees could learn and do on site. Added a sponsor hall and a VIP area.
-4. Made installations the highlight, built for selfies and content. When South Florida installation companies could not produce what we needed, we built them ourselves.</t>
+          <t>1. Ran teaser videos while the venue was still being secured, building curiosity before there was anything to buy. When they landed, ticket sales jumped from 100 to over 300 overnight.
+2. Secured the Seminole Hard Rock Hotel &amp; Casino Hollywood, the Guitar Hotel, on one of the most popular weekends of the year.
+3. Ran two stages at once like a music festival: one for business, one for practice, so attendees could learn and do on site. Added a sponsor hall and a VIP area.
+4. Built more than 16 interactive installations ourselves, made for selfies and content, after South Florida installation companies could not produce what we needed.</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>About 600 attendees showed up on day one. By the end, as word spread, 900 were on site, making it the largest PMU event in North America. Five months earlier there was no event at all.
+          <t>More than 800 attendees were on site, against a projection of 600, making it the largest PMU event in North America. Seven months earlier the brand did not exist.
 Attendees loved the two stage format and left wanting to come back next year.</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>900 | Attendees on site
+          <t>800+ | Attendees on site, against 600 projected
 #1 | Largest PMU event in North America
 $148K | Saved off contracts</t>
         </is>
@@ -2280,7 +2280,7 @@
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>The permanent makeup industry's largest live event drew about 300 people. Danny Tran, CEO of HighStoke Media, wanted to build the biggest one in North America in five months, with no audience behind him and an industry that doubted him. We teased the event with media for months before tickets went on sale, secured the Seminole Hard Rock, ran two stages like a music festival, one for business and one for practice, and built the installations ourselves. Sales went from 0 to about 400 in 45 days, and 900 attendees were on site by the end.</t>
+          <t>The permanent makeup industry's largest live event drew about 300 people. Danny Tran, founder and CEO of Highstoke Media, wanted to build the biggest one in North America with a seven month old brand, no attendee list and an industry that doubted him. We ran teaser videos while the venue was still being secured, took the Seminole Hard Rock in Hollywood, Florida, ran two stages like a music festival and built more than 16 interactive installations ourselves. More than 800 attendees came, against a projection of 600.</t>
         </is>
       </c>
       <c r="L28" s="7" t="inlineStr">
@@ -2295,12 +2295,12 @@
       </c>
       <c r="N28" s="7" t="inlineStr">
         <is>
-          <t>Seminole Hard Rock (the Guitar Hotel), Hollywood, FL</t>
+          <t>Seminole Hard Rock Hotel &amp; Casino Hollywood, Hollywood, FL</t>
         </is>
       </c>
       <c r="O28" s="7" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>800+</t>
         </is>
       </c>
       <c r="P28" s="5" t="inlineStr"/>
@@ -2314,17 +2314,26 @@
       <c r="T28" s="5" t="inlineStr"/>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>Drafted from the old site's own copy (row 5) plus the interview. Left out: the event cost (rule 2) and the failed festival comparison. Confirm: Hollywood, FL; HighStoke capitalization. Still to answer: Right for, Steal This, days on site, aftermovie. Order: PMUW 2023, then 2024, then 2025.</t>
+          <t>Built from the old site's copy, Iconic's research (Juan's Slack draft, Apr 26 2023) and the interview. Left out: the event cost (rule 2), the failed festival comparison, and claims the research could not support (60 days out, 0 to 400 in 45 days, 850, almost 900). Still to answer: days on site, aftermovie. Order: PMUW 2023, then 2024, then 2025.</t>
         </is>
       </c>
       <c r="V28" s="7" t="inlineStr">
         <is>
-          <t>Nobody believed in this event. Danny ran a marketing agency in an industry that is mostly women, and many doubted a man could pull it off. No permanent makeup event had ever been attempted at this size, so he was trying to build the biggest event the industry had seen while beating a wave of doubt from people who did not know him.
-The answer was to let the event prove itself before asking anyone to buy. Months of teaser media built curiosity first, so when tickets opened 60 days out, sales went from 0 to about 400 in 45 days and sponsors started coming to us. By the last day, 900 people were on site.</t>
-        </is>
-      </c>
-      <c r="W28" s="5" t="n"/>
-      <c r="X28" s="5" t="n"/>
+          <t>Nobody believed in this event. Danny ran a marketing agency in an industry that is mostly women, and many doubted a man could pull it off. No permanent makeup event had ever been attempted at this size, and the brand was only seven months old, with no attendee list and no past footage to show.
+So the event had to prove itself before anyone could see it. Teaser videos built the story while the venue was still being secured, and when they landed, ticket sales jumped from 100 to over 300 overnight. By the event, more than 800 people were on site, against a projection of 600.</t>
+        </is>
+      </c>
+      <c r="W28" s="7" t="inlineStr">
+        <is>
+          <t>Female beauty entrepreneurs and salon owners in an underserved niche, and the founders who serve a niche like that and want to give it an event of its own.</t>
+        </is>
+      </c>
+      <c r="X28" s="7" t="inlineStr">
+        <is>
+          <t>The riches are in the niches. PMU World could have been a beauty world or a beauty con, and it would have been too wide. Focusing on permanent makeup, a corner of the beauty industry many people do not even know exists, made a room built for one group of people, where they felt at home and every session and piece of content was made for them.
+Sell the story before the venue is signed. Teaser videos that ran while the Hard Rock was still being secured took ticket sales from 100 to over 300 overnight.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Settle the PMUW 2023 headline and start PMUW 2024
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1963,7 +1963,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Interviewing</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr"/>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="L28" s="7" t="inlineStr">
         <is>
-          <t>How Danny Tran Built the Largest Permanent Makeup Event in North America in Five Months</t>
+          <t>How Danny Tran Defied the Odds and Built the Largest Permanent Makeup Event in North America on His First Try</t>
         </is>
       </c>
       <c r="M28" s="7" t="inlineStr">
@@ -2303,13 +2303,21 @@
           <t>800+</t>
         </is>
       </c>
-      <c r="P28" s="5" t="inlineStr"/>
+      <c r="P28" s="7" t="inlineStr">
+        <is>
+          <t>4 (April 3 to 6), confirm</t>
+        </is>
+      </c>
       <c r="Q28" s="7" t="inlineStr">
         <is>
           <t>$148,000</t>
         </is>
       </c>
-      <c r="R28" s="5" t="inlineStr"/>
+      <c r="R28" s="7" t="inlineStr">
+        <is>
+          <t>On Iconic's YouTube, link to come later</t>
+        </is>
+      </c>
       <c r="S28" s="5" t="inlineStr"/>
       <c r="T28" s="5" t="inlineStr"/>
       <c r="U28" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Record the PMUW 2024 research leads and draft its Steal This
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1940,7 +1940,7 @@
       <c r="W21" s="5" t="n"/>
       <c r="X21" s="5" t="n"/>
     </row>
-    <row r="22" ht="18" customHeight="1">
+    <row r="22" ht="150" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>PMUW 2024</t>
@@ -1956,9 +1956,9 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Danny Tran</t>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Danny Tran, Founder and CEO, Highstoke Media</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1974,17 +1974,30 @@
       <c r="K22" s="5" t="inlineStr"/>
       <c r="L22" s="5" t="inlineStr"/>
       <c r="M22" s="5" t="inlineStr"/>
-      <c r="N22" s="5" t="inlineStr"/>
+      <c r="N22" s="7" t="inlineStr">
+        <is>
+          <t>A Hard Rock in Florida (Hollywood unconfirmed)</t>
+        </is>
+      </c>
       <c r="O22" s="5" t="inlineStr"/>
       <c r="P22" s="5" t="inlineStr"/>
       <c r="Q22" s="5" t="inlineStr"/>
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr"/>
       <c r="T22" s="5" t="inlineStr"/>
-      <c r="U22" s="5" t="inlineStr"/>
+      <c r="U22" s="5" t="inlineStr">
+        <is>
+          <t>Leads from Iconic's research: final attendance unknown (about 560 tickets in early July against a 900 target); venue Hollywood unconfirmed; month unknown. Challenges known (ASL interpreter request, Florida registration and bloodborne pathogen rules for live tattoo workshops, a tropical storm watched a week out, badge printing and second stage content problems) but not yet how each was handled.</t>
+        </is>
+      </c>
       <c r="V22" s="5" t="n"/>
       <c r="W22" s="5" t="n"/>
-      <c r="X22" s="5" t="n"/>
+      <c r="X22" s="7" t="inlineStr">
+        <is>
+          <t>Sell year two with year one. A soft launch in December used a teaser cut from the 2023 footage, so the event sold on proof instead of promises.
+Sell next year in the room. Pre-sale tickets for 2025 went on sale at the 2024 event itself, while attendees were at their most convinced.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Record the PMUW 2024 interview and draft its row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1940,7 +1940,7 @@
       <c r="W21" s="5" t="n"/>
       <c r="X21" s="5" t="n"/>
     </row>
-    <row r="22" ht="150" customHeight="1">
+    <row r="22" ht="300" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>PMUW 2024</t>
@@ -1966,20 +1966,61 @@
           <t>Interviewing</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr"/>
-      <c r="G22" s="5" t="inlineStr"/>
-      <c r="H22" s="5" t="inlineStr"/>
-      <c r="I22" s="5" t="inlineStr"/>
-      <c r="J22" s="5" t="inlineStr"/>
-      <c r="K22" s="5" t="inlineStr"/>
-      <c r="L22" s="5" t="inlineStr"/>
-      <c r="M22" s="5" t="inlineStr"/>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Year one proved PMU World could fill a room. Year two had to make that room work harder. Danny Tran wanted an elegant sponsor hall and an event where sponsors got real value, without losing what attendees loved.
+The rules changed too. New Florida requirements meant an ASL interpreter request and registration rules for the live tattoo workshops, on top of a bigger crowd.</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>1. Halved the size of the room and went from two stages to one, with one major sponsor hall beside it.
+2. Sold smaller sponsorship packages, so more brands could buy in, and used that room to open a new expo floor.
+3. Covered the ballroom floors end to end in visqueen plastic, turning them into temporary, near medical grade stations for the live tattoo workshops.
+4. Started sourcing backup local vendors a week out, the moment a tropical storm appeared on the forecast.</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>PMU World grew to 1,237 attendees in its second year, up from more than 800 in 2023. Attendees enjoyed the new expo floor more than the old format, sponsors got better value from a single, focused hall, and the event felt more dynamic for everyone in it.</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>1,237 | Attendees, up from 800+ in year one
+1 | Stage, focused, with a full expo floor beside it</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>Room and floor plan redesign, sponsorship packaging and the sponsor hall, the expo floor, compliance for the live tattoo workshops, accessibility accommodation, contingency vendor sourcing, badge production, production and on site execution.</t>
+        </is>
+      </c>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>For year two of PMU World, Danny Tran wanted an elegant sponsor hall and a room where sponsors got real value. We halved the room, cut to one stage, opened a sponsor hall and a new expo floor sold in smaller packages, and turned the ballrooms into compliant stations for live tattoo workshops. When a tropical storm delayed shipments, backup vendors lined up a week earlier kept everything on schedule, down to badges reprinted at a local print shop. Attendance grew to 1,237.</t>
+        </is>
+      </c>
+      <c r="L22" s="7" t="inlineStr">
+        <is>
+          <t>How PMU World Grew to 1,237 Attendees in Year Two by Making the Room Smaller</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>Want year two to beat year one?</t>
+        </is>
+      </c>
       <c r="N22" s="7" t="inlineStr">
         <is>
-          <t>A Hard Rock in Florida (Hollywood unconfirmed)</t>
-        </is>
-      </c>
-      <c r="O22" s="5" t="inlineStr"/>
+          <t>Seminole Hard Rock Hotel &amp; Casino Hollywood, Hollywood, FL</t>
+        </is>
+      </c>
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>1,237</t>
+        </is>
+      </c>
       <c r="P22" s="5" t="inlineStr"/>
       <c r="Q22" s="5" t="inlineStr"/>
       <c r="R22" s="5" t="inlineStr"/>
@@ -1987,10 +2028,15 @@
       <c r="T22" s="5" t="inlineStr"/>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>Leads from Iconic's research: final attendance unknown (about 560 tickets in early July against a 900 target); venue Hollywood unconfirmed; month unknown. Challenges known (ASL interpreter request, Florida registration and bloodborne pathogen rules for live tattoo workshops, a tropical storm watched a week out, badge printing and second stage content problems) but not yet how each was handled.</t>
-        </is>
-      </c>
-      <c r="V22" s="5" t="n"/>
+          <t>Sponsorship dollars ($5,000 to $6,000 packages; hundreds of thousands added) left off: house rule 1, unless Iconic makes an exception. Month and dates unknown. Days on site? Aftermovie? Right for? Steal This drafted from Iconic's research.</t>
+        </is>
+      </c>
+      <c r="V22" s="7" t="inlineStr">
+        <is>
+          <t>An ASL interpreter request would have broken the budget. Instead we turned on a real time caption service on the event livestream, which the attendee could follow from the crowd. It met the accommodation and cost Danny nothing.
+A tropical storm came out of nowhere. Because backup vendors were already lined up a week out, delayed shipments did not stop the event. When the badges did not arrive, a local vinyl print shop printed them on a different cardstock, on time and still with the luxury feel.</t>
+        </is>
+      </c>
       <c r="W22" s="5" t="n"/>
       <c r="X22" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Approve PMUW 2023 and 2024 rows and start PMUW 2025
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1427,7 +1427,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Interviewing</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr"/>
@@ -1953,92 +1953,108 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
+          <t>August 2024</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>Danny Tran, Founder and CEO, Highstoke Media</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
+          <t>Ready to build</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>Year one proved PMU World could fill a room. Year two had to make that room work harder. Danny Tran wanted an elegant sponsor hall and an event where sponsors got real value, without losing what attendees loved.
 The rules changed too. New Florida requirements meant an ASL interpreter request and registration rules for the live tattoo workshops, on top of a bigger crowd.</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr">
         <is>
           <t>1. Halved the size of the room and went from two stages to one, with one major sponsor hall beside it.
 2. Sold smaller sponsorship packages, so more brands could buy in, and used that room to open a new expo floor.
 3. Covered the ballroom floors end to end in visqueen plastic, turning them into temporary, near medical grade stations for the live tattoo workshops.
-4. Started sourcing backup local vendors a week out, the moment a tropical storm appeared on the forecast.</t>
-        </is>
-      </c>
-      <c r="H22" s="7" t="inlineStr">
+4. Started sourcing backup local vendors a week out, the moment a tropical storm appeared on the forecast, and made the virtual options far more deliberate for attendees the storm might keep at home.</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
         <is>
           <t>PMU World grew to 1,237 attendees in its second year, up from more than 800 in 2023. Attendees enjoyed the new expo floor more than the old format, sponsors got better value from a single, focused hall, and the event felt more dynamic for everyone in it.</t>
         </is>
       </c>
-      <c r="I22" s="7" t="inlineStr">
+      <c r="I22" s="8" t="inlineStr">
         <is>
           <t>1,237 | Attendees, up from 800+ in year one
 1 | Stage, focused, with a full expo floor beside it</t>
         </is>
       </c>
-      <c r="J22" s="7" t="inlineStr">
+      <c r="J22" s="8" t="inlineStr">
         <is>
           <t>Room and floor plan redesign, sponsorship packaging and the sponsor hall, the expo floor, compliance for the live tattoo workshops, accessibility accommodation, contingency vendor sourcing, badge production, production and on site execution.</t>
         </is>
       </c>
-      <c r="K22" s="7" t="inlineStr">
-        <is>
-          <t>For year two of PMU World, Danny Tran wanted an elegant sponsor hall and a room where sponsors got real value. We halved the room, cut to one stage, opened a sponsor hall and a new expo floor sold in smaller packages, and turned the ballrooms into compliant stations for live tattoo workshops. When a tropical storm delayed shipments, backup vendors lined up a week earlier kept everything on schedule, down to badges reprinted at a local print shop. Attendance grew to 1,237.</t>
-        </is>
-      </c>
-      <c r="L22" s="7" t="inlineStr">
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>For year two of PMU World, Danny Tran wanted an elegant sponsor hall and a room where sponsors got real value. We halved the room, cut to one stage, opened a sponsor hall and a new expo floor sold in smaller packages, and turned the ballrooms into compliant stations for live tattoo workshops. When a tropical storm delayed shipments, backup vendors lined up a week earlier kept everything on schedule, down to badges reprinted at a local print shop. Attendance grew to 1,237 over three days in August 2024.</t>
+        </is>
+      </c>
+      <c r="L22" s="8" t="inlineStr">
         <is>
           <t>How PMU World Grew to 1,237 Attendees in Year Two by Making the Room Smaller</t>
         </is>
       </c>
-      <c r="M22" s="7" t="inlineStr">
+      <c r="M22" s="8" t="inlineStr">
         <is>
           <t>Want year two to beat year one?</t>
         </is>
       </c>
-      <c r="N22" s="7" t="inlineStr">
+      <c r="N22" s="8" t="inlineStr">
         <is>
           <t>Seminole Hard Rock Hotel &amp; Casino Hollywood, Hollywood, FL</t>
         </is>
       </c>
-      <c r="O22" s="7" t="inlineStr">
+      <c r="O22" s="8" t="inlineStr">
         <is>
           <t>1,237</t>
         </is>
       </c>
-      <c r="P22" s="5" t="inlineStr"/>
+      <c r="P22" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="Q22" s="5" t="inlineStr"/>
-      <c r="R22" s="5" t="inlineStr"/>
+      <c r="R22" s="7" t="inlineStr">
+        <is>
+          <t>Link to come later</t>
+        </is>
+      </c>
       <c r="S22" s="5" t="inlineStr"/>
-      <c r="T22" s="5" t="inlineStr"/>
+      <c r="T22" s="7" t="inlineStr">
+        <is>
+          <t>Photos to come later</t>
+        </is>
+      </c>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>Sponsorship dollars ($5,000 to $6,000 packages; hundreds of thousands added) left off: house rule 1, unless Iconic makes an exception. Month and dates unknown. Days on site? Aftermovie? Right for? Steal This drafted from Iconic's research.</t>
-        </is>
-      </c>
-      <c r="V22" s="7" t="inlineStr">
+          <t>Approved by Iconic 2026-10-20. Sponsorship dollars stay off (house rule 1). Aftermovie link and photos to come later. Grid date: August 2024.</t>
+        </is>
+      </c>
+      <c r="V22" s="8" t="inlineStr">
         <is>
           <t>An ASL interpreter request would have broken the budget. Instead we turned on a real time caption service on the event livestream, which the attendee could follow from the crowd. It met the accommodation and cost Danny nothing.
-A tropical storm came out of nowhere. Because backup vendors were already lined up a week out, delayed shipments did not stop the event. When the badges did not arrive, a local vinyl print shop printed them on a different cardstock, on time and still with the luxury feel.</t>
-        </is>
-      </c>
-      <c r="W22" s="5" t="n"/>
-      <c r="X22" s="7" t="inlineStr">
+A tropical storm came out of nowhere. Because backup vendors were already lined up a week out, delayed shipments did not stop the event, and attendees held back by the storm still had a deliberate way to take part virtually. When the badges did not arrive, a local vinyl print shop printed them on a different cardstock, on time and still with the luxury feel.</t>
+        </is>
+      </c>
+      <c r="W22" s="5" t="inlineStr">
+        <is>
+          <t>Female beauty entrepreneurs and salon owners in an underserved niche, and the founders who serve a niche like that, along with any conference or expo that wants its sponsors and its attendees to both come out ahead.</t>
+        </is>
+      </c>
+      <c r="X22" s="8" t="inlineStr">
         <is>
           <t>Sell year two with year one. A soft launch in December used a teaser cut from the 2023 footage, so the event sold on proof instead of promises.
 Sell next year in the room. Pre-sale tickets for 2025 went on sale at the 2024 event itself, while attendees were at their most convinced.</t>
@@ -2295,23 +2311,23 @@
           <t>April 2023</t>
         </is>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>Danny Tran, Founder and CEO, Highstoke Media</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr">
+          <t>Ready to build</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
         <is>
           <t>The permanent makeup industry had been underserved for too long: its largest live event drew only about 300 people. Danny Tran wanted to blow that out of the water, and not with another boring PMU conference. He wanted workshops and business combined, and he wanted it to be the largest PMU event in the country.
 This was the first PMU World. The brand was only seven months old, with no attendee list and no past footage to market with, and Danny had never run an event this size. We had five months to build it.</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G28" s="8" t="inlineStr">
         <is>
           <t>1. Ran teaser videos while the venue was still being secured, building curiosity before there was anything to buy. When they landed, ticket sales jumped from 100 to over 300 overnight.
 2. Secured the Seminole Hard Rock Hotel &amp; Casino Hollywood, the Guitar Hotel, on one of the most popular weekends of the year.
@@ -2319,45 +2335,45 @@
 4. Built more than 16 interactive installations ourselves, made for selfies and content, after South Florida installation companies could not produce what we needed.</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="H28" s="8" t="inlineStr">
         <is>
           <t>More than 800 attendees were on site, against a projection of 600, making it the largest PMU event in North America. Seven months earlier the brand did not exist.
 Attendees loved the two stage format and left wanting to come back next year.</t>
         </is>
       </c>
-      <c r="I28" s="7" t="inlineStr">
+      <c r="I28" s="8" t="inlineStr">
         <is>
           <t>800+ | Attendees on site, against 600 projected
 #1 | Largest PMU event in North America
 $148K | Saved off contracts</t>
         </is>
       </c>
-      <c r="J28" s="7" t="inlineStr">
+      <c r="J28" s="8" t="inlineStr">
         <is>
           <t>Coordination, production, content, installation buildout, attendee management, negotiations, sponsorship management, speaker management, post production content.</t>
         </is>
       </c>
-      <c r="K28" s="7" t="inlineStr">
+      <c r="K28" s="8" t="inlineStr">
         <is>
           <t>The permanent makeup industry's largest live event drew about 300 people. Danny Tran, founder and CEO of Highstoke Media, wanted to build the biggest one in North America with a seven month old brand, no attendee list and an industry that doubted him. We ran teaser videos while the venue was still being secured, took the Seminole Hard Rock in Hollywood, Florida, ran two stages like a music festival and built more than 16 interactive installations ourselves. More than 800 attendees came, against a projection of 600.</t>
         </is>
       </c>
-      <c r="L28" s="7" t="inlineStr">
+      <c r="L28" s="8" t="inlineStr">
         <is>
           <t>How Danny Tran Defied the Odds and Built the Largest Permanent Makeup Event in North America on His First Try</t>
         </is>
       </c>
-      <c r="M28" s="7" t="inlineStr">
+      <c r="M28" s="8" t="inlineStr">
         <is>
           <t>Want to build the biggest event in your industry?</t>
         </is>
       </c>
-      <c r="N28" s="7" t="inlineStr">
+      <c r="N28" s="8" t="inlineStr">
         <is>
           <t>Seminole Hard Rock Hotel &amp; Casino Hollywood, Hollywood, FL</t>
         </is>
       </c>
-      <c r="O28" s="7" t="inlineStr">
+      <c r="O28" s="8" t="inlineStr">
         <is>
           <t>800+</t>
         </is>
@@ -2367,7 +2383,7 @@
           <t>4 (April 3 to 6), confirm</t>
         </is>
       </c>
-      <c r="Q28" s="7" t="inlineStr">
+      <c r="Q28" s="8" t="inlineStr">
         <is>
           <t>$148,000</t>
         </is>
@@ -2381,21 +2397,21 @@
       <c r="T28" s="5" t="inlineStr"/>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>Built from the old site's copy, Iconic's research (Juan's Slack draft, Apr 26 2023) and the interview. Left out: the event cost (rule 2), the failed festival comparison, and claims the research could not support (60 days out, 0 to 400 in 45 days, 850, almost 900). Still to answer: days on site, aftermovie. Order: PMUW 2023, then 2024, then 2025.</t>
-        </is>
-      </c>
-      <c r="V28" s="7" t="inlineStr">
+          <t>Built from the old site's copy, Iconic's research (Juan's Slack draft, Apr 26 2023) and the interview. Left out: the event cost (rule 2), the failed festival comparison, and claims the research could not support (60 days out, 0 to 400 in 45 days, 850, almost 900). Still to answer: days on site, aftermovie. Order: PMUW 2023, then 2024, then 2025. Approved by Iconic 2026-10-20, except days on site (4 by the show dates, unconfirmed) and the aftermovie link.</t>
+        </is>
+      </c>
+      <c r="V28" s="8" t="inlineStr">
         <is>
           <t>Nobody believed in this event. Danny ran a marketing agency in an industry that is mostly women, and many doubted a man could pull it off. No permanent makeup event had ever been attempted at this size, and the brand was only seven months old, with no attendee list and no past footage to show.
 So the event had to prove itself before anyone could see it. Teaser videos built the story while the venue was still being secured, and when they landed, ticket sales jumped from 100 to over 300 overnight. By the event, more than 800 people were on site, against a projection of 600.</t>
         </is>
       </c>
-      <c r="W28" s="7" t="inlineStr">
+      <c r="W28" s="8" t="inlineStr">
         <is>
           <t>Female beauty entrepreneurs and salon owners in an underserved niche, and the founders who serve a niche like that and want to give it an event of its own.</t>
         </is>
       </c>
-      <c r="X28" s="7" t="inlineStr">
+      <c r="X28" s="8" t="inlineStr">
         <is>
           <t>The riches are in the niches. PMU World could have been a beauty world or a beauty con, and it would have been too wide. Focusing on permanent makeup, a corner of the beauty industry many people do not even know exists, made a room built for one group of people, where they felt at home and every session and piece of content was made for them.
 Sell the story before the venue is signed. Teaser videos that ran while the Hard Rock was still being secured took ticket sales from 100 to over 300 overnight.</t>

</xml_diff>

<commit_message>
Record the first PMUW 2025 answer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1404,7 +1404,7 @@
       <c r="W11" s="5" t="n"/>
       <c r="X11" s="5" t="n"/>
     </row>
-    <row r="12" ht="18" customHeight="1">
+    <row r="12" ht="110" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>PMUW 2025</t>
@@ -1420,9 +1420,9 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Danny Tran</t>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Danny Tran, Founder and CEO, Highstoke Media</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -1430,22 +1430,40 @@
           <t>Interviewing</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr"/>
-      <c r="G12" s="5" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>By year three, PMU World had the room and the sponsors. Danny Tran wanted the event to travel further than the room: less straight event footage, more social content that attendees and creators would actually post.</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>1. Returned to the Seminole Hard Rock Hotel &amp; Casino Hollywood for a third year.
+2. Hired red carpet hosts to turn arrivals into content.
+3. Built more installations designed to be shared on social media.</t>
+        </is>
+      </c>
       <c r="H12" s="5" t="inlineStr"/>
       <c r="I12" s="5" t="inlineStr"/>
       <c r="J12" s="5" t="inlineStr"/>
       <c r="K12" s="5" t="inlineStr"/>
       <c r="L12" s="5" t="inlineStr"/>
       <c r="M12" s="5" t="inlineStr"/>
-      <c r="N12" s="5" t="inlineStr"/>
+      <c r="N12" s="7" t="inlineStr">
+        <is>
+          <t>Seminole Hard Rock Hotel &amp; Casino Hollywood, Hollywood, FL</t>
+        </is>
+      </c>
       <c r="O12" s="5" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr"/>
       <c r="Q12" s="5" t="inlineStr"/>
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr"/>
       <c r="T12" s="5" t="inlineStr"/>
-      <c r="U12" s="5" t="inlineStr"/>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>Month and attendance to come.</t>
+        </is>
+      </c>
       <c r="V12" s="5" t="n"/>
       <c r="W12" s="5" t="n"/>
       <c r="X12" s="5" t="n"/>

</xml_diff>

<commit_message>
Record the PMUW 2025 research and headcount, and draft its row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1404,7 +1404,7 @@
       <c r="W11" s="5" t="n"/>
       <c r="X11" s="5" t="n"/>
     </row>
-    <row r="12" ht="110" customHeight="1">
+    <row r="12" ht="300" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>PMUW 2025</t>
@@ -1415,9 +1415,9 @@
           <t>pmuw-2025</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>September 2025</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -1432,41 +1432,91 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>By year three, PMU World had the room and the sponsors. Danny Tran wanted the event to travel further than the room: less straight event footage, more social content that attendees and creators would actually post.</t>
+          <t>By year three, PMU World had the room and the sponsors. Danny Tran wanted the event to travel further than the room: less straight event footage, more social content that attendees and creators would actually post.
+The show also had to be rebuilt to close a budget gap, without the attendees or sponsors feeling the cut.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
           <t>1. Returned to the Seminole Hard Rock Hotel &amp; Casino Hollywood for a third year.
 2. Hired red carpet hosts to turn arrivals into content.
-3. Built more installations designed to be shared on social media.</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr"/>
-      <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr"/>
-      <c r="K12" s="5" t="inlineStr"/>
-      <c r="L12" s="5" t="inlineStr"/>
-      <c r="M12" s="5" t="inlineStr"/>
+3. Built more installations designed to be shared on social media.
+4. Put an editor on site to cut daily recap videos, and gave sponsors testimonial cuts for their own decks. Every session was recorded in 4K.</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>PMU World reached 1,500 attendees in person and 500 more virtually in its third year. The daily recaps, sponsor testimonial cuts and 4K recordings gave the event a life well beyond the room.
+Within a week of the show, about 130 rooms were already booked for the 2026 PMU World cruise.</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>1,500 | Attendees in person
+500 | Attendees virtual
+70% | Saved on AV</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>Show redesign to close a budget gap, social content strategy, red carpet hosts, social first installations, on site editing and daily recaps, sponsor testimonial cuts, 4K recording, sponsor booth layout, closing party, production and on site execution.</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>For year three of PMU World, Danny Tran wanted the event to live on social media as much as in the room, and the show had to close a budget gap. We hired red carpet hosts, built social first installations and put an editor on site for daily recaps, while cutting to one main stage to save about 70% on AV and trading the VIP lounge for more sponsor booths. 1,500 people came in person and 500 joined virtually, and about 130 rooms for the 2026 cruise were booked within a week.</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>How PMU World Reached 2,000 Attendees in Year Three by Building the Event for Social</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>Want an event that keeps selling after it ends?</t>
+        </is>
+      </c>
       <c r="N12" s="7" t="inlineStr">
         <is>
           <t>Seminole Hard Rock Hotel &amp; Casino Hollywood, Hollywood, FL</t>
         </is>
       </c>
-      <c r="O12" s="5" t="inlineStr"/>
+      <c r="O12" s="7" t="inlineStr">
+        <is>
+          <t>1,500 in person, 500 virtual</t>
+        </is>
+      </c>
       <c r="P12" s="5" t="inlineStr"/>
       <c r="Q12" s="5" t="inlineStr"/>
-      <c r="R12" s="5" t="inlineStr"/>
+      <c r="R12" s="7" t="inlineStr">
+        <is>
+          <t>Link to come later</t>
+        </is>
+      </c>
       <c r="S12" s="5" t="inlineStr"/>
       <c r="T12" s="5" t="inlineStr"/>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>Month and attendance to come.</t>
-        </is>
-      </c>
-      <c r="V12" s="5" t="n"/>
-      <c r="W12" s="5" t="n"/>
-      <c r="X12" s="5" t="n"/>
+          <t>Exact September dates and days on site to confirm. Wi-Fi challenge: how was the footage moved? The 70% AV saving could also be the cost saved metric. DAER (nightclub name) left out; the page says the pool areas. Red carpet hosts as a second Steal This? Danny's title: founder and CEO (newest source 2023).</t>
+        </is>
+      </c>
+      <c r="V12" s="7" t="inlineStr">
+        <is>
+          <t>Closing the budget gap meant rebuilding the show. Cutting to one main stage saved about 70% on AV, and dropping the VIP lounge made room for more sponsor booths. The closing party moved to the Hard Rock's own pool areas.
+Slow hotel Wi-Fi made moving about 100 GB of footage a challenge, with daily recaps still going out from the on site editor.</t>
+        </is>
+      </c>
+      <c r="W12" s="7" t="inlineStr">
+        <is>
+          <t>Founders in permanent makeup and the neighboring corners of the beauty industry, who want an event that lives on social media as much as in the room.</t>
+        </is>
+      </c>
+      <c r="X12" s="7" t="inlineStr">
+        <is>
+          <t>Sell next year at this year's show. PMU World sold its 2025 pre-sale at the 2024 event, and about 130 rooms for the 2026 cruise were booked within a week of the 2025 show. Attendees never buy more easily than while they are still in the room.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Drop the budget gap from PMUW 2025 and add the AV saving
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1432,8 +1432,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>By year three, PMU World had the room and the sponsors. Danny Tran wanted the event to travel further than the room: less straight event footage, more social content that attendees and creators would actually post.
-The show also had to be rebuilt to close a budget gap, without the attendees or sponsors feeling the cut.</t>
+          <t>By year three, PMU World had the room and the sponsors. Danny Tran wanted the event to travel further than the room: less straight event footage, more social content that attendees and creators would actually post.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1441,7 +1440,9 @@
           <t>1. Returned to the Seminole Hard Rock Hotel &amp; Casino Hollywood for a third year.
 2. Hired red carpet hosts to turn arrivals into content.
 3. Built more installations designed to be shared on social media.
-4. Put an editor on site to cut daily recap videos, and gave sponsors testimonial cuts for their own decks. Every session was recorded in 4K.</t>
+4. Put an editor on site to cut daily recap videos, and gave sponsors testimonial cuts for their own decks. Every session was recorded in 4K.
+5. Focused the show on one main stage, saving $140,000 on AV, and traded the VIP lounge for more sponsor booths.
+6. Moved the closing party to the Hard Rock's own pool areas.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -1454,17 +1455,17 @@
         <is>
           <t>1,500 | Attendees in person
 500 | Attendees virtual
-70% | Saved on AV</t>
+$140K | Saved on AV</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>Show redesign to close a budget gap, social content strategy, red carpet hosts, social first installations, on site editing and daily recaps, sponsor testimonial cuts, 4K recording, sponsor booth layout, closing party, production and on site execution.</t>
+          <t>Social content strategy, red carpet hosts, social first installations, on site editing and daily recaps, sponsor testimonial cuts, 4K recording, stage and sponsor booth layout, closing party, production and on site execution.</t>
         </is>
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>For year three of PMU World, Danny Tran wanted the event to live on social media as much as in the room, and the show had to close a budget gap. We hired red carpet hosts, built social first installations and put an editor on site for daily recaps, while cutting to one main stage to save about 70% on AV and trading the VIP lounge for more sponsor booths. 1,500 people came in person and 500 joined virtually, and about 130 rooms for the 2026 cruise were booked within a week.</t>
+          <t>For year three of PMU World, Danny Tran wanted the event to live on social media as much as in the room. We hired red carpet hosts, built social first installations and put an editor on site for daily recaps and sponsor testimonial cuts, all recorded in 4K. Focusing the show on one main stage saved $140,000 on AV and made room for more sponsor booths. 1,500 people came in person and 500 joined virtually, and about 130 rooms for the 2026 cruise were booked within a week.</t>
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr">
@@ -1488,7 +1489,11 @@
         </is>
       </c>
       <c r="P12" s="5" t="inlineStr"/>
-      <c r="Q12" s="5" t="inlineStr"/>
+      <c r="Q12" s="7" t="inlineStr">
+        <is>
+          <t>$140,000</t>
+        </is>
+      </c>
       <c r="R12" s="7" t="inlineStr">
         <is>
           <t>Link to come later</t>
@@ -1498,13 +1503,12 @@
       <c r="T12" s="5" t="inlineStr"/>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>Exact September dates and days on site to confirm. Wi-Fi challenge: how was the footage moved? The 70% AV saving could also be the cost saved metric. DAER (nightclub name) left out; the page says the pool areas. Red carpet hosts as a second Steal This? Danny's title: founder and CEO (newest source 2023).</t>
-        </is>
-      </c>
-      <c r="V12" s="7" t="inlineStr">
-        <is>
-          <t>Closing the budget gap meant rebuilding the show. Cutting to one main stage saved about 70% on AV, and dropping the VIP lounge made room for more sponsor booths. The closing party moved to the Hard Rock's own pool areas.
-Slow hotel Wi-Fi made moving about 100 GB of footage a challenge, with daily recaps still going out from the on site editor.</t>
+          <t>No budget gap on the page (Iconic). Exact September dates and days on site to confirm. Steal This overlaps PMUW 2024 (sell next year at this year's show): red carpet hosts instead? DAER (nightclub name) left out.</t>
+        </is>
+      </c>
+      <c r="V12" s="5" t="inlineStr">
+        <is>
+          <t>None for now. The budget gap stays off the page (Iconic). Add the Wi-Fi story only if Iconic says how the footage was moved.</t>
         </is>
       </c>
       <c r="W12" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Approve the PMUW 2025 row with its dates and Steal This
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1415,27 +1415,27 @@
           <t>pmuw-2025</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>September 2025</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Danny Tran, Founder and CEO, Highstoke Media</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
+          <t>Ready to build</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>By year three, PMU World had the room and the sponsors. Danny Tran wanted the event to travel further than the room: less straight event footage, more social content that attendees and creators would actually post.</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="8" t="inlineStr">
         <is>
           <t>1. Returned to the Seminole Hard Rock Hotel &amp; Casino Hollywood for a third year.
 2. Hired red carpet hosts to turn arrivals into content.
@@ -1445,51 +1445,55 @@
 6. Moved the closing party to the Hard Rock's own pool areas.</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>PMU World reached 1,500 attendees in person and 500 more virtually in its third year. The daily recaps, sponsor testimonial cuts and 4K recordings gave the event a life well beyond the room.
 Within a week of the show, about 130 rooms were already booked for the 2026 PMU World cruise.</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>1,500 | Attendees in person
 500 | Attendees virtual
 $140K | Saved on AV</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr">
         <is>
           <t>Social content strategy, red carpet hosts, social first installations, on site editing and daily recaps, sponsor testimonial cuts, 4K recording, stage and sponsor booth layout, closing party, production and on site execution.</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
-        <is>
-          <t>For year three of PMU World, Danny Tran wanted the event to live on social media as much as in the room. We hired red carpet hosts, built social first installations and put an editor on site for daily recaps and sponsor testimonial cuts, all recorded in 4K. Focusing the show on one main stage saved $140,000 on AV and made room for more sponsor booths. 1,500 people came in person and 500 joined virtually, and about 130 rooms for the 2026 cruise were booked within a week.</t>
-        </is>
-      </c>
-      <c r="L12" s="7" t="inlineStr">
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>For year three of PMU World, Danny Tran wanted the event to live on social media as much as in the room. We hired red carpet hosts, built social first installations and put an editor on site for daily recaps and sponsor testimonial cuts, all recorded in 4K. Focusing the show on one main stage saved $140,000 on AV and made room for more sponsor booths. Over four days in September 2025, 1,500 people came in person and 500 joined virtually, and about 130 rooms for the 2026 cruise were booked within a week.</t>
+        </is>
+      </c>
+      <c r="L12" s="8" t="inlineStr">
         <is>
           <t>How PMU World Reached 2,000 Attendees in Year Three by Building the Event for Social</t>
         </is>
       </c>
-      <c r="M12" s="7" t="inlineStr">
+      <c r="M12" s="8" t="inlineStr">
         <is>
           <t>Want an event that keeps selling after it ends?</t>
         </is>
       </c>
-      <c r="N12" s="7" t="inlineStr">
+      <c r="N12" s="8" t="inlineStr">
         <is>
           <t>Seminole Hard Rock Hotel &amp; Casino Hollywood, Hollywood, FL</t>
         </is>
       </c>
-      <c r="O12" s="7" t="inlineStr">
+      <c r="O12" s="8" t="inlineStr">
         <is>
           <t>1,500 in person, 500 virtual</t>
         </is>
       </c>
-      <c r="P12" s="5" t="inlineStr"/>
-      <c r="Q12" s="7" t="inlineStr">
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="Q12" s="8" t="inlineStr">
         <is>
           <t>$140,000</t>
         </is>
@@ -1500,10 +1504,14 @@
         </is>
       </c>
       <c r="S12" s="5" t="inlineStr"/>
-      <c r="T12" s="5" t="inlineStr"/>
+      <c r="T12" s="7" t="inlineStr">
+        <is>
+          <t>Photos to come later</t>
+        </is>
+      </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>No budget gap on the page (Iconic). Exact September dates and days on site to confirm. Steal This overlaps PMUW 2024 (sell next year at this year's show): red carpet hosts instead? DAER (nightclub name) left out.</t>
+          <t>Approved by Iconic 2026-10-20. September 8 to 11, 2025 (load-in Sep 7, load-out Sep 12). Days on site counted as 4 show days, matching the other pages. No budget gap on the page. Aftermovie and photos to come later.</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
@@ -1511,14 +1519,14 @@
           <t>None for now. The budget gap stays off the page (Iconic). Add the Wi-Fi story only if Iconic says how the footage was moved.</t>
         </is>
       </c>
-      <c r="W12" s="7" t="inlineStr">
+      <c r="W12" s="8" t="inlineStr">
         <is>
           <t>Founders in permanent makeup and the neighboring corners of the beauty industry, who want an event that lives on social media as much as in the room.</t>
         </is>
       </c>
-      <c r="X12" s="7" t="inlineStr">
-        <is>
-          <t>Sell next year at this year's show. PMU World sold its 2025 pre-sale at the 2024 event, and about 130 rooms for the 2026 cruise were booked within a week of the 2025 show. Attendees never buy more easily than while they are still in the room.</t>
+      <c r="X12" s="8" t="inlineStr">
+        <is>
+          <t>Hire red carpet hosts. Arrival becomes a moment worth posting, and the event's social content starts before the first session does.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Start the Net Rev Summit 2026 interview with leads from Fathom calls
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -836,7 +836,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Interviewing</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr"/>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Ready to build</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Ready to build</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Ready to build</t>
+          <t>Built</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Park Net Rev Summit 2026 until the testimonial links arrive
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -836,7 +836,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr"/>
@@ -856,9 +856,17 @@
       <c r="P3" s="5" t="inlineStr"/>
       <c r="Q3" s="5" t="inlineStr"/>
       <c r="R3" s="5" t="inlineStr"/>
-      <c r="S3" s="5" t="inlineStr"/>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>Video testimonials coming as YouTube links</t>
+        </is>
+      </c>
       <c r="T3" s="5" t="inlineStr"/>
-      <c r="U3" s="5" t="inlineStr"/>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>Parked 2026-10-20 until Iconic sends the YouTube testimonial links. Leads in the notes file (Fathom summaries).</t>
+        </is>
+      </c>
       <c r="V3" s="5" t="n"/>
       <c r="W3" s="5" t="n"/>
       <c r="X3" s="5" t="n"/>

</xml_diff>

<commit_message>
Start the Decentralized Masters Live interview with Fathom leads
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -894,7 +894,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Interviewing</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr"/>
@@ -912,7 +912,11 @@
       <c r="R4" s="5" t="inlineStr"/>
       <c r="S4" s="5" t="inlineStr"/>
       <c r="T4" s="5" t="inlineStr"/>
-      <c r="U4" s="5" t="inlineStr"/>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>This row is the March 2026 Fontainebleau event. Vegas (Nov 2026, not yet happened) and Austin (Sep 2026) are separate DML events, not on the grid yet.</t>
+        </is>
+      </c>
       <c r="V4" s="5" t="n"/>
       <c r="W4" s="5" t="n"/>
       <c r="X4" s="5" t="n"/>

</xml_diff>

<commit_message>
Record the first Decentralized Masters Live answer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -871,7 +871,7 @@
       <c r="W3" s="5" t="n"/>
       <c r="X3" s="5" t="n"/>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4" ht="140" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Decentralized Masters Live</t>
@@ -897,7 +897,11 @@
           <t>Interviewing</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Tan and Salim had built a community of accredited investors, an established and discerning group. They wanted to bring them together in person for the first time, to impress them and connect them with the team, but they did not know where to start. This was their first live event, and the guests were coming from countries and cultures around the world.</t>
+        </is>
+      </c>
       <c r="G4" s="5" t="inlineStr"/>
       <c r="H4" s="5" t="inlineStr"/>
       <c r="I4" s="5" t="inlineStr"/>
@@ -908,16 +912,24 @@
       <c r="N4" s="5" t="inlineStr"/>
       <c r="O4" s="5" t="inlineStr"/>
       <c r="P4" s="5" t="inlineStr"/>
-      <c r="Q4" s="5" t="inlineStr"/>
+      <c r="Q4" s="7" t="inlineStr">
+        <is>
+          <t>About $70,000 (exact figure?)</t>
+        </is>
+      </c>
       <c r="R4" s="5" t="inlineStr"/>
       <c r="S4" s="5" t="inlineStr"/>
       <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>This row is the March 2026 Fontainebleau event. Vegas (Nov 2026, not yet happened) and Austin (Sep 2026) are separate DML events, not on the grid yet.</t>
-        </is>
-      </c>
-      <c r="V4" s="5" t="n"/>
+          <t>This row is the March 2026 Fontainebleau event. Vegas (Nov 2026, not yet happened) and Austin (Sep 2026) are separate DML events, not on the grid yet. Leave out the two years of date talks (Iconic). Confirm: Tan or Dan; Fontainebleau Miami Beach; exact saving.</t>
+        </is>
+      </c>
+      <c r="V4" s="7" t="inlineStr">
+        <is>
+          <t>Shortly before the event, war broke out where Tan and Salim were staying in Dubai, and the hotel commitments became almost impossible to honor. Plenty of event companies would have walked away. We went to the Eden Roc and worked with them to waive the contractual hotel commitments, which saved the client about $70,000, and the event went ahead.</t>
+        </is>
+      </c>
       <c r="W4" s="5" t="n"/>
       <c r="X4" s="5" t="n"/>
     </row>

</xml_diff>

<commit_message>
Record the Decentralized Masters Live names, venue and saving
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -887,9 +887,9 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Tan and Salim</t>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Tan and Salim, Co-Founders, Decentralized Masters</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -909,12 +909,16 @@
       <c r="K4" s="5" t="inlineStr"/>
       <c r="L4" s="5" t="inlineStr"/>
       <c r="M4" s="5" t="inlineStr"/>
-      <c r="N4" s="5" t="inlineStr"/>
+      <c r="N4" s="7" t="inlineStr">
+        <is>
+          <t>Fontainebleau Miami Beach, Miami Beach, FL</t>
+        </is>
+      </c>
       <c r="O4" s="5" t="inlineStr"/>
       <c r="P4" s="5" t="inlineStr"/>
       <c r="Q4" s="7" t="inlineStr">
         <is>
-          <t>About $70,000 (exact figure?)</t>
+          <t>$51,000</t>
         </is>
       </c>
       <c r="R4" s="5" t="inlineStr"/>
@@ -922,12 +926,12 @@
       <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>This row is the March 2026 Fontainebleau event. Vegas (Nov 2026, not yet happened) and Austin (Sep 2026) are separate DML events, not on the grid yet. Leave out the two years of date talks (Iconic). Confirm: Tan or Dan; Fontainebleau Miami Beach; exact saving.</t>
+          <t>This row is the March 2026 Fontainebleau event. Vegas (Nov 2026) and Austin (Sep 2026) are separate DML events. Leave out the two years of date talks (Iconic).</t>
         </is>
       </c>
       <c r="V4" s="7" t="inlineStr">
         <is>
-          <t>Shortly before the event, war broke out where Tan and Salim were staying in Dubai, and the hotel commitments became almost impossible to honor. Plenty of event companies would have walked away. We went to the Eden Roc and worked with them to waive the contractual hotel commitments, which saved the client about $70,000, and the event went ahead.</t>
+          <t>Shortly before the event, war broke out where Tan and Salim were staying in Dubai, and the hotel commitments became almost impossible to honor. Plenty of event companies would have walked away. We went to the Eden Roc and worked with them to waive the contractual hotel commitments, which saved the client $51,000 in attrition fees they would otherwise have had to pay, and the event went ahead.</t>
         </is>
       </c>
       <c r="W4" s="5" t="n"/>

</xml_diff>

<commit_message>
Record the Decentralized Masters Live decisions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -902,7 +902,12 @@
           <t>Tan and Salim had built a community of accredited investors, an established and discerning group. They wanted to bring them together in person for the first time, to impress them and connect them with the team, but they did not know where to start. This was their first live event, and the guests were coming from countries and cultures around the world.</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>1. Took the Fontainebleau's Presidential Suite for the VIP opening mixer, negotiating it from $22,000 a night down to $16,000, so the first night opened in a penthouse with views over the ocean and the whole city.
+2. Moved fast when plans changed, from hotel commitments to the program, so attendees never felt the pivots.</t>
+        </is>
+      </c>
       <c r="H4" s="5" t="inlineStr"/>
       <c r="I4" s="5" t="inlineStr"/>
       <c r="J4" s="5" t="inlineStr"/>
@@ -926,7 +931,7 @@
       <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>This row is the March 2026 Fontainebleau event. Vegas (Nov 2026) and Austin (Sep 2026) are separate DML events. Leave out the two years of date talks (Iconic).</t>
+          <t>This row is the March 2026 Fontainebleau event. Vegas (Nov 2026) and Austin (Sep 2026) are separate DML events. Leave out the two years of date talks (Iconic). Never mention the yacht (Iconic).</t>
         </is>
       </c>
       <c r="V4" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Draft the rest of the Decentralized Masters Live row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -871,7 +871,7 @@
       <c r="W3" s="5" t="n"/>
       <c r="X3" s="5" t="n"/>
     </row>
-    <row r="4" ht="140" customHeight="1">
+    <row r="4" ht="260" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Decentralized Masters Live</t>
@@ -882,9 +882,9 @@
           <t>decentralized-masters-live</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>March 2026</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -908,19 +908,54 @@
 2. Moved fast when plans changed, from hotel commitments to the program, so attendees never felt the pivots.</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="5" t="inlineStr"/>
-      <c r="K4" s="5" t="inlineStr"/>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>The investors loved it. Meeting Tan and Salim in person, among peers from around the world, turned an online community into a room that wanted more.
+So much more that Tan and Salim launched their first high ticket offer on the back of it: the Inflection Club, built as a continuation of the community attendees had just experienced. More than 30 new members joined. Attendees kept asking where the next one would be, and the answer is Las Vegas in November 2026, which we are producing.</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>280 | Accredited investors on site
+30+ | New Inflection Club members
+$51K | Hotel attrition fees waived</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>Event design for a first live event, venue and hotel negotiations including the Presidential Suite and the attrition waiver, the VIP opening mixer, program and production, on site execution across three and a half days.</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Tan and Salim, co-founders of Decentralized Masters, had a community of accredited investors from around the world and no live event behind them. We designed their first, at the Fontainebleau Miami Beach, opening with a VIP mixer in the Presidential Suite. When war broke out where they were staying, we worked with the Eden Roc to waive $51,000 in hotel attrition fees and kept the event on track. About 280 investors attended, more than 30 joined the new Inflection Club, and attendees asked for the next one.</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>How Decentralized Masters Turned Its First Live Event Into a High Ticket Club With 30+ New Members</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>Want your community's first event to launch your next offer?</t>
+        </is>
+      </c>
       <c r="N4" s="7" t="inlineStr">
         <is>
           <t>Fontainebleau Miami Beach, Miami Beach, FL</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr"/>
-      <c r="P4" s="5" t="inlineStr"/>
+      <c r="O4" s="7" t="inlineStr">
+        <is>
+          <t>280 (given as just about 280)</t>
+        </is>
+      </c>
+      <c r="P4" s="7" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
       <c r="Q4" s="7" t="inlineStr">
         <is>
           <t>$51,000</t>
@@ -931,7 +966,7 @@
       <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>This row is the March 2026 Fontainebleau event. Vegas (Nov 2026) and Austin (Sep 2026) are separate DML events. Leave out the two years of date talks (Iconic). Never mention the yacht (Iconic).</t>
+          <t>This row is the March 2026 Fontainebleau event. Vegas (Nov 2026) and Austin (Sep 2026) are separate DML events. Leave out the two years of date talks (Iconic). Never mention the yacht (Iconic). Attendance given as just about 280. Sign up amounts never disclosed. Nightly suite rate on the page: OK to publish? Right for and Steal This drafted, not yet answered.</t>
         </is>
       </c>
       <c r="V4" s="7" t="inlineStr">
@@ -939,8 +974,16 @@
           <t>Shortly before the event, war broke out where Tan and Salim were staying in Dubai, and the hotel commitments became almost impossible to honor. Plenty of event companies would have walked away. We went to the Eden Roc and worked with them to waive the contractual hotel commitments, which saved the client $51,000 in attrition fees they would otherwise have had to pay, and the event went ahead.</t>
         </is>
       </c>
-      <c r="W4" s="5" t="n"/>
-      <c r="X4" s="5" t="n"/>
+      <c r="W4" s="7" t="inlineStr">
+        <is>
+          <t>Founders with an established online community, especially investors or other high value members, who are hosting their first live event and want it to open the door to a premium offer.</t>
+        </is>
+      </c>
+      <c r="X4" s="7" t="inlineStr">
+        <is>
+          <t>Design the room as the first chapter of your next offer. Decentralized Masters built the Inflection Club as a continuation of the community attendees had just experienced in person, so joining felt like staying, not buying.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Approve the Decentralized Masters Live row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -882,104 +882,112 @@
           <t>decentralized-masters-live</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>March 2026</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Tan and Salim, Co-Founders, Decentralized Masters</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
+          <t>Ready to build</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Tan and Salim had built a community of accredited investors, an established and discerning group. They wanted to bring them together in person for the first time, to impress them and connect them with the team, but they did not know where to start. This was their first live event, and the guests were coming from countries and cultures around the world.</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>1. Took the Fontainebleau's Presidential Suite for the VIP opening mixer, negotiating it from $22,000 a night down to $16,000, so the first night opened in a penthouse with views over the ocean and the whole city.
 2. Moved fast when plans changed, from hotel commitments to the program, so attendees never felt the pivots.</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>The investors loved it. Meeting Tan and Salim in person, among peers from around the world, turned an online community into a room that wanted more.
-So much more that Tan and Salim launched their first high ticket offer on the back of it: the Inflection Club, built as a continuation of the community attendees had just experienced. More than 30 new members joined. Attendees kept asking where the next one would be, and the answer is Las Vegas in November 2026, which we are producing.</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr">
+So much more that Tan and Salim launched their first high ticket offer on the back of it: the Inflection Club, built as a continuation of the community attendees had just experienced. More than 30 new members joined. Attendees kept asking where the next one would be. Now members build their year around it: Miami first, then Austin with the Inflection Club, and next Las Vegas in November 2026, which we are producing.</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>280 | Accredited investors on site
 30+ | New Inflection Club members
 $51K | Hotel attrition fees waived</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="J4" s="8" t="inlineStr">
         <is>
           <t>Event design for a first live event, venue and hotel negotiations including the Presidential Suite and the attrition waiver, the VIP opening mixer, program and production, on site execution across three and a half days.</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
+      <c r="K4" s="8" t="inlineStr">
         <is>
           <t>Tan and Salim, co-founders of Decentralized Masters, had a community of accredited investors from around the world and no live event behind them. We designed their first, at the Fontainebleau Miami Beach, opening with a VIP mixer in the Presidential Suite. When war broke out where they were staying, we worked with the Eden Roc to waive $51,000 in hotel attrition fees and kept the event on track. About 280 investors attended, more than 30 joined the new Inflection Club, and attendees asked for the next one.</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr">
+      <c r="L4" s="8" t="inlineStr">
         <is>
           <t>How Decentralized Masters Turned Its First Live Event Into a High Ticket Club With 30+ New Members</t>
         </is>
       </c>
-      <c r="M4" s="7" t="inlineStr">
+      <c r="M4" s="8" t="inlineStr">
         <is>
           <t>Want your community's first event to launch your next offer?</t>
         </is>
       </c>
-      <c r="N4" s="7" t="inlineStr">
+      <c r="N4" s="8" t="inlineStr">
         <is>
           <t>Fontainebleau Miami Beach, Miami Beach, FL</t>
         </is>
       </c>
-      <c r="O4" s="7" t="inlineStr">
-        <is>
-          <t>280 (given as just about 280)</t>
-        </is>
-      </c>
-      <c r="P4" s="7" t="inlineStr">
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t>280</t>
+        </is>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="Q4" s="7" t="inlineStr">
+      <c r="Q4" s="8" t="inlineStr">
         <is>
           <t>$51,000</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr"/>
+      <c r="R4" s="7" t="inlineStr">
+        <is>
+          <t>Link to come later</t>
+        </is>
+      </c>
       <c r="S4" s="5" t="inlineStr"/>
-      <c r="T4" s="5" t="inlineStr"/>
+      <c r="T4" s="7" t="inlineStr">
+        <is>
+          <t>Photos to come later</t>
+        </is>
+      </c>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>This row is the March 2026 Fontainebleau event. Vegas (Nov 2026) and Austin (Sep 2026) are separate DML events. Leave out the two years of date talks (Iconic). Never mention the yacht (Iconic). Attendance given as just about 280. Sign up amounts never disclosed. Nightly suite rate on the page: OK to publish? Right for and Steal This drafted, not yet answered.</t>
-        </is>
-      </c>
-      <c r="V4" s="7" t="inlineStr">
+          <t>Approved by Iconic 2026-10-23. March 2026 Fontainebleau event; Vegas (Nov 2026) and Austin are separate. Never mention the yacht. Leave out the two years of date talks. Sign up amounts never disclosed. Suite rate OK to publish.</t>
+        </is>
+      </c>
+      <c r="V4" s="8" t="inlineStr">
         <is>
           <t>Shortly before the event, war broke out where Tan and Salim were staying in Dubai, and the hotel commitments became almost impossible to honor. Plenty of event companies would have walked away. We went to the Eden Roc and worked with them to waive the contractual hotel commitments, which saved the client $51,000 in attrition fees they would otherwise have had to pay, and the event went ahead.</t>
         </is>
       </c>
-      <c r="W4" s="7" t="inlineStr">
-        <is>
-          <t>Founders with an established online community, especially investors or other high value members, who are hosting their first live event and want it to open the door to a premium offer.</t>
-        </is>
-      </c>
-      <c r="X4" s="7" t="inlineStr">
+      <c r="W4" s="8" t="inlineStr">
+        <is>
+          <t>Any founder with an investment community, or any community they want to keep for the long term. The strongest way to retain it is to strengthen the connections between members by bringing them together in person. That is what Decentralized Masters did, and it is what let them launch the Inflection Club, open new investment opportunities and build an experience members plan their year around.</t>
+        </is>
+      </c>
+      <c r="X4" s="8" t="inlineStr">
         <is>
           <t>Design the room as the first chapter of your next offer. Decentralized Masters built the Inflection Club as a continuation of the community attendees had just experienced in person, so joining felt like staying, not buying.</t>
         </is>

</xml_diff>

<commit_message>
Start the Fast Start Forum 2024 interview
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -2241,17 +2241,21 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Tom Wall</t>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Tom Wall, Whole Life Mastermind</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr"/>
+          <t>Interviewing</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Life insurance events had a reputation: stuffy ballrooms, no excitement and no mixers worth staying for. Tom Wall, who runs Whole Life Mastermind, a mastermind and support group for life insurance agents, wanted to build something better for the agents in his community.</t>
+        </is>
+      </c>
       <c r="G23" s="5" t="inlineStr"/>
       <c r="H23" s="5" t="inlineStr"/>
       <c r="I23" s="5" t="inlineStr"/>
@@ -2259,14 +2263,22 @@
       <c r="K23" s="5" t="inlineStr"/>
       <c r="L23" s="5" t="inlineStr"/>
       <c r="M23" s="5" t="inlineStr"/>
-      <c r="N23" s="5" t="inlineStr"/>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>Hilton Fort Lauderdale Marina, Fort Lauderdale, FL</t>
+        </is>
+      </c>
       <c r="O23" s="5" t="inlineStr"/>
       <c r="P23" s="5" t="inlineStr"/>
       <c r="Q23" s="5" t="inlineStr"/>
       <c r="R23" s="5" t="inlineStr"/>
       <c r="S23" s="5" t="inlineStr"/>
       <c r="T23" s="5" t="inlineStr"/>
-      <c r="U23" s="5" t="inlineStr"/>
+      <c r="U23" s="5" t="inlineStr">
+        <is>
+          <t>Date to come. Confirm the venue name and Tom's title.</t>
+        </is>
+      </c>
       <c r="V23" s="5" t="n"/>
       <c r="W23" s="5" t="n"/>
       <c r="X23" s="5" t="n"/>

</xml_diff>

<commit_message>
Record the Fast Start Forum research without its financial figures
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -2236,9 +2236,9 @@
           <t>fast-start-forum-2024</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>2024</t>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>February 2025 (sold in 2024)</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -2256,7 +2256,15 @@
           <t>Life insurance events had a reputation: stuffy ballrooms, no excitement and no mixers worth staying for. Tom Wall, who runs Whole Life Mastermind, a mastermind and support group for life insurance agents, wanted to build something better for the agents in his community.</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr"/>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>1. Launched publicly on November 6 for a February event, a three month window to sell the room.
+2. Opened Sunday with registration and a mixer, so agents met before the first session.
+3. Ended Monday's sessions at Topgolf instead of another ballroom reception.
+4. Closed Tuesday with a VIP dinner at YOLO.
+5. Built a speaker lineup of 11, hosted by Tom Wall, including Garrett Gunderson, Vince D'Addona and Kristin Andree.</t>
+        </is>
+      </c>
       <c r="H23" s="5" t="inlineStr"/>
       <c r="I23" s="5" t="inlineStr"/>
       <c r="J23" s="5" t="inlineStr"/>
@@ -2276,7 +2284,7 @@
       <c r="T23" s="5" t="inlineStr"/>
       <c r="U23" s="5" t="inlineStr">
         <is>
-          <t>Date to come. Confirm the venue name and Tom's title.</t>
+          <t>Research: held Feb 2 to 4, 2025 though sold in 2024; no earlier edition found. Financial figures from the research kept out of the notes and sheet (house rules 1 and 2). Attendance: tracker 194 including 10 speakers and 8 team (176 ticketed); which to publish? Is fast-start-forum-2025 a later edition, or the same event?</t>
         </is>
       </c>
       <c r="V23" s="5" t="n"/>

</xml_diff>

<commit_message>
Confirm Fast Start Forum 2024 venue, year and attendance
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -2238,7 +2238,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>February 2025 (sold in 2024)</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>1. Launched publicly on November 6 for a February event, a three month window to sell the room.
+          <t>1. Launched publicly with about three months to sell the room.
 2. Opened Sunday with registration and a mixer, so agents met before the first session.
 3. Ended Monday's sessions at Topgolf instead of another ballroom reception.
 4. Closed Tuesday with a VIP dinner at YOLO.
@@ -2276,7 +2276,11 @@
           <t>Hilton Fort Lauderdale Marina, Fort Lauderdale, FL</t>
         </is>
       </c>
-      <c r="O23" s="5" t="inlineStr"/>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>194</t>
+        </is>
+      </c>
       <c r="P23" s="5" t="inlineStr"/>
       <c r="Q23" s="5" t="inlineStr"/>
       <c r="R23" s="5" t="inlineStr"/>
@@ -2284,7 +2288,7 @@
       <c r="T23" s="5" t="inlineStr"/>
       <c r="U23" s="5" t="inlineStr">
         <is>
-          <t>Research: held Feb 2 to 4, 2025 though sold in 2024; no earlier edition found. Financial figures from the research kept out of the notes and sheet (house rules 1 and 2). Attendance: tracker 194 including 10 speakers and 8 team (176 ticketed); which to publish? Is fast-start-forum-2025 a later edition, or the same event?</t>
+          <t>Iconic: first event, held in 2024, 194 attendees, Hilton Fort Lauderdale Marina. (Research had Feb 2 to 4, 2025; Iconic's answer stands.) Financial figures from the research kept out (house rules 1 and 2). Still to answer: what made it hard, why Topgolf and YOLO.</t>
         </is>
       </c>
       <c r="V23" s="5" t="n"/>

</xml_diff>

<commit_message>
Record why Fast Start Forum 2024 went to Topgolf and YOLO
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -2260,8 +2260,8 @@
         <is>
           <t>1. Launched publicly with about three months to sell the room.
 2. Opened Sunday with registration and a mixer, so agents met before the first session.
-3. Ended Monday's sessions at Topgolf instead of another ballroom reception.
-4. Closed Tuesday with a VIP dinner at YOLO.
+3. Took Monday night to Topgolf instead of another ballroom reception and open bar, so agents bonded over something they could do together. Tom is a big golfer, and it gave him the chance to show it.
+4. Closed Tuesday with a VIP dinner at YOLO, one of Fort Lauderdale's hottest destinations, with live jazz and a floor to dance on.
 5. Built a speaker lineup of 11, hosted by Tom Wall, including Garrett Gunderson, Vince D'Addona and Kristin Andree.</t>
         </is>
       </c>
@@ -2291,7 +2291,11 @@
           <t>Iconic: first event, held in 2024, 194 attendees, Hilton Fort Lauderdale Marina. (Research had Feb 2 to 4, 2025; Iconic's answer stands.) Financial figures from the research kept out (house rules 1 and 2). Still to answer: what made it hard, why Topgolf and YOLO.</t>
         </is>
       </c>
-      <c r="V23" s="5" t="n"/>
+      <c r="V23" s="5" t="inlineStr">
+        <is>
+          <t>None (Iconic: no "what made it hard" for this event).</t>
+        </is>
+      </c>
       <c r="W23" s="5" t="n"/>
       <c r="X23" s="5" t="n"/>
     </row>

</xml_diff>

<commit_message>
Draft the rest of the Fast Start Forum 2024 row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -2225,7 +2225,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
+    <row r="23" ht="260" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Fast Start Forum 2024</t>
@@ -2265,12 +2265,37 @@
 5. Built a speaker lineup of 11, hosted by Tom Wall, including Garrett Gunderson, Vince D'Addona and Kristin Andree.</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr"/>
-      <c r="I23" s="5" t="inlineStr"/>
-      <c r="J23" s="5" t="inlineStr"/>
-      <c r="K23" s="5" t="inlineStr"/>
-      <c r="L23" s="5" t="inlineStr"/>
-      <c r="M23" s="5" t="inlineStr"/>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>It went really well. 194 attendees came to the first Fast Start Forum, and Tom sold several spots in his first offer, along with a couple of places in the Inner Circle Mastermind we helped him design. The agents left having bonded over golf and jazz instead of another ballroom reception, and Tom brought the event back the next year.</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>194 | Attendees at the first Fast Start Forum
+11 | Speakers on the program</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>Event design and management, the Inner Circle Mastermind offer design, venue at the Hilton Fort Lauderdale Marina, the speaker program, the Topgolf night and the VIP dinner at YOLO, production and on site execution.</t>
+        </is>
+      </c>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>Life insurance events usually start and end in a stuffy ballroom. Tom Wall of Whole Life Mastermind wanted something better for his agents. For the first Fast Start Forum, at the Hilton Fort Lauderdale Marina, we opened with a Sunday mixer, took Monday night to Topgolf and closed with a VIP dinner and live jazz at YOLO, around a program of 11 speakers. 194 attendees came, and Tom sold several spots in his first offer and in the Inner Circle Mastermind we helped him design.</t>
+        </is>
+      </c>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>How Fast Start Forum Took Life Insurance Agents Out of the Ballroom and Launched Tom Wall's Inner Circle Mastermind</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>Want an event your industry has never seen before?</t>
+        </is>
+      </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
           <t>Hilton Fort Lauderdale Marina, Fort Lauderdale, FL</t>
@@ -2288,7 +2313,7 @@
       <c r="T23" s="5" t="inlineStr"/>
       <c r="U23" s="5" t="inlineStr">
         <is>
-          <t>Iconic: first event, held in 2024, 194 attendees, Hilton Fort Lauderdale Marina. (Research had Feb 2 to 4, 2025; Iconic's answer stands.) Financial figures from the research kept out (house rules 1 and 2). Still to answer: what made it hard, why Topgolf and YOLO.</t>
+          <t>Iconic: first event, held in 2024, 194 attendees, Hilton Fort Lauderdale Marina. (Research had Feb 2 to 4, 2025; Iconic's answer stands.) Financial figures from the research kept out (house rules 1 and 2). "City council" in the right for answer read as a transcription error; check. "Brought the event back the next year" assumes the 2025 edition followed this one.</t>
         </is>
       </c>
       <c r="V23" s="5" t="inlineStr">
@@ -2296,8 +2321,16 @@
           <t>None (Iconic: no "what made it hard" for this event).</t>
         </is>
       </c>
-      <c r="W23" s="5" t="n"/>
-      <c r="X23" s="5" t="n"/>
+      <c r="W23" s="7" t="inlineStr">
+        <is>
+          <t>Any industry whose events tend to be standardized and stale, such as insurance or health and wellness, where events usually start and end in a ballroom. Fast Start Forum is a model for breaking that pattern.</t>
+        </is>
+      </c>
+      <c r="X23" s="7" t="inlineStr">
+        <is>
+          <t>Replace the ballroom mixer with an experience. A night at Topgolf gave agents something to do together, not just something to drink, and the bonding carried back into the sessions. Pick an activity your host loves, too: Tom is a big golfer, and it showed.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Build Fast Start Forum 2024 and size highlights to their count
Add the approved Fast Start Forum 2024 row as a case study. The How It
Went highlights now take as many columns as a page has highlights, so two
no longer leave an empty third column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -2236,27 +2236,27 @@
           <t>fast-start-forum-2024</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Tom Wall, Whole Life Mastermind</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>Life insurance events had a reputation: stuffy ballrooms, no excitement and no mixers worth staying for. Tom Wall, who runs Whole Life Mastermind, a mastermind and support group for life insurance agents, wanted to build something better for the agents in his community.</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>1. Launched publicly with about three months to sell the room.
 2. Opened Sunday with registration and a mixer, so agents met before the first session.
@@ -2265,55 +2265,63 @@
 5. Built a speaker lineup of 11, hosted by Tom Wall, including Garrett Gunderson, Vince D'Addona and Kristin Andree.</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="H23" s="8" t="inlineStr">
         <is>
           <t>It went really well. 194 attendees came to the first Fast Start Forum, and Tom sold several spots in his first offer, along with a couple of places in the Inner Circle Mastermind we helped him design. The agents left having bonded over golf and jazz instead of another ballroom reception, and Tom brought the event back the next year.</t>
         </is>
       </c>
-      <c r="I23" s="7" t="inlineStr">
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>194 | Attendees at the first Fast Start Forum
 11 | Speakers on the program</t>
         </is>
       </c>
-      <c r="J23" s="7" t="inlineStr">
+      <c r="J23" s="8" t="inlineStr">
         <is>
           <t>Event design and management, the Inner Circle Mastermind offer design, venue at the Hilton Fort Lauderdale Marina, the speaker program, the Topgolf night and the VIP dinner at YOLO, production and on site execution.</t>
         </is>
       </c>
-      <c r="K23" s="7" t="inlineStr">
+      <c r="K23" s="8" t="inlineStr">
         <is>
           <t>Life insurance events usually start and end in a stuffy ballroom. Tom Wall of Whole Life Mastermind wanted something better for his agents. For the first Fast Start Forum, at the Hilton Fort Lauderdale Marina, we opened with a Sunday mixer, took Monday night to Topgolf and closed with a VIP dinner and live jazz at YOLO, around a program of 11 speakers. 194 attendees came, and Tom sold several spots in his first offer and in the Inner Circle Mastermind we helped him design.</t>
         </is>
       </c>
-      <c r="L23" s="7" t="inlineStr">
+      <c r="L23" s="8" t="inlineStr">
         <is>
           <t>How Fast Start Forum Took Life Insurance Agents Out of the Ballroom and Launched Tom Wall's Inner Circle Mastermind</t>
         </is>
       </c>
-      <c r="M23" s="7" t="inlineStr">
+      <c r="M23" s="8" t="inlineStr">
         <is>
           <t>Want an event your industry has never seen before?</t>
         </is>
       </c>
-      <c r="N23" s="7" t="inlineStr">
+      <c r="N23" s="8" t="inlineStr">
         <is>
           <t>Hilton Fort Lauderdale Marina, Fort Lauderdale, FL</t>
         </is>
       </c>
-      <c r="O23" s="7" t="inlineStr">
+      <c r="O23" s="8" t="inlineStr">
         <is>
           <t>194</t>
         </is>
       </c>
       <c r="P23" s="5" t="inlineStr"/>
       <c r="Q23" s="5" t="inlineStr"/>
-      <c r="R23" s="5" t="inlineStr"/>
+      <c r="R23" s="7" t="inlineStr">
+        <is>
+          <t>Link to come later</t>
+        </is>
+      </c>
       <c r="S23" s="5" t="inlineStr"/>
-      <c r="T23" s="5" t="inlineStr"/>
+      <c r="T23" s="7" t="inlineStr">
+        <is>
+          <t>Photos to come later</t>
+        </is>
+      </c>
       <c r="U23" s="5" t="inlineStr">
         <is>
-          <t>Iconic: first event, held in 2024, 194 attendees, Hilton Fort Lauderdale Marina. (Research had Feb 2 to 4, 2025; Iconic's answer stands.) Financial figures from the research kept out (house rules 1 and 2). "City council" in the right for answer read as a transcription error; check. "Brought the event back the next year" assumes the 2025 edition followed this one.</t>
+          <t>Approved by Iconic 2026-10-25 and built. First event, 2024, 194 attendees. Financial figures from the research kept out.</t>
         </is>
       </c>
       <c r="V23" s="5" t="inlineStr">
@@ -2321,12 +2329,12 @@
           <t>None (Iconic: no "what made it hard" for this event).</t>
         </is>
       </c>
-      <c r="W23" s="7" t="inlineStr">
+      <c r="W23" s="8" t="inlineStr">
         <is>
           <t>Any industry whose events tend to be standardized and stale, such as insurance or health and wellness, where events usually start and end in a ballroom. Fast Start Forum is a model for breaking that pattern.</t>
         </is>
       </c>
-      <c r="X23" s="7" t="inlineStr">
+      <c r="X23" s="8" t="inlineStr">
         <is>
           <t>Replace the ballroom mixer with an experience. A night at Topgolf gave agents something to do together, not just something to drink, and the bonding carried back into the sessions. Pick an activity your host loves, too: Tom is a big golfer, and it showed.</t>
         </is>

</xml_diff>

<commit_message>
Record the first Fast Start Forum 2025 answer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1614,7 +1614,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
+    <row r="13" ht="110" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Fast Start Forum 2025</t>
@@ -1630,9 +1630,9 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Tom Wall</t>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Tom Wall, Whole Life Mastermind</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1640,22 +1640,40 @@
           <t>Interviewing</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr"/>
-      <c r="G13" s="5" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Year one proved that life insurance agents wanted something better than a ballroom. For year two, Tom Wall wanted to go bigger and more premium, and to have sponsors carry more of the event.</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>1. Moved from the Hilton Fort Lauderdale Marina to the Hard Rock Hotel &amp; Casino, one of the most exciting venues in the country.
+2. Designed a room big enough for more attendees and a full sponsor hall, so sponsors could carry more of the event.
+3. Brought in Michael Phelps as a speaker.</t>
+        </is>
+      </c>
       <c r="H13" s="5" t="inlineStr"/>
       <c r="I13" s="5" t="inlineStr"/>
       <c r="J13" s="5" t="inlineStr"/>
       <c r="K13" s="5" t="inlineStr"/>
       <c r="L13" s="5" t="inlineStr"/>
       <c r="M13" s="5" t="inlineStr"/>
-      <c r="N13" s="5" t="inlineStr"/>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>Hard Rock Hotel &amp; Casino (Seminole Hard Rock Hollywood? confirm)</t>
+        </is>
+      </c>
       <c r="O13" s="5" t="inlineStr"/>
       <c r="P13" s="5" t="inlineStr"/>
       <c r="Q13" s="5" t="inlineStr"/>
       <c r="R13" s="5" t="inlineStr"/>
       <c r="S13" s="5" t="inlineStr"/>
       <c r="T13" s="5" t="inlineStr"/>
-      <c r="U13" s="5" t="inlineStr"/>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>The sponsor goal is written as "carry more of the event": no budget wording on the page. Confirm the venue (the Guitar Hotel in Hollywood, FL?). Month and attendance to come.</t>
+        </is>
+      </c>
       <c r="V13" s="5" t="n"/>
       <c r="W13" s="5" t="n"/>
       <c r="X13" s="5" t="n"/>

</xml_diff>

<commit_message>
Record the Fast Start Forum 2025 research without its financial figures
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1614,7 +1614,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="110" customHeight="1">
+    <row r="13" ht="220" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Fast Start Forum 2025</t>
@@ -1647,9 +1647,10 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>1. Moved from the Hilton Fort Lauderdale Marina to the Hard Rock Hotel &amp; Casino, one of the most exciting venues in the country.
-2. Designed a room big enough for more attendees and a full sponsor hall, so sponsors could carry more of the event.
-3. Brought in Michael Phelps as a speaker.</t>
+          <t>1. Moved from the Hilton Fort Lauderdale Marina to the Seminole Hard Rock Hotel &amp; Casino, the Guitar Hotel, one of the most exciting venues in the country.
+2. Designed a room big enough for more attendees and a full sponsor hall, and brought in a dedicated sponsor liaison. Three title sponsors and about 16 partners in all signed on.
+3. Brought in Michael Phelps as the keynote, alongside a program led by Tom Wall with speakers including Wade Pfau and Garrett Gunderson.
+4. Added a VIP track: a VIP cocktail hour and dinner, and a full VIP day to close the event.</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr"/>
@@ -1660,10 +1661,14 @@
       <c r="M13" s="5" t="inlineStr"/>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>Hard Rock Hotel &amp; Casino (Seminole Hard Rock Hollywood? confirm)</t>
-        </is>
-      </c>
-      <c r="O13" s="5" t="inlineStr"/>
+          <t>Seminole Hard Rock Hotel &amp; Casino Hollywood (the Guitar Hotel), Hollywood, FL</t>
+        </is>
+      </c>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>473</t>
+        </is>
+      </c>
       <c r="P13" s="5" t="inlineStr"/>
       <c r="Q13" s="5" t="inlineStr"/>
       <c r="R13" s="5" t="inlineStr"/>
@@ -1671,10 +1676,14 @@
       <c r="T13" s="5" t="inlineStr"/>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>The sponsor goal is written as "carry more of the event": no budget wording on the page. Confirm the venue (the Guitar Hotel in Hollywood, FL?). Month and attendance to come.</t>
-        </is>
-      </c>
-      <c r="V13" s="5" t="n"/>
+          <t>Held January 19 to 22, 2026, but listed on the grid as 2025: which year should the page show? Financial figures from the research kept out (house rules 1 and 2; public repo). Sponsor names: OK to name the title sponsors? Still to answer: how the sponsor hall landed, how it went.</t>
+        </is>
+      </c>
+      <c r="V13" s="7" t="inlineStr">
+        <is>
+          <t>The original dates landed on a school vacation week, and the hotel's only other window was January 19 to 22, with very few rooms on the Sunday. We moved the event, then negotiated 50 more Sunday rooms so attendees could arrive the night before.</t>
+        </is>
+      </c>
       <c r="W13" s="5" t="n"/>
       <c r="X13" s="5" t="n"/>
     </row>

</xml_diff>

<commit_message>
Correct the Fast Start Forum years and draft the 2026 edition
The first Fast Start Forum was held in February 2025, so its page now
reads Fast Start Forum 2025; its live URL stays fast-start-forum-2024.
The second edition, held January 2026, becomes fast-start-forum-2026 in
the index, and its interview row is drafted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1614,20 +1614,20 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="220" customHeight="1">
+    <row r="13" ht="300" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Fast Start Forum 2025</t>
+          <t>Fast Start Forum 2026</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>fast-start-forum-2025</t>
+          <t>fast-start-forum-2026</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>January 2026</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -1648,17 +1648,46 @@
       <c r="G13" s="7" t="inlineStr">
         <is>
           <t>1. Moved from the Hilton Fort Lauderdale Marina to the Seminole Hard Rock Hotel &amp; Casino, the Guitar Hotel, one of the most exciting venues in the country.
-2. Designed a room big enough for more attendees and a full sponsor hall, and brought in a dedicated sponsor liaison. Three title sponsors and about 16 partners in all signed on.
-3. Brought in Michael Phelps as the keynote, alongside a program led by Tom Wall with speakers including Wade Pfau and Garrett Gunderson.
-4. Added a VIP track: a VIP cocktail hour and dinner, and a full VIP day to close the event.</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr"/>
-      <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr"/>
-      <c r="K13" s="5" t="inlineStr"/>
-      <c r="L13" s="5" t="inlineStr"/>
-      <c r="M13" s="5" t="inlineStr"/>
+2. Designed a room big enough for more attendees and a full sponsor hall, and brought in a dedicated sponsor liaison. Title sponsors Madan+, Wealth Building Cornerstones and OneAmerica led about 16 partners in all.
+3. Brought in Olympic legend Michael Phelps as the keynote, alongside a program led by Tom Wall with speakers including Wade Pfau and Garrett Gunderson.
+4. Built Tom a custom booth for his Inner Circle Mastermind on the sponsor floor.
+5. Added a VIP track: a VIP cocktail hour and dinner, and a full VIP day to close the event.
+6. Threw an on the water afterparty, and put Tom's logo on the Guitar Hotel itself for everyone to see.</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>It went well. 473 people came, more than double the 194 at the first Fast Start Forum, and everyone loved the chance to learn from an Olympic legend.
+Tom sold more of his Inner Circle Mastermind than the year before, from the custom booth we set up for him. And the attendees loved the on the water afterparty, with Tom's logo lit up on the Guitar for everyone to see.</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>473 | Attendees, up from 194 in year one
+3 | Title sponsors
+1 | Olympic legend on the main stage</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>Venue move to the Seminole Hard Rock, room and sponsor hall design, sponsor liaison, the Michael Phelps keynote and speaker program, Tom's Inner Circle Mastermind booth, the VIP track, the on the water afterparty and the logo on the Guitar, production and on site execution.</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>For year two of Fast Start Forum, Tom Wall of Whole Life Mastermind wanted to go bigger and more premium, with sponsors carrying more of the event. We moved it to the Seminole Hard Rock, the Guitar Hotel, built a room with a full sponsor hall led by title sponsors Madan+, Wealth Building Cornerstones and OneAmerica, and brought in Michael Phelps as the keynote. Tom sold more of his Inner Circle Mastermind from a custom booth, the afterparty went out on the water with Tom's logo on the Guitar, and attendance grew from 194 to 473.</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>How Fast Start Forum More Than Doubled to 473 Attendees, With Michael Phelps and Its Own Logo on the Guitar Hotel</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>Want your event's second year to make the first look small?</t>
+        </is>
+      </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
           <t>Seminole Hard Rock Hotel &amp; Casino Hollywood (the Guitar Hotel), Hollywood, FL</t>
@@ -1676,7 +1705,7 @@
       <c r="T13" s="5" t="inlineStr"/>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>Held January 19 to 22, 2026, but listed on the grid as 2025: which year should the page show? Financial figures from the research kept out (house rules 1 and 2; public repo). Sponsor names: OK to name the title sponsors? Still to answer: how the sponsor hall landed, how it went.</t>
+          <t>Held January 19 to 22, 2026. Financial figures from the research kept out (house rules 1 and 2). Title sponsors named (Iconic OK). Right for and Steal This drafted, not yet answered.</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
@@ -1684,8 +1713,16 @@
           <t>The original dates landed on a school vacation week, and the hotel's only other window was January 19 to 22, with very few rooms on the Sunday. We moved the event, then negotiated 50 more Sunday rooms so attendees could arrive the night before.</t>
         </is>
       </c>
-      <c r="W13" s="5" t="n"/>
-      <c r="X13" s="5" t="n"/>
+      <c r="W13" s="7" t="inlineStr">
+        <is>
+          <t>Membership and mastermind communities ready to step up from a first event to a premium, sponsor backed one, especially in industries whose events usually start and end in a ballroom.</t>
+        </is>
+      </c>
+      <c r="X13" s="7" t="inlineStr">
+        <is>
+          <t>Put the client's name on the landmark. Tom's logo on the Guitar Hotel turned a venue into a moment, and every photo from the afterparty carried his brand.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -2255,7 +2292,7 @@
     <row r="23" ht="260" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Fast Start Forum 2024</t>
+          <t>Fast Start Forum 2025 (URL fast-start-forum-2024)</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -2265,7 +2302,7 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>February 2025</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Build Fast Start Forum 2026
Add the approved Fast Start Forum 2026 row as a case study: the move to
the Seminole Hard Rock, title sponsors, the Michael Phelps keynote, Tom's
Inner Circle booth and the afterparty with his logo on the Guitar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1630,22 +1630,22 @@
           <t>January 2026</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>Tom Wall, Whole Life Mastermind</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>Year one proved that life insurance agents wanted something better than a ballroom. For year two, Tom Wall wanted to go bigger and more premium, and to have sponsors carry more of the event.</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>1. Moved from the Hilton Fort Lauderdale Marina to the Seminole Hard Rock Hotel &amp; Casino, the Guitar Hotel, one of the most exciting venues in the country.
 2. Designed a room big enough for more attendees and a full sponsor hall, and brought in a dedicated sponsor liaison. Title sponsors Madan+, Wealth Building Cornerstones and OneAmerica led about 16 partners in all.
@@ -1655,70 +1655,82 @@
 6. Threw an on the water afterparty, and put Tom's logo on the Guitar Hotel itself for everyone to see.</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>It went well. 473 people came, more than double the 194 at the first Fast Start Forum, and everyone loved the chance to learn from an Olympic legend.
 Tom sold more of his Inner Circle Mastermind than the year before, from the custom booth we set up for him. And the attendees loved the on the water afterparty, with Tom's logo lit up on the Guitar for everyone to see.</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr">
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>473 | Attendees, up from 194 in year one
 3 | Title sponsors
 1 | Olympic legend on the main stage</t>
         </is>
       </c>
-      <c r="J13" s="7" t="inlineStr">
+      <c r="J13" s="8" t="inlineStr">
         <is>
           <t>Venue move to the Seminole Hard Rock, room and sponsor hall design, sponsor liaison, the Michael Phelps keynote and speaker program, Tom's Inner Circle Mastermind booth, the VIP track, the on the water afterparty and the logo on the Guitar, production and on site execution.</t>
         </is>
       </c>
-      <c r="K13" s="7" t="inlineStr">
+      <c r="K13" s="8" t="inlineStr">
         <is>
           <t>For year two of Fast Start Forum, Tom Wall of Whole Life Mastermind wanted to go bigger and more premium, with sponsors carrying more of the event. We moved it to the Seminole Hard Rock, the Guitar Hotel, built a room with a full sponsor hall led by title sponsors Madan+, Wealth Building Cornerstones and OneAmerica, and brought in Michael Phelps as the keynote. Tom sold more of his Inner Circle Mastermind from a custom booth, the afterparty went out on the water with Tom's logo on the Guitar, and attendance grew from 194 to 473.</t>
         </is>
       </c>
-      <c r="L13" s="7" t="inlineStr">
+      <c r="L13" s="8" t="inlineStr">
         <is>
           <t>How Fast Start Forum More Than Doubled to 473 Attendees, With Michael Phelps and Its Own Logo on the Guitar Hotel</t>
         </is>
       </c>
-      <c r="M13" s="7" t="inlineStr">
+      <c r="M13" s="8" t="inlineStr">
         <is>
           <t>Want your event's second year to make the first look small?</t>
         </is>
       </c>
-      <c r="N13" s="7" t="inlineStr">
+      <c r="N13" s="8" t="inlineStr">
         <is>
           <t>Seminole Hard Rock Hotel &amp; Casino Hollywood (the Guitar Hotel), Hollywood, FL</t>
         </is>
       </c>
-      <c r="O13" s="7" t="inlineStr">
+      <c r="O13" s="8" t="inlineStr">
         <is>
           <t>473</t>
         </is>
       </c>
-      <c r="P13" s="5" t="inlineStr"/>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="Q13" s="5" t="inlineStr"/>
-      <c r="R13" s="5" t="inlineStr"/>
+      <c r="R13" s="7" t="inlineStr">
+        <is>
+          <t>Link to come later</t>
+        </is>
+      </c>
       <c r="S13" s="5" t="inlineStr"/>
-      <c r="T13" s="5" t="inlineStr"/>
+      <c r="T13" s="7" t="inlineStr">
+        <is>
+          <t>Photos to come later</t>
+        </is>
+      </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>Held January 19 to 22, 2026. Financial figures from the research kept out (house rules 1 and 2). Title sponsors named (Iconic OK). Right for and Steal This drafted, not yet answered.</t>
-        </is>
-      </c>
-      <c r="V13" s="7" t="inlineStr">
+          <t>Approved by Iconic 2026-10-25 and built. Held January 19 to 22, 2026. Financial figures from the research kept out. Title sponsors named with Iconic OK.</t>
+        </is>
+      </c>
+      <c r="V13" s="8" t="inlineStr">
         <is>
           <t>The original dates landed on a school vacation week, and the hotel's only other window was January 19 to 22, with very few rooms on the Sunday. We moved the event, then negotiated 50 more Sunday rooms so attendees could arrive the night before.</t>
         </is>
       </c>
-      <c r="W13" s="7" t="inlineStr">
+      <c r="W13" s="8" t="inlineStr">
         <is>
           <t>Membership and mastermind communities ready to step up from a first event to a premium, sponsor backed one, especially in industries whose events usually start and end in a ballroom.</t>
         </is>
       </c>
-      <c r="X13" s="7" t="inlineStr">
+      <c r="X13" s="8" t="inlineStr">
         <is>
           <t>Put the client's name on the landmark. Tom's logo on the Guitar Hotel turned a venue into a moment, and every photo from the afterparty carried his brand.</t>
         </is>

</xml_diff>

<commit_message>
Record The Sales Summit research without financial or billing details
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1004,14 +1004,14 @@
           <t>the-sales-summit</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Jeremy Miner</t>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Jeremy Miner, 7th Level</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1027,14 +1027,22 @@
       <c r="K5" s="5" t="inlineStr"/>
       <c r="L5" s="5" t="inlineStr"/>
       <c r="M5" s="5" t="inlineStr"/>
-      <c r="N5" s="5" t="inlineStr"/>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>Irving Convention Center at Las Colinas, Irving, TX</t>
+        </is>
+      </c>
       <c r="O5" s="5" t="inlineStr"/>
       <c r="P5" s="5" t="inlineStr"/>
       <c r="Q5" s="5" t="inlineStr"/>
       <c r="R5" s="5" t="inlineStr"/>
       <c r="S5" s="5" t="inlineStr"/>
       <c r="T5" s="5" t="inlineStr"/>
-      <c r="U5" s="5" t="inlineStr"/>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>Research kept without financial figures or the open billing matters. Final attendance not found (653 registered July 6). Back end sales are client revenue (house rule 1).</t>
+        </is>
+      </c>
       <c r="V5" s="5" t="n"/>
       <c r="W5" s="5" t="n"/>
       <c r="X5" s="5" t="n"/>

</xml_diff>

<commit_message>
Record the first Sales Summit answer and draft its copy
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -993,7 +993,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
+    <row r="5" ht="220" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>The Sales Summit</t>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Jeremy Miner, 7th Level</t>
+          <t>Jeremy Miner, CEO, 7th Level</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1019,8 +1019,20 @@
           <t>Interviewing</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Jeremy Miner was riding a massive wave of authority and impact, and his team at 7th Level wanted to grow it until it filled stadiums. The Sales Summit was the first step: the largest event they had ever put on. Until then, most of their events had been virtual. Jeremy wanted this one large and loud.</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>1. Took the Irving Convention Center at Las Colinas, outside Dallas, with the Westin next door so attendees could walk to every session.
+2. Opened with a gala on the outdoor terrace the night before day one.
+3. Built a three day program around Jeremy, Anthony Vizzari and Michael Bernoff, with live call reviews from the stage, guest panels and sponsor spotlights.
+4. Went large and loud with a Rolex giveaway and a car giveaway, built around a skill based challenge.
+5. Gave Elite attendees their own track: a private workshop and an offsite dinner at the Constellation Club.</t>
+        </is>
+      </c>
       <c r="H5" s="5" t="inlineStr"/>
       <c r="I5" s="5" t="inlineStr"/>
       <c r="J5" s="5" t="inlineStr"/>
@@ -1040,10 +1052,14 @@
       <c r="T5" s="5" t="inlineStr"/>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>Research kept without financial figures or the open billing matters. Final attendance not found (653 registered July 6). Back end sales are client revenue (house rule 1).</t>
-        </is>
-      </c>
-      <c r="V5" s="5" t="n"/>
+          <t>Never mention: hotel block pickup, the billing dispute, one on site detail (Iconic). Car value ($100,000): publish? Final attendance not found (653 registered July 6). Back end sales are client revenue (house rule 1).</t>
+        </is>
+      </c>
+      <c r="V5" s="7" t="inlineStr">
+        <is>
+          <t>A competing event landed on the same weekend, and the public launch moved to April 20, leaving about two months to sell the room. The fire marshal declined the permit at first; it was approved on July 7, three days before the doors opened.</t>
+        </is>
+      </c>
       <c r="W5" s="5" t="n"/>
       <c r="X5" s="5" t="n"/>
     </row>

</xml_diff>

<commit_message>
Draft the rest of The Sales Summit row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -993,7 +993,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="220" customHeight="1">
+    <row r="5" ht="300" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>The Sales Summit</t>
@@ -1029,22 +1029,53 @@
           <t>1. Took the Irving Convention Center at Las Colinas, outside Dallas, with the Westin next door so attendees could walk to every session.
 2. Opened with a gala on the outdoor terrace the night before day one.
 3. Built a three day program around Jeremy, Anthony Vizzari and Michael Bernoff, with live call reviews from the stage, guest panels and sponsor spotlights.
-4. Went large and loud with a Rolex giveaway and a car giveaway, built around a skill based challenge.
+4. Went large and loud: a $10,000 Rolex giveaway and a $100,000 car, a 2023 Mercedes-AMG C 63, given away from the stage, built around a skill based challenge.
 5. Gave Elite attendees their own track: a private workshop and an offsite dinner at the Constellation Club.</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="5" t="inlineStr"/>
-      <c r="K5" s="5" t="inlineStr"/>
-      <c r="L5" s="5" t="inlineStr"/>
-      <c r="M5" s="5" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>The room loved it. There were lines out the door every single day, and locals passing by came in to see what was happening. People stayed for hours, from the first session to the last, to level up their sales skills.
+Companies sent whole teams, some of 10 to 12 people, paid for by the business. 700 people attended, and the Sales Summit became the first step toward the stadiums Jeremy is building toward.</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>700 | Attendees
+3 | Days, with lines out the door every one
+10 to 12 | Person sales teams sent by their companies</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Venue and hotel, the opening gala, the three day program and speakers, the Rolex and car giveaways, the Elite track and dinner, sponsor spotlights, production, on site execution and post event content including recordings, storymonials and a trailer.</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Jeremy Miner, CEO of 7th Level, wanted to grow his impact until it filled stadiums, and the Sales Summit was the first step: the largest event 7th Level had ever put on, after years of mostly virtual events. We took the Irving Convention Center at Las Colinas, opened with a gala on the terrace and built three days around live call reviews from the stage, a Rolex giveaway and a 2023 Mercedes-AMG C 63 given away from the stage. 700 people attended, with lines out the door every day.</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>How 7th Level Drew 700 to Its Largest Event Yet, the First Step Toward Filling Stadiums</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>Want your first big live event to feel like a stadium tour?</t>
+        </is>
+      </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
           <t>Irving Convention Center at Las Colinas, Irving, TX</t>
         </is>
       </c>
-      <c r="O5" s="5" t="inlineStr"/>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
       <c r="P5" s="5" t="inlineStr"/>
       <c r="Q5" s="5" t="inlineStr"/>
       <c r="R5" s="5" t="inlineStr"/>
@@ -1052,7 +1083,7 @@
       <c r="T5" s="5" t="inlineStr"/>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>Never mention: hotel block pickup, the billing dispute, one on site detail (Iconic). Car value ($100,000): publish? Final attendance not found (653 registered July 6). Back end sales are client revenue (house rule 1).</t>
+          <t>Never mention: hotel block pickup, the billing dispute, one on site detail (Iconic). 700 attended per Iconic (653 registered July 6). Car value and model OK to publish. Back end sales are client revenue (house rule 1).</t>
         </is>
       </c>
       <c r="V5" s="7" t="inlineStr">
@@ -1060,8 +1091,16 @@
           <t>A competing event landed on the same weekend, and the public launch moved to April 20, leaving about two months to sell the room. The fire marshal declined the permit at first; it was approved on July 7, three days before the doors opened.</t>
         </is>
       </c>
-      <c r="W5" s="5" t="n"/>
-      <c r="X5" s="5" t="n"/>
+      <c r="W5" s="7" t="inlineStr">
+        <is>
+          <t>Experts and brands with a fast growing audience who have run mostly virtual events and are ready for a large, loud live one, and companies that want to send their whole sales team to level up together.</t>
+        </is>
+      </c>
+      <c r="X5" s="7" t="inlineStr">
+        <is>
+          <t>Use the giveaway to send people to your sponsors. A $10,000 Rolex giveaway drove a huge turnout at the sponsor booths. If that is what it costs to engage your sponsors and bring them back year over year, you make the money back on sponsorship and then some.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Build The Sales Summit
Add the approved Sales Summit row as a case study: 7th Level's largest
event to date, at the Irving Convention Center at Las Colinas, with 700
attendees, the Rolex and car giveaways and the Rolex sponsor Steal This.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1004,27 +1004,27 @@
           <t>the-sales-summit</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>July 2026</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Jeremy Miner, CEO, 7th Level</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Jeremy Miner was riding a massive wave of authority and impact, and his team at 7th Level wanted to grow it until it filled stadiums. The Sales Summit was the first step: the largest event they had ever put on. Until then, most of their events had been virtual. Jeremy wanted this one large and loud.</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>1. Took the Irving Convention Center at Las Colinas, outside Dallas, with the Westin next door so attendees could walk to every session.
 2. Opened with a gala on the outdoor terrace the night before day one.
@@ -1033,70 +1033,82 @@
 5. Gave Elite attendees their own track: a private workshop and an offsite dinner at the Constellation Club.</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>The room loved it. There were lines out the door every single day, and locals passing by came in to see what was happening. People stayed for hours, from the first session to the last, to level up their sales skills.
 Companies sent whole teams, some of 10 to 12 people, paid for by the business. 700 people attended, and the Sales Summit became the first step toward the stadiums Jeremy is building toward.</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>700 | Attendees
 3 | Days, with lines out the door every one
 10 to 12 | Person sales teams sent by their companies</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>Venue and hotel, the opening gala, the three day program and speakers, the Rolex and car giveaways, the Elite track and dinner, sponsor spotlights, production, on site execution and post event content including recordings, storymonials and a trailer.</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
         <is>
           <t>Jeremy Miner, CEO of 7th Level, wanted to grow his impact until it filled stadiums, and the Sales Summit was the first step: the largest event 7th Level had ever put on, after years of mostly virtual events. We took the Irving Convention Center at Las Colinas, opened with a gala on the terrace and built three days around live call reviews from the stage, a Rolex giveaway and a 2023 Mercedes-AMG C 63 given away from the stage. 700 people attended, with lines out the door every day.</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr">
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>How 7th Level Drew 700 to Its Largest Event Yet, the First Step Toward Filling Stadiums</t>
         </is>
       </c>
-      <c r="M5" s="7" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Want your first big live event to feel like a stadium tour?</t>
         </is>
       </c>
-      <c r="N5" s="7" t="inlineStr">
+      <c r="N5" s="8" t="inlineStr">
         <is>
           <t>Irving Convention Center at Las Colinas, Irving, TX</t>
         </is>
       </c>
-      <c r="O5" s="7" t="inlineStr">
+      <c r="O5" s="8" t="inlineStr">
         <is>
           <t>700</t>
         </is>
       </c>
-      <c r="P5" s="5" t="inlineStr"/>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="Q5" s="5" t="inlineStr"/>
-      <c r="R5" s="5" t="inlineStr"/>
+      <c r="R5" s="7" t="inlineStr">
+        <is>
+          <t>Trailer delivered; link to come</t>
+        </is>
+      </c>
       <c r="S5" s="5" t="inlineStr"/>
-      <c r="T5" s="5" t="inlineStr"/>
+      <c r="T5" s="7" t="inlineStr">
+        <is>
+          <t>Photos to come later</t>
+        </is>
+      </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>Never mention: hotel block pickup, the billing dispute, one on site detail (Iconic). 700 attended per Iconic (653 registered July 6). Car value and model OK to publish. Back end sales are client revenue (house rule 1).</t>
-        </is>
-      </c>
-      <c r="V5" s="7" t="inlineStr">
+          <t>Approved by Iconic 2026-10-25 and built. Never mention: hotel block pickup, the billing dispute, one on site detail. 700 attended per Iconic.</t>
+        </is>
+      </c>
+      <c r="V5" s="8" t="inlineStr">
         <is>
           <t>A competing event landed on the same weekend, and the public launch moved to April 20, leaving about two months to sell the room. The fire marshal declined the permit at first; it was approved on July 7, three days before the doors opened.</t>
         </is>
       </c>
-      <c r="W5" s="7" t="inlineStr">
+      <c r="W5" s="8" t="inlineStr">
         <is>
           <t>Experts and brands with a fast growing audience who have run mostly virtual events and are ready for a large, loud live one, and companies that want to send their whole sales team to level up together.</t>
         </is>
       </c>
-      <c r="X5" s="7" t="inlineStr">
+      <c r="X5" s="8" t="inlineStr">
         <is>
           <t>Use the giveaway to send people to your sponsors. A $10,000 Rolex giveaway drove a huge turnout at the sponsor booths. If that is what it costs to engage your sponsors and bring them back year over year, you make the money back on sponsorship and then some.</t>
         </is>

</xml_diff>

<commit_message>
Publish Net Rev Summit 2026 with its gaps flagged
At Iconic's request the parked Net Rev page goes live from the Fathom call
summaries: the run of show, the virtual ticket and livestream with 7th
Level, attendee hospitality and the hotel overage cut from $16,000 to
$1,067. The interview sheet lists what it still needs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -813,7 +813,7 @@
       <c r="W2" s="5" t="n"/>
       <c r="X2" s="5" t="n"/>
     </row>
-    <row r="3" ht="18" customHeight="1">
+    <row r="3" ht="260" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Net Rev Summit 2026</t>
@@ -824,37 +824,80 @@
           <t>net-rev-summit-2026</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>May 2026</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Ambro Dipilato</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr"/>
-      <c r="J3" s="5" t="inlineStr"/>
-      <c r="K3" s="5" t="inlineStr"/>
-      <c r="L3" s="5" t="inlineStr"/>
-      <c r="M3" s="5" t="inlineStr"/>
-      <c r="N3" s="5" t="inlineStr">
-        <is>
-          <t>Marana, AZ</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="inlineStr"/>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Net Rev wanted its summit to reach beyond the room: an in person weekend at the Ritz-Carlton Dove Mountain, plus a virtual audience far larger than the ballroom could hold.</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>1. Restructured the run of show for narrative flow, moving the event's "why" talk to Sunday morning and adding a Sunday afternoon roundtable.
+2. Added a virtual ticket and a livestream, hosted with 7th Level, so the stage reached people who could not be in Arizona.
+3. Put the full catering minimum to work for attendees: a continental breakfast and Ritz-Carlton gift cards.
+4. Redesigned the LED wall graphics to match the brand.</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>The weekend ran at the Ritz-Carlton Dove Mountain as planned, and the full set of event content was delivered after the show.</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>$14.9K | Hotel overage negotiated away</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>Run of show and session order, built for the weekend's narrative.; A virtual ticket and livestream, hosted with 7th Level.; Catering, a continental breakfast and Ritz-Carlton gift cards for attendees.; LED wall graphics redesigned to match the brand.; The hotel overage, cut from $16,000 to $1,067.; Event content delivered after the show.</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Net Rev Summit 2026 brought its community to the Ritz-Carlton Dove Mountain in Marana, Arizona, and opened the stage to a virtual audience as well. We restructured the run of show so the story built across the weekend, added a virtual ticket and livestream hosted with 7th Level, turned the full catering minimum into extras for attendees, and after the event negotiated a $16,000 hotel overage down to $1,067.</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>How Net Rev Summit 2026 Took Its Ritz-Carlton Stage Online</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>Want your summit to reach far beyond the room?</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>Ritz-Carlton Dove Mountain, Marana, AZ</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr">
+        <is>
+          <t>Needed</t>
+        </is>
+      </c>
       <c r="P3" s="5" t="inlineStr"/>
-      <c r="Q3" s="5" t="inlineStr"/>
+      <c r="Q3" s="7" t="inlineStr">
+        <is>
+          <t>$14,933</t>
+        </is>
+      </c>
       <c r="R3" s="5" t="inlineStr"/>
       <c r="S3" s="5" t="inlineStr">
         <is>
@@ -864,10 +907,14 @@
       <c r="T3" s="5" t="inlineStr"/>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>Parked 2026-10-20 until Iconic sends the YouTube testimonial links. Leads in the notes file (Fathom summaries).</t>
-        </is>
-      </c>
-      <c r="V3" s="5" t="n"/>
+          <t>PUBLISHED WITH GAPS at Iconic's request (2026-10-25), drafted from Fathom call summaries without an interview. Needs: Iconic's review of every yellow cell, the client's goal in Iconic's words, final attendance (in person and virtual), Ambro's title and company, how it went, right for, Steal This, photos, aftermovie, the video testimonial YouTube links.</t>
+        </is>
+      </c>
+      <c r="V3" s="7" t="inlineStr">
+        <is>
+          <t>A $16,000 hotel overage arrived after the event. We negotiated it down to $1,067, saving the client $14,933.</t>
+        </is>
+      </c>
       <c r="W3" s="5" t="n"/>
       <c r="X3" s="5" t="n"/>
     </row>

</xml_diff>

<commit_message>
Record the Hell Yes Live 2026 research and draft its row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1858,10 +1858,10 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
+    <row r="14" ht="300" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Hell Yes Live</t>
+          <t>Hell Yes Live 2026</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -1869,14 +1869,14 @@
           <t>hell-yes-live</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Becca Pike</t>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>July 2026</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Becca Pike, Hell Yes Coaching</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1884,25 +1884,97 @@
           <t>Interviewing</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr"/>
-      <c r="G14" s="5" t="inlineStr"/>
-      <c r="H14" s="5" t="inlineStr"/>
-      <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="5" t="inlineStr"/>
-      <c r="K14" s="5" t="inlineStr"/>
-      <c r="L14" s="5" t="inlineStr"/>
-      <c r="M14" s="5" t="inlineStr"/>
-      <c r="N14" s="5" t="inlineStr"/>
-      <c r="O14" s="5" t="inlineStr"/>
-      <c r="P14" s="5" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Becca Pike runs Hell Yes Coaching, which sells coaching and masterminds including Scale to Seven and The Circle. For her second live event she wanted something bigger, a room that worked as a selling room, and she hired Icon as her event coach to get there.
+Tickets sold slowly for months in a regional market, the fire department capped the room, and a target sponsor dropped out.</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>1. Reframed the event around one promise: from overextended and underpaid to Hell Yes CEO.
+2. Merged everything into one playbook and one tracker, to protect Becca's time.
+3. Put GA and VIP on one checkout page.
+4. Pivoted sales in June: plus-one and gifted tickets, a local campaign that excluded existing leads, and personal calls to people who abandoned checkout.
+5. Led the on stage offer with the transformation, and kept it to a single public offer.</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>The room was packed, 99 people on site, and Becca's opening drew praise. Sign-ups from the stage were strong, and 42 tickets for next year sold within days of the event. The next Hell Yes Live moves to the larger Manchester Reserve.</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>99 | Attendees on site
+42 | Tickets for next year sold within days
+5 of 6 | Scholarship seats became high ticket clients</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>Event coaching and direction: the vision brief, promise and transformation copy, playbook and tracker, funnel and checkout changes, ad review, sales coaching, run of show, pitch and slides review, biweekly calls and the debrief.</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>Becca Pike of Hell Yes Coaching wanted her second live event to be bigger and to work as a selling room, and she hired Icon as her event coach. With months of slow sales, a capped room and a key team member gone 72 hours before she was needed, we reframed the event around one promise, rebuilt the sales plan in June and coached the offer on stage. 99 people packed the room, sign-ups from the stage were strong, and 42 tickets for next year sold within days.</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>How Hell Yes Live Packed the Room and Sold 42 Seats for Next Year Within Days</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>Want an event coach in your corner?</t>
+        </is>
+      </c>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>The Manchester Hotel, Lexington, KY</t>
+        </is>
+      </c>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="P14" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="Q14" s="5" t="inlineStr"/>
       <c r="R14" s="5" t="inlineStr"/>
-      <c r="S14" s="5" t="inlineStr"/>
+      <c r="S14" s="7" t="inlineStr">
+        <is>
+          <t>Stage thank-you video exists (sent as a file, not hosted). Needs a YouTube link.</t>
+        </is>
+      </c>
       <c r="T14" s="5" t="inlineStr"/>
-      <c r="U14" s="5" t="inlineStr"/>
-      <c r="V14" s="5" t="n"/>
-      <c r="W14" s="5" t="n"/>
-      <c r="X14" s="5" t="n"/>
+      <c r="U14" s="5" t="inlineStr">
+        <is>
+          <t>Iconic coached and directed remotely, not on site production: page copy must not claim on site execution. Becca's stage quotes need written permission to publish (house rule 4). Left out: a private campaign message, a named staff member, remarks about the 2025 edition. 'Within days of the event' = by July 20. Title not found.</t>
+        </is>
+      </c>
+      <c r="V14" s="7" t="inlineStr">
+        <is>
+          <t>Mid-build, the team member who held every moving part for Becca left without warning, and she had about 72 hours to replace her. She called Icon, who gave her love, reassurance and a plan. A replacement stepped in, and the show went on.
+In June, a full week passed with zero ticket sales. The June pivots, from gifted tickets to personal calls on abandoned checkouts, brought the room back.</t>
+        </is>
+      </c>
+      <c r="W14" s="7" t="inlineStr">
+        <is>
+          <t>Coaches and hosts whose live event is the front door to a high ticket offer, and who have a small team that needs structure.</t>
+        </is>
+      </c>
+      <c r="X14" s="7" t="inlineStr">
+        <is>
+          <t>Give a handful of scholarship tickets to qualified owners. Hell Yes Live gave out 6, and 5 became high ticket clients.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Build Hell Yes Live 2026, an EPIC Consulting case study
Add Hell Yes Live 2026 as a case study for Iconic's EPIC Consulting offer:
Icon coached Becca Pike's team remotely. A page can now replace the line
beside What We Did, so this one does not claim on site production.
Becca's stage quotes are published with Iconic's OK; her stage video is
to come.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1869,28 +1869,28 @@
           <t>hell-yes-live</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>July 2026</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Becca Pike, Hell Yes Coaching</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Becca Pike runs Hell Yes Coaching, which sells coaching and masterminds including Scale to Seven and The Circle. For her second live event she wanted something bigger, a room that worked as a selling room, and she hired Icon as her event coach to get there.
 Tickets sold slowly for months in a regional market, the fire department capped the room, and a target sponsor dropped out.</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
         <is>
           <t>1. Reframed the event around one promise: from overextended and underpaid to Hell Yes CEO.
 2. Merged everything into one playbook and one tracker, to protect Becca's time.
@@ -1899,49 +1899,49 @@
 5. Led the on stage offer with the transformation, and kept it to a single public offer.</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>The room was packed, 99 people on site, and Becca's opening drew praise. Sign-ups from the stage were strong, and 42 tickets for next year sold within days of the event. The next Hell Yes Live moves to the larger Manchester Reserve.</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
         <is>
           <t>99 | Attendees on site
 42 | Tickets for next year sold within days
 5 of 6 | Scholarship seats became high ticket clients</t>
         </is>
       </c>
-      <c r="J14" s="7" t="inlineStr">
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>Event coaching and direction: the vision brief, promise and transformation copy, playbook and tracker, funnel and checkout changes, ad review, sales coaching, run of show, pitch and slides review, biweekly calls and the debrief.</t>
         </is>
       </c>
-      <c r="K14" s="7" t="inlineStr">
+      <c r="K14" s="8" t="inlineStr">
         <is>
           <t>Becca Pike of Hell Yes Coaching wanted her second live event to be bigger and to work as a selling room, and she hired Icon as her event coach. With months of slow sales, a capped room and a key team member gone 72 hours before she was needed, we reframed the event around one promise, rebuilt the sales plan in June and coached the offer on stage. 99 people packed the room, sign-ups from the stage were strong, and 42 tickets for next year sold within days.</t>
         </is>
       </c>
-      <c r="L14" s="7" t="inlineStr">
+      <c r="L14" s="8" t="inlineStr">
         <is>
           <t>How Hell Yes Live Packed the Room and Sold 42 Seats for Next Year Within Days</t>
         </is>
       </c>
-      <c r="M14" s="7" t="inlineStr">
+      <c r="M14" s="8" t="inlineStr">
         <is>
           <t>Want an event coach in your corner?</t>
         </is>
       </c>
-      <c r="N14" s="7" t="inlineStr">
+      <c r="N14" s="8" t="inlineStr">
         <is>
           <t>The Manchester Hotel, Lexington, KY</t>
         </is>
       </c>
-      <c r="O14" s="7" t="inlineStr">
+      <c r="O14" s="8" t="inlineStr">
         <is>
           <t>99</t>
         </is>
       </c>
-      <c r="P14" s="7" t="inlineStr">
+      <c r="P14" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -1950,27 +1950,31 @@
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="7" t="inlineStr">
         <is>
-          <t>Stage thank-you video exists (sent as a file, not hosted). Needs a YouTube link.</t>
-        </is>
-      </c>
-      <c r="T14" s="5" t="inlineStr"/>
+          <t>Stage video: Iconic to upload to YouTube later</t>
+        </is>
+      </c>
+      <c r="T14" s="7" t="inlineStr">
+        <is>
+          <t>Photos to come later</t>
+        </is>
+      </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>Iconic coached and directed remotely, not on site production: page copy must not claim on site execution. Becca's stage quotes need written permission to publish (house rule 4). Left out: a private campaign message, a named staff member, remarks about the 2025 edition. 'Within days of the event' = by July 20. Title not found.</t>
-        </is>
-      </c>
-      <c r="V14" s="7" t="inlineStr">
+          <t>Approved by Iconic 2026-10-25 and built. An EPIC Consulting engagement (event coaching, remote), not production. Becca's stage quotes published with Iconic's OK (said publicly from the stage). Stage video link to come.</t>
+        </is>
+      </c>
+      <c r="V14" s="8" t="inlineStr">
         <is>
           <t>Mid-build, the team member who held every moving part for Becca left without warning, and she had about 72 hours to replace her. She called Icon, who gave her love, reassurance and a plan. A replacement stepped in, and the show went on.
 In June, a full week passed with zero ticket sales. The June pivots, from gifted tickets to personal calls on abandoned checkouts, brought the room back.</t>
         </is>
       </c>
-      <c r="W14" s="7" t="inlineStr">
+      <c r="W14" s="8" t="inlineStr">
         <is>
           <t>Coaches and hosts whose live event is the front door to a high ticket offer, and who have a small team that needs structure.</t>
         </is>
       </c>
-      <c r="X14" s="7" t="inlineStr">
+      <c r="X14" s="8" t="inlineStr">
         <is>
           <t>Give a handful of scholarship tickets to qualified owners. Hell Yes Live gave out 6, and 5 became high ticket clients.</t>
         </is>

</xml_diff>

<commit_message>
Record the Creator Fest research and draft its row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1502,10 +1502,10 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="320" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Creator Fest</t>
+          <t>Creator Fest 2024</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -1528,33 +1528,104 @@
           <t>Interviewing</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr"/>
-      <c r="G10" s="5" t="inlineStr"/>
-      <c r="H10" s="5" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr"/>
-      <c r="K10" s="5" t="inlineStr"/>
-      <c r="L10" s="5" t="inlineStr"/>
-      <c r="M10" s="5" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Creators had events built for fans and events built for video growth, but none built around the business of being a creator. Creator Fest set out to be that event, built on five pillars: product, distribution, management, monetization and growth.
+As a brand new event, it had to earn credibility with creators, sponsors and the industry from scratch.</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>1. Partnered from the start with Patrick Israel of Stem Media Group: Iconic ran the venue, production and speakers, and Stem ran talent, sponsors and ticket sales.
+2. Built the program on five pillars of the creator business: product, distribution, management, monetization and growth.
+3. Closed general admission the Saturday before and sold only VIP from then on, to push upgrades.
+4. Turned a sponsor bought block of 100 tickets into giveaways, five per speaker, so every speaker brought part of their own audience.
+5. Reworked the founder's opening into a hero's journey talk with an intro video, to build trust from the first minute.
+6. Gave every attendee a lanyard by category: Creator, Industry, Production or Brand, so the right people found each other.</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>About 610 people came, making Creator Fest the largest creator event on the East Coast. Breakout rooms ran anywhere from 45 minutes to three and a half hours, more than 70 podcasts were recorded on site, and about 7 TB of content was captured. Snapchat's representative and former VidCon CEO Jim Louderback both praised the event.
+The lessons shaped what came next. The event was renamed CreatorHub, stayed at the JW Marriott, added virtual tickets and returned in 2025 as CreatorHub Live.</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>610 | Attendees in year one
+70+ | Podcasts recorded on site
+7 TB | Of content captured</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>Venue, production and the speaker program, with partner Stem Media Group running talent, sponsors and ticket sales.</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>Creator Fest was built to be the first business first event for creators, on five pillars from product to growth. With partner Stem Media Group running talent and sales, Iconic ran the venue, production and speakers at the JW Marriott Orlando Bonnet Creek, sold VIP only in the final week, turned sponsor tickets into speaker giveaways and opened with a hero's journey film. About 610 people came, more than 70 podcasts were recorded on site, and the event returned in 2025 as CreatorHub Live.</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>How Creator Fest Launched a Business First Event for Creators and Drew 610 in Year One</t>
+        </is>
+      </c>
+      <c r="M10" s="7" t="inlineStr">
+        <is>
+          <t>Want to launch the event your industry is missing?</t>
+        </is>
+      </c>
       <c r="N10" s="7" t="inlineStr">
         <is>
-          <t>Marriott Bonnet Creek, Orlando, FL</t>
-        </is>
-      </c>
-      <c r="O10" s="5" t="inlineStr"/>
-      <c r="P10" s="5" t="inlineStr"/>
+          <t>JW Marriott Orlando Bonnet Creek Resort &amp; Spa, Orlando, FL</t>
+        </is>
+      </c>
+      <c r="O10" s="7" t="inlineStr">
+        <is>
+          <t>610</t>
+        </is>
+      </c>
+      <c r="P10" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="Q10" s="5" t="inlineStr"/>
-      <c r="R10" s="5" t="inlineStr"/>
+      <c r="R10" s="7" t="inlineStr">
+        <is>
+          <t>On Google Drive; needs a YouTube or Vimeo link to embed</t>
+        </is>
+      </c>
       <c r="S10" s="5" t="inlineStr"/>
-      <c r="T10" s="5" t="inlineStr"/>
+      <c r="T10" s="7" t="inlineStr">
+        <is>
+          <t>Gallery at klevr.client-gallery.com/gallery/creatorfest-2024 (not reachable from this session); send selects as a zip</t>
+        </is>
+      </c>
       <c r="U10" s="7" t="inlineStr">
         <is>
-          <t>The first edition of what became CreatorHub Live. Not on the website grid yet; add it with the next approved site change. Skipped for now (Iconic, 2026-09-30).</t>
-        </is>
-      </c>
-      <c r="V10" s="5" t="n"/>
-      <c r="W10" s="5" t="n"/>
-      <c r="X10" s="5" t="n"/>
+          <t>Third person, no client line (Iconic's own event). Internal details left out per the research's own flag. 'Largest creator event on the East Coast' is from the debrief. Co-owner question: CreatorHub Live's live page says Xtend Creators; research says Stem Media Group. Venue: the JW Marriott Orlando Bonnet Creek (CreatorHub page says Marriott Bonnet Creek).</t>
+        </is>
+      </c>
+      <c r="V10" s="7" t="inlineStr">
+        <is>
+          <t>The speaker lineup kept shifting in the final weeks, and sponsor management changed hands three weeks before the doors opened. The program was reshaped around the speakers who were confirmed, and the event ran its full four days.</t>
+        </is>
+      </c>
+      <c r="W10" s="7" t="inlineStr">
+        <is>
+          <t>A first time event that needs industry credibility fast, with a partner who brings the talent and the sales.</t>
+        </is>
+      </c>
+      <c r="X10" s="7" t="inlineStr">
+        <is>
+          <t>Open with the founder's story. A hero's journey film before the first talk builds trust before anyone takes the stage.
+Sort the room with lanyards. Creator, Industry, Production and Brand lanyards told everyone who to talk to.
+Let sponsors fund the seats. A sponsor bought block of tickets, given away by speakers, filled the room with each speaker's audience.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Build Creator Fest 2024 and correct the CreatorHub hotel name
Add Creator Fest 2024 as a third person case study: the third largest
creator event in the country in its first year, with partner Xtend
Creators. Both Orlando pages now name the JW Marriott Orlando Bonnet
Creek.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HYnkdKH84MqhUZRmWtnDEv
</commit_message>
<xml_diff>
--- a/docs/case-studies/Case-Study-Interviews.xlsx
+++ b/docs/case-studies/Case-Study-Interviews.xlsx
@@ -1525,69 +1525,70 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Interviewing</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Creators had events built for fans and events built for video growth, but none built around the business of being a creator. Creator Fest set out to be that event, built on five pillars: product, distribution, management, monetization and growth.
-As a brand new event, it had to earn credibility with creators, sponsors and the industry from scratch.</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>1. Partnered from the start with Patrick Israel of Stem Media Group: Iconic ran the venue, production and speakers, and Stem ran talent, sponsors and ticket sales.
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Creators had events built for fans, and the only creator event aimed at business owners belonged to the largest creator in the world: MrBeast's VidSummit. Creator Fest set out to be the first true business event for the creator economy, built on five pillars: product, distribution, management, monetization and growth.
+Nobody wanted to back it at first. Sponsors wanted to see what the first three years looked like before they committed, and a brand new event had to earn its credibility with creators and the industry from scratch.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>1. Partnered from the start with Patrick Israel of Xtend Creators: Iconic ran the venue, production and speakers, and Xtend ran talent, sponsors and ticket sales.
 2. Built the program on five pillars of the creator business: product, distribution, management, monetization and growth.
-3. Closed general admission the Saturday before and sold only VIP from then on, to push upgrades.
-4. Turned a sponsor bought block of 100 tickets into giveaways, five per speaker, so every speaker brought part of their own audience.
-5. Reworked the founder's opening into a hero's journey talk with an intro video, to build trust from the first minute.
-6. Gave every attendee a lanyard by category: Creator, Industry, Production or Brand, so the right people found each other.</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>About 610 people came, making Creator Fest the largest creator event on the East Coast. Breakout rooms ran anywhere from 45 minutes to three and a half hours, more than 70 podcasts were recorded on site, and about 7 TB of content was captured. Snapchat's representative and former VidCon CEO Jim Louderback both praised the event.
+3. Got tactical with speakers and relational capital, until major players like Snapchat and former VidCon CEO Jim Louderback were behind the event.
+4. Closed general admission the Saturday before and sold only VIP from then on, to push upgrades.
+5. Turned a sponsor bought block of 100 tickets into giveaways, five per speaker, so every speaker brought part of their own audience.
+6. Reworked the founder's opening into a hero's journey talk with an intro video, to build trust from the first minute.
+7. Gave every attendee a lanyard by category: Creator, Industry, Production or Brand, so the right people found each other.</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>1,031 people came, making Creator Fest the third largest creator event in the country in its first year, and the first true business event for the creator economy. Breakout rooms ran anywhere from 45 minutes to three and a half hours, more than 70 podcasts were recorded on site, and about 7 TB of content was captured. Snapchat's representative and former VidCon CEO Jim Louderback both praised the event.
 The lessons shaped what came next. The event was renamed CreatorHub, stayed at the JW Marriott, added virtual tickets and returned in 2025 as CreatorHub Live.</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
-        <is>
-          <t>610 | Attendees in year one
-70+ | Podcasts recorded on site
-7 TB | Of content captured</t>
-        </is>
-      </c>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>Venue, production and the speaker program, with partner Stem Media Group running talent, sponsors and ticket sales.</t>
-        </is>
-      </c>
-      <c r="K10" s="7" t="inlineStr">
-        <is>
-          <t>Creator Fest was built to be the first business first event for creators, on five pillars from product to growth. With partner Stem Media Group running talent and sales, Iconic ran the venue, production and speakers at the JW Marriott Orlando Bonnet Creek, sold VIP only in the final week, turned sponsor tickets into speaker giveaways and opened with a hero's journey film. About 610 people came, more than 70 podcasts were recorded on site, and the event returned in 2025 as CreatorHub Live.</t>
-        </is>
-      </c>
-      <c r="L10" s="7" t="inlineStr">
-        <is>
-          <t>How Creator Fest Launched a Business First Event for Creators and Drew 610 in Year One</t>
-        </is>
-      </c>
-      <c r="M10" s="7" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>1,031 | Attendees in year one
+#3 | Largest creator event in the country
+70+ | Podcasts recorded on site</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>Venue, production and the speaker program, with partner Xtend Creators running talent, sponsors and ticket sales.</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>Creator Fest set out to be the first true business event for the creator economy, up against an event owned by the largest creator in the world, with no sponsors willing to back year one. With partner Xtend Creators running talent and sales, Iconic ran the venue, production and speakers at the JW Marriott Orlando Bonnet Creek and won over backers like Snapchat and former VidCon CEO Jim Louderback. 1,031 people came, making it the third largest creator event in the country in its first year, and it returned in 2025 as CreatorHub Live.</t>
+        </is>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>How Creator Fest Became the Third Largest Creator Event in the Country in Its First Year</t>
+        </is>
+      </c>
+      <c r="M10" s="8" t="inlineStr">
         <is>
           <t>Want to launch the event your industry is missing?</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr">
+      <c r="N10" s="8" t="inlineStr">
         <is>
           <t>JW Marriott Orlando Bonnet Creek Resort &amp; Spa, Orlando, FL</t>
         </is>
       </c>
-      <c r="O10" s="7" t="inlineStr">
-        <is>
-          <t>610</t>
-        </is>
-      </c>
-      <c r="P10" s="7" t="inlineStr">
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>1,031</t>
+        </is>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -1606,20 +1607,20 @@
       </c>
       <c r="U10" s="7" t="inlineStr">
         <is>
-          <t>Third person, no client line (Iconic's own event). Internal details left out per the research's own flag. 'Largest creator event on the East Coast' is from the debrief. Co-owner question: CreatorHub Live's live page says Xtend Creators; research says Stem Media Group. Venue: the JW Marriott Orlando Bonnet Creek (CreatorHub page says Marriott Bonnet Creek).</t>
-        </is>
-      </c>
-      <c r="V10" s="7" t="inlineStr">
-        <is>
-          <t>The speaker lineup kept shifting in the final weeks, and sponsor management changed hands three weeks before the doors opened. The program was reshaped around the speakers who were confirmed, and the event ran its full four days.</t>
-        </is>
-      </c>
-      <c r="W10" s="7" t="inlineStr">
+          <t>Approved by Iconic 2026-10-25 and built. Third person, no client line. Partner Xtend Creators only. 1,031 attendees per Iconic. Aftermovie needs a YouTube link; photos as a zip.</t>
+        </is>
+      </c>
+      <c r="V10" s="8" t="inlineStr">
+        <is>
+          <t>With no sponsors willing to bet on year one, the event had to win its backers one relationship at a time. It started slow and ramped up quickly, until Snapchat and the former CEO of VidCon were behind it. In the final weeks the speaker lineup kept shifting and sponsor management changed hands, and the program was reshaped around the speakers who were confirmed. The event ran its full four days.</t>
+        </is>
+      </c>
+      <c r="W10" s="8" t="inlineStr">
         <is>
           <t>A first time event that needs industry credibility fast, with a partner who brings the talent and the sales.</t>
         </is>
       </c>
-      <c r="X10" s="7" t="inlineStr">
+      <c r="X10" s="8" t="inlineStr">
         <is>
           <t>Open with the founder's story. A hero's journey film before the first talk builds trust before anyone takes the stage.
 Sort the room with lanyards. Creator, Industry, Production and Brand lanyards told everyone who to talk to.

</xml_diff>